<commit_message>
data: update 2026-04-26 10:09
</commit_message>
<xml_diff>
--- a/output/nb_master.xlsx
+++ b/output/nb_master.xlsx
@@ -4940,7 +4940,7 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>NINGBO KAIRONG SHIP MACHINERY CO.,LTD.</t>
+          <t>NINGBO KAIRONG SHIP MACHINERY CO., LTD</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
@@ -6798,7 +6798,7 @@
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>MAN B&amp;W</t>
+          <t>MAN-B&amp;W</t>
         </is>
       </c>
       <c r="C172" s="2" t="inlineStr">
@@ -6835,7 +6835,7 @@
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>MAN B&amp;W</t>
+          <t>MAN-B&amp;W</t>
         </is>
       </c>
       <c r="C173" s="4" t="inlineStr">
@@ -16665,7 +16665,7 @@
       </c>
       <c r="B439" s="4" t="inlineStr">
         <is>
-          <t>JIANGYANCITY MARINE OUTFITTING CO., LTD</t>
+          <t>JIANGYAN CITY MARINE OUTFITTING CO.,LTD</t>
         </is>
       </c>
       <c r="C439" s="4" t="inlineStr">
@@ -16702,7 +16702,7 @@
       </c>
       <c r="B440" s="2" t="inlineStr">
         <is>
-          <t>JIANGYANCITY MARINE OUTFITTING CO., LTD</t>
+          <t>JIANGYAN CITY MARINE OUTFITTING CO.,LTD</t>
         </is>
       </c>
       <c r="C440" s="2" t="inlineStr">
@@ -16739,7 +16739,7 @@
       </c>
       <c r="B441" s="4" t="inlineStr">
         <is>
-          <t>JIANGYANCITY MARINE OUTFITTING CO., LTD</t>
+          <t>JIANGYAN CITY MARINE OUTFITTING CO.,LTD</t>
         </is>
       </c>
       <c r="C441" s="4" t="inlineStr">
@@ -22104,7 +22104,7 @@
       </c>
       <c r="B586" s="2" t="inlineStr">
         <is>
-          <t>HI-AIR KOREA</t>
+          <t>HI AIR KOREA</t>
         </is>
       </c>
       <c r="C586" s="2" t="inlineStr">
@@ -22141,7 +22141,7 @@
       </c>
       <c r="B587" s="4" t="inlineStr">
         <is>
-          <t>HI-AIR KOREA</t>
+          <t>HI AIR KOREA</t>
         </is>
       </c>
       <c r="C587" s="4" t="inlineStr">
@@ -25064,7 +25064,7 @@
       </c>
       <c r="B666" s="2" t="inlineStr">
         <is>
-          <t>MAN B&amp;W</t>
+          <t>MAN-B&amp;W</t>
         </is>
       </c>
       <c r="C666" s="2" t="inlineStr">
@@ -25175,7 +25175,7 @@
       </c>
       <c r="B669" s="4" t="inlineStr">
         <is>
-          <t>MAN B&amp;W</t>
+          <t>MAN-B&amp;W</t>
         </is>
       </c>
       <c r="C669" s="4" t="inlineStr">
@@ -25434,7 +25434,7 @@
       </c>
       <c r="B676" s="2" t="inlineStr">
         <is>
-          <t>MAN B&amp;W</t>
+          <t>MAN-B&amp;W</t>
         </is>
       </c>
       <c r="C676" s="2" t="inlineStr">
@@ -28468,7 +28468,7 @@
       </c>
       <c r="B758" s="2" t="inlineStr">
         <is>
-          <t>MAN B&amp;W</t>
+          <t>MAN-B&amp;W</t>
         </is>
       </c>
       <c r="C758" s="2" t="inlineStr">
@@ -28505,7 +28505,7 @@
       </c>
       <c r="B759" s="4" t="inlineStr">
         <is>
-          <t>MAN B&amp;W</t>
+          <t>MAN-B&amp;W</t>
         </is>
       </c>
       <c r="C759" s="4" t="inlineStr">
@@ -28542,7 +28542,7 @@
       </c>
       <c r="B760" s="2" t="inlineStr">
         <is>
-          <t>MAN B&amp;W</t>
+          <t>MAN-B&amp;W</t>
         </is>
       </c>
       <c r="C760" s="2" t="inlineStr">
@@ -28579,7 +28579,7 @@
       </c>
       <c r="B761" s="4" t="inlineStr">
         <is>
-          <t>MAN B&amp;W</t>
+          <t>MAN-B&amp;W</t>
         </is>
       </c>
       <c r="C761" s="4" t="inlineStr">
@@ -28875,7 +28875,7 @@
       </c>
       <c r="B769" s="4" t="inlineStr">
         <is>
-          <t>J.P.SAUER&amp;SOHN</t>
+          <t>J.P. SAUER &amp; SOHN</t>
         </is>
       </c>
       <c r="C769" s="4" t="inlineStr">
@@ -28912,7 +28912,7 @@
       </c>
       <c r="B770" s="2" t="inlineStr">
         <is>
-          <t>J.P.SAUER&amp;SOHN</t>
+          <t>J.P. SAUER &amp; SOHN</t>
         </is>
       </c>
       <c r="C770" s="2" t="inlineStr">
@@ -31206,7 +31206,7 @@
       </c>
       <c r="B832" s="2" t="inlineStr">
         <is>
-          <t>ALFA-LAVAL</t>
+          <t>ALFA LAVAL</t>
         </is>
       </c>
       <c r="C832" s="2" t="inlineStr">
@@ -31243,7 +31243,7 @@
       </c>
       <c r="B833" s="4" t="inlineStr">
         <is>
-          <t>ALFA-LAVAL</t>
+          <t>ALFA LAVAL</t>
         </is>
       </c>
       <c r="C833" s="4" t="inlineStr">
@@ -31280,7 +31280,7 @@
       </c>
       <c r="B834" s="2" t="inlineStr">
         <is>
-          <t>ALFA-LAVAL</t>
+          <t>ALFA LAVAL</t>
         </is>
       </c>
       <c r="C834" s="2" t="inlineStr">
@@ -31650,7 +31650,7 @@
       </c>
       <c r="B844" s="2" t="inlineStr">
         <is>
-          <t>JIANGSU MASADA HEAVY INDUSTRIES CO.,LTD.</t>
+          <t>JIANGSU MASADA HEAVY INDUSTRIES CO.,LTD</t>
         </is>
       </c>
       <c r="C844" s="2" t="inlineStr">
@@ -31687,7 +31687,7 @@
       </c>
       <c r="B845" s="4" t="inlineStr">
         <is>
-          <t>JIANGSU MASADA HEAVY INDUSTRIES CO.,LTD.</t>
+          <t>JIANGSU MASADA HEAVY INDUSTRIES CO.,LTD</t>
         </is>
       </c>
       <c r="C845" s="4" t="inlineStr">
@@ -31724,7 +31724,7 @@
       </c>
       <c r="B846" s="2" t="inlineStr">
         <is>
-          <t>JIANGSU MASADA HEAVY INDUSTRIES CO.,LTD.</t>
+          <t>JIANGSU MASADA HEAVY INDUSTRIES CO.,LTD</t>
         </is>
       </c>
       <c r="C846" s="2" t="inlineStr">
@@ -31761,7 +31761,7 @@
       </c>
       <c r="B847" s="4" t="inlineStr">
         <is>
-          <t>JIANGSU MASADA HEAVY INDUSTRIES CO.,LTD.</t>
+          <t>JIANGSU MASADA HEAVY INDUSTRIES CO.,LTD</t>
         </is>
       </c>
       <c r="C847" s="4" t="inlineStr">
@@ -37977,7 +37977,7 @@
       </c>
       <c r="B1015" s="4" t="inlineStr">
         <is>
-          <t>ALFALAVAL</t>
+          <t>ALFA LAVAL</t>
         </is>
       </c>
       <c r="C1015" s="4" t="inlineStr">
@@ -38014,7 +38014,7 @@
       </c>
       <c r="B1016" s="2" t="inlineStr">
         <is>
-          <t>ALFALAVAL</t>
+          <t>ALFA LAVAL</t>
         </is>
       </c>
       <c r="C1016" s="2" t="inlineStr">
@@ -38051,7 +38051,7 @@
       </c>
       <c r="B1017" s="4" t="inlineStr">
         <is>
-          <t>ALFALAVAL</t>
+          <t>ALFA LAVAL</t>
         </is>
       </c>
       <c r="C1017" s="4" t="inlineStr">
@@ -38088,7 +38088,7 @@
       </c>
       <c r="B1018" s="2" t="inlineStr">
         <is>
-          <t>ALFALAVAL</t>
+          <t>ALFA LAVAL</t>
         </is>
       </c>
       <c r="C1018" s="2" t="inlineStr">
@@ -38162,7 +38162,7 @@
       </c>
       <c r="B1020" s="2" t="inlineStr">
         <is>
-          <t>ALFALAVAL</t>
+          <t>ALFA LAVAL</t>
         </is>
       </c>
       <c r="C1020" s="2" t="inlineStr">
@@ -38199,7 +38199,7 @@
       </c>
       <c r="B1021" s="4" t="inlineStr">
         <is>
-          <t>ALFALAVAL</t>
+          <t>ALFA LAVAL</t>
         </is>
       </c>
       <c r="C1021" s="4" t="inlineStr">
@@ -40937,7 +40937,7 @@
       </c>
       <c r="B1095" s="4" t="inlineStr">
         <is>
-          <t>HEINEN &amp; HOPMAN</t>
+          <t>HEINEN&amp;HOPMAN</t>
         </is>
       </c>
       <c r="C1095" s="4" t="inlineStr">
@@ -40974,7 +40974,7 @@
       </c>
       <c r="B1096" s="2" t="inlineStr">
         <is>
-          <t>HEINEN &amp; HOPMAN</t>
+          <t>HEINEN&amp;HOPMAN</t>
         </is>
       </c>
       <c r="C1096" s="2" t="inlineStr">

</xml_diff>

<commit_message>
data: update 2026-04-26 10:39
</commit_message>
<xml_diff>
--- a/output/nb_master.xlsx
+++ b/output/nb_master.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1107"/>
+  <dimension ref="A1:G1106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -4987,7 +4987,7 @@
       </c>
       <c r="D123" s="4" t="inlineStr">
         <is>
-          <t>GEARBOX</t>
+          <t>GEAR BOX</t>
         </is>
       </c>
       <c r="E123" s="4" t="inlineStr">
@@ -5172,7 +5172,7 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>GEARBOX</t>
+          <t>GEAR BOX</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -5320,7 +5320,7 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>GEARBOX</t>
+          <t>GEAR BOX</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
@@ -7692,7 +7692,7 @@
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>TURNING GEAR CHAIN</t>
+          <t>TURNING GEAR(CHAIN)</t>
         </is>
       </c>
       <c r="E196" s="2" t="inlineStr">
@@ -8025,7 +8025,7 @@
       </c>
       <c r="D205" s="4" t="inlineStr">
         <is>
-          <t>ENGINE L.O SYSTEM</t>
+          <t>ENGINE LO SYSTEM</t>
         </is>
       </c>
       <c r="E205" s="4" t="inlineStr">
@@ -10023,7 +10023,7 @@
       </c>
       <c r="D259" s="4" t="inlineStr">
         <is>
-          <t>ENCLOSED GEAR</t>
+          <t>ENCLOSED GEAR-</t>
         </is>
       </c>
       <c r="E259" s="4" t="inlineStr">
@@ -10504,7 +10504,7 @@
       </c>
       <c r="D272" s="2" t="inlineStr">
         <is>
-          <t>GEARBOX</t>
+          <t>GEAR BOX</t>
         </is>
       </c>
       <c r="E272" s="2" t="inlineStr">
@@ -12531,7 +12531,7 @@
       </c>
       <c r="D327" s="4" t="inlineStr">
         <is>
-          <t>WIRE ROPES</t>
+          <t>WIRE ROPES-</t>
         </is>
       </c>
       <c r="E327" s="4" t="inlineStr">
@@ -13234,7 +13234,7 @@
       </c>
       <c r="D346" s="2" t="inlineStr">
         <is>
-          <t>WIRE ROPES</t>
+          <t>WIRE ROPES-</t>
         </is>
       </c>
       <c r="E346" s="2" t="inlineStr">
@@ -16675,7 +16675,7 @@
       </c>
       <c r="D439" s="4" t="inlineStr">
         <is>
-          <t>WINCH GEARBOX</t>
+          <t>WINCH GEAR BOX</t>
         </is>
       </c>
       <c r="E439" s="4" t="inlineStr">
@@ -19228,7 +19228,7 @@
       </c>
       <c r="D508" s="2" t="inlineStr">
         <is>
-          <t>WTS SEPARATOR</t>
+          <t>WTS(SEPARATOR)</t>
         </is>
       </c>
       <c r="E508" s="2" t="inlineStr">
@@ -19524,7 +19524,7 @@
       </c>
       <c r="D516" s="2" t="inlineStr">
         <is>
-          <t>CRANKCASE</t>
+          <t>CRANK CASE</t>
         </is>
       </c>
       <c r="E516" s="2" t="inlineStr">
@@ -19561,7 +19561,7 @@
       </c>
       <c r="D517" s="4" t="inlineStr">
         <is>
-          <t>CRANKCASE</t>
+          <t>CRANK CASE</t>
         </is>
       </c>
       <c r="E517" s="4" t="inlineStr">
@@ -22114,7 +22114,7 @@
       </c>
       <c r="D586" s="2" t="inlineStr">
         <is>
-          <t>CRANKCASE</t>
+          <t>CRANK CASE</t>
         </is>
       </c>
       <c r="E586" s="2" t="inlineStr">
@@ -22151,7 +22151,7 @@
       </c>
       <c r="D587" s="4" t="inlineStr">
         <is>
-          <t>CRANKCASE</t>
+          <t>CRANK CASE</t>
         </is>
       </c>
       <c r="E587" s="4" t="inlineStr">
@@ -22965,7 +22965,7 @@
       </c>
       <c r="D609" s="4" t="inlineStr">
         <is>
-          <t>CRANKCASE</t>
+          <t>CRANK CASE</t>
         </is>
       </c>
       <c r="E609" s="4" t="inlineStr">
@@ -23002,7 +23002,7 @@
       </c>
       <c r="D610" s="2" t="inlineStr">
         <is>
-          <t>CRANKCASE</t>
+          <t>CRANK CASE</t>
         </is>
       </c>
       <c r="E610" s="2" t="inlineStr">
@@ -23113,7 +23113,7 @@
       </c>
       <c r="D613" s="4" t="inlineStr">
         <is>
-          <t>CRANKCASE</t>
+          <t>CRANK CASE</t>
         </is>
       </c>
       <c r="E613" s="4" t="inlineStr">
@@ -23372,7 +23372,7 @@
       </c>
       <c r="D620" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER OIL-</t>
+          <t>CYLINDER OIL</t>
         </is>
       </c>
       <c r="E620" s="2" t="inlineStr">
@@ -23409,7 +23409,7 @@
       </c>
       <c r="D621" s="4" t="inlineStr">
         <is>
-          <t>CRANKCASE-</t>
+          <t>CRANK CASE</t>
         </is>
       </c>
       <c r="E621" s="4" t="inlineStr">
@@ -23446,7 +23446,7 @@
       </c>
       <c r="D622" s="2" t="inlineStr">
         <is>
-          <t>CRANKCASE-</t>
+          <t>CRANK CASE</t>
         </is>
       </c>
       <c r="E622" s="2" t="inlineStr">
@@ -23483,7 +23483,7 @@
       </c>
       <c r="D623" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM OIL-</t>
+          <t>SYSTEM OIL</t>
         </is>
       </c>
       <c r="E623" s="4" t="inlineStr">
@@ -23557,7 +23557,7 @@
       </c>
       <c r="D625" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM OIL-</t>
+          <t>SYSTEM OIL</t>
         </is>
       </c>
       <c r="E625" s="4" t="inlineStr">
@@ -23594,7 +23594,7 @@
       </c>
       <c r="D626" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL-</t>
+          <t>SYSTEM OIL</t>
         </is>
       </c>
       <c r="E626" s="2" t="inlineStr">
@@ -23705,7 +23705,7 @@
       </c>
       <c r="D629" s="4" t="inlineStr">
         <is>
-          <t>GREASE POINT-</t>
+          <t>GREASE POINT</t>
         </is>
       </c>
       <c r="E629" s="4" t="inlineStr">
@@ -23742,7 +23742,7 @@
       </c>
       <c r="D630" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL-</t>
+          <t>SYSTEM OIL</t>
         </is>
       </c>
       <c r="E630" s="2" t="inlineStr">
@@ -23890,7 +23890,7 @@
       </c>
       <c r="D634" s="2" t="inlineStr">
         <is>
-          <t>HYDRAULIC SYSTEM-</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E634" s="2" t="inlineStr">
@@ -23964,7 +23964,7 @@
       </c>
       <c r="D636" s="2" t="inlineStr">
         <is>
-          <t>WIRE ROPE-</t>
+          <t>WIRE ROPE</t>
         </is>
       </c>
       <c r="E636" s="2" t="inlineStr">
@@ -24001,7 +24001,7 @@
       </c>
       <c r="D637" s="4" t="inlineStr">
         <is>
-          <t>GREASE POINT-</t>
+          <t>GREASE POINT</t>
         </is>
       </c>
       <c r="E637" s="4" t="inlineStr">
@@ -24038,7 +24038,7 @@
       </c>
       <c r="D638" s="2" t="inlineStr">
         <is>
-          <t>HYDRAULIC SYSTEM-</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E638" s="2" t="inlineStr">
@@ -24112,7 +24112,7 @@
       </c>
       <c r="D640" s="2" t="inlineStr">
         <is>
-          <t>WIRE ROPE-</t>
+          <t>WIRE ROPE</t>
         </is>
       </c>
       <c r="E640" s="2" t="inlineStr">
@@ -24149,7 +24149,7 @@
       </c>
       <c r="D641" s="4" t="inlineStr">
         <is>
-          <t>GREASE POINT-</t>
+          <t>GREASE POINT</t>
         </is>
       </c>
       <c r="E641" s="4" t="inlineStr">
@@ -24223,7 +24223,7 @@
       </c>
       <c r="D643" s="4" t="inlineStr">
         <is>
-          <t>GREASE POINT-</t>
+          <t>GREASE POINT</t>
         </is>
       </c>
       <c r="E643" s="4" t="inlineStr">
@@ -24260,7 +24260,7 @@
       </c>
       <c r="D644" s="2" t="inlineStr">
         <is>
-          <t>ENGINE-</t>
+          <t>ENGINE</t>
         </is>
       </c>
       <c r="E644" s="2" t="inlineStr">
@@ -24297,7 +24297,7 @@
       </c>
       <c r="D645" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOX-</t>
+          <t>GEAR BOX</t>
         </is>
       </c>
       <c r="E645" s="4" t="inlineStr">
@@ -24334,7 +24334,7 @@
       </c>
       <c r="D646" s="2" t="inlineStr">
         <is>
-          <t>PROPELLER SHAFT-</t>
+          <t>PROPELLER SHAFT</t>
         </is>
       </c>
       <c r="E646" s="2" t="inlineStr">
@@ -24371,7 +24371,7 @@
       </c>
       <c r="D647" s="4" t="inlineStr">
         <is>
-          <t>GREASE POINT-</t>
+          <t>GREASE POINT</t>
         </is>
       </c>
       <c r="E647" s="4" t="inlineStr">
@@ -24482,7 +24482,7 @@
       </c>
       <c r="D650" s="2" t="inlineStr">
         <is>
-          <t>GEAR-</t>
+          <t>GEAR</t>
         </is>
       </c>
       <c r="E650" s="2" t="inlineStr">
@@ -24519,7 +24519,7 @@
       </c>
       <c r="D651" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM OIL-</t>
+          <t>SYSTEM OIL</t>
         </is>
       </c>
       <c r="E651" s="4" t="inlineStr">
@@ -24556,7 +24556,7 @@
       </c>
       <c r="D652" s="2" t="inlineStr">
         <is>
-          <t>GREASE POINT-</t>
+          <t>GREASE POINT</t>
         </is>
       </c>
       <c r="E652" s="2" t="inlineStr">
@@ -24630,7 +24630,7 @@
       </c>
       <c r="D654" s="2" t="inlineStr">
         <is>
-          <t>BEARINGS-</t>
+          <t>BEARINGS</t>
         </is>
       </c>
       <c r="E654" s="2" t="inlineStr">
@@ -24667,7 +24667,7 @@
       </c>
       <c r="D655" s="4" t="inlineStr">
         <is>
-          <t>OPEN GEAR-</t>
+          <t>OPEN GEAR</t>
         </is>
       </c>
       <c r="E655" s="4" t="inlineStr">
@@ -24704,7 +24704,7 @@
       </c>
       <c r="D656" s="2" t="inlineStr">
         <is>
-          <t>REDUCER-</t>
+          <t>REDUCER</t>
         </is>
       </c>
       <c r="E656" s="2" t="inlineStr">
@@ -24778,7 +24778,7 @@
       </c>
       <c r="D658" s="2" t="inlineStr">
         <is>
-          <t>OPEN GEAR-</t>
+          <t>OPEN GEAR</t>
         </is>
       </c>
       <c r="E658" s="2" t="inlineStr">
@@ -24815,7 +24815,7 @@
       </c>
       <c r="D659" s="4" t="inlineStr">
         <is>
-          <t>BEARINGS-</t>
+          <t>BEARINGS</t>
         </is>
       </c>
       <c r="E659" s="4" t="inlineStr">
@@ -24852,7 +24852,7 @@
       </c>
       <c r="D660" s="2" t="inlineStr">
         <is>
-          <t>REDUCER-</t>
+          <t>REDUCER</t>
         </is>
       </c>
       <c r="E660" s="2" t="inlineStr">
@@ -24963,7 +24963,7 @@
       </c>
       <c r="D663" s="4" t="inlineStr">
         <is>
-          <t>GREASE POINT-</t>
+          <t>GREASE POINT</t>
         </is>
       </c>
       <c r="E663" s="4" t="inlineStr">
@@ -25000,7 +25000,7 @@
       </c>
       <c r="D664" s="2" t="inlineStr">
         <is>
-          <t>GREASE POINT-</t>
+          <t>GREASE POINT</t>
         </is>
       </c>
       <c r="E664" s="2" t="inlineStr">
@@ -25037,7 +25037,7 @@
       </c>
       <c r="D665" s="4" t="inlineStr">
         <is>
-          <t>GREASE-</t>
+          <t>GREASE</t>
         </is>
       </c>
       <c r="E665" s="4" t="inlineStr">
@@ -25407,7 +25407,7 @@
       </c>
       <c r="D675" s="4" t="inlineStr">
         <is>
-          <t>ENCLOSED GEAR</t>
+          <t>ENCLOSED GEAR-</t>
         </is>
       </c>
       <c r="E675" s="4" t="inlineStr">
@@ -26147,7 +26147,7 @@
       </c>
       <c r="D695" s="4" t="inlineStr">
         <is>
-          <t>INTER SHAFT BEARING</t>
+          <t>INTER. SHAFT BEARING</t>
         </is>
       </c>
       <c r="E695" s="4" t="inlineStr">
@@ -26887,7 +26887,7 @@
       </c>
       <c r="D715" s="4" t="inlineStr">
         <is>
-          <t>HYDR. OIL</t>
+          <t>HYDR.OIL</t>
         </is>
       </c>
       <c r="E715" s="4" t="inlineStr">
@@ -26998,7 +26998,7 @@
       </c>
       <c r="D718" s="2" t="inlineStr">
         <is>
-          <t>HYDR. OIL</t>
+          <t>HYDR.OIL</t>
         </is>
       </c>
       <c r="E718" s="2" t="inlineStr">
@@ -29551,7 +29551,7 @@
       </c>
       <c r="D787" s="4" t="inlineStr">
         <is>
-          <t>ENCLOSED GEAR</t>
+          <t>ENCLOSED GEAR-</t>
         </is>
       </c>
       <c r="E787" s="4" t="inlineStr">
@@ -32511,7 +32511,7 @@
       </c>
       <c r="D867" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOXES FOR WINCH</t>
+          <t>GEAR BOXES FOR WINCH-</t>
         </is>
       </c>
       <c r="E867" s="4" t="inlineStr">
@@ -39282,12 +39282,12 @@
       </c>
       <c r="D1050" s="2" t="inlineStr">
         <is>
-          <t>BEARING- YARD MAINTERNANCE</t>
+          <t>HOISTING GEAR BOX OPEN GEAR/ WIRE ROPE - YARD</t>
         </is>
       </c>
       <c r="E1050" s="2" t="inlineStr">
         <is>
-          <t>CERAN XM 220</t>
+          <t>CERAN AD PLUS</t>
         </is>
       </c>
       <c r="F1050" s="3" t="inlineStr">
@@ -39304,27 +39304,27 @@
     <row r="1051">
       <c r="A1051" s="4" t="inlineStr">
         <is>
-          <t>PROVISION CRANE CARGO MACHINERY ROOM EQUIPMENT</t>
+          <t>MAIN ENGINE</t>
         </is>
       </c>
       <c r="B1051" s="4" t="inlineStr">
         <is>
-          <t>KS INDUSTRY</t>
+          <t>HANWHA ENGINE HANMI HYDRAULIC</t>
         </is>
       </c>
       <c r="C1051" s="4" t="inlineStr">
         <is>
-          <t>PORT/STB'D</t>
+          <t>9G95ME-C10.5-LGIM-EGRTC</t>
         </is>
       </c>
       <c r="D1051" s="4" t="inlineStr">
         <is>
-          <t>HOISTING GEAR BOX OPEN GEAR/ WIRE ROPE - YARD</t>
+          <t>LO SYSTEM, TURBOCHARGER, PIPING,</t>
         </is>
       </c>
       <c r="E1051" s="4" t="inlineStr">
         <is>
-          <t>CERAN AD PLUS</t>
+          <t>ATLANTA MARINE D 3005</t>
         </is>
       </c>
       <c r="F1051" s="5" t="inlineStr">
@@ -39334,7 +39334,7 @@
       </c>
       <c r="G1051" s="4" t="inlineStr">
         <is>
-          <t>SN2662 MF00201 LO ChartRev.C.pdf</t>
+          <t>SN2672 76 79 81 83 85 L.O chart(TOTAL)_HSHFO_rev.D_2025-09-19.pdf</t>
         </is>
       </c>
     </row>
@@ -39356,7 +39356,7 @@
       </c>
       <c r="D1052" s="2" t="inlineStr">
         <is>
-          <t>LO SYSTEM, TURBOCHARGER, PIPING,</t>
+          <t>SYSTEM OIL_T/C LO TANK(95%)</t>
         </is>
       </c>
       <c r="E1052" s="2" t="inlineStr">
@@ -39393,7 +39393,7 @@
       </c>
       <c r="D1053" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM OIL_T/C LO TANK(95%)</t>
+          <t>SYSTEM OIL_T/C LO TANK(95%) SYSTEM OIL_STERN TUBE L.O SUMP</t>
         </is>
       </c>
       <c r="E1053" s="4" t="inlineStr">
@@ -39430,7 +39430,7 @@
       </c>
       <c r="D1054" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL_T/C LO TANK(95%) SYSTEM OIL_STERN TUBE L.O SUMP</t>
+          <t>SYSTEM OIL_T/C LO TANK(95%) SYSTEM OIL_STERN TUBE L.O SUMP TANK(100%) SYSTEM OIL_STERN TUBE L.O TANK</t>
         </is>
       </c>
       <c r="E1054" s="2" t="inlineStr">
@@ -39467,7 +39467,7 @@
       </c>
       <c r="D1055" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM OIL_T/C LO TANK(95%) SYSTEM OIL_STERN TUBE L.O SUMP TANK(100%) SYSTEM OIL_STERN TUBE L.O TANK</t>
+          <t>SYSTEM OIL_T/C LO TANK(95%) SYSTEM OIL_STERN TUBE L.O SUMP TANK(100%) SYSTEM OIL_STERN TUBE L.O TANK UNIT(100%) M/E HYDRAULIC CONTROL OIL</t>
         </is>
       </c>
       <c r="E1055" s="4" t="inlineStr">
@@ -39504,12 +39504,12 @@
       </c>
       <c r="D1056" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL_T/C LO TANK(95%) SYSTEM OIL_STERN TUBE L.O SUMP TANK(100%) SYSTEM OIL_STERN TUBE L.O TANK UNIT(100%) M/E HYDRAULIC CONTROL OIL</t>
+          <t>TANK(95%) CYLINDER OIL CONSUMPTION(ABT. 5</t>
         </is>
       </c>
       <c r="E1056" s="2" t="inlineStr">
         <is>
-          <t>ATLANTA MARINE D 3005</t>
+          <t>TALUSIA HR 140</t>
         </is>
       </c>
       <c r="F1056" s="3" t="inlineStr">
@@ -39541,7 +39541,7 @@
       </c>
       <c r="D1057" s="4" t="inlineStr">
         <is>
-          <t>TANK(95%) CYLINDER OIL CONSUMPTION(ABT. 5</t>
+          <t>TANK(95%) CYLINDER OIL CONSUMPTION(ABT. 5 DAYS) DEAD OIL OF CYLINDER OIL STORAGE</t>
         </is>
       </c>
       <c r="E1057" s="4" t="inlineStr">
@@ -39578,7 +39578,7 @@
       </c>
       <c r="D1058" s="2" t="inlineStr">
         <is>
-          <t>TANK(95%) CYLINDER OIL CONSUMPTION(ABT. 5 DAYS) DEAD OIL OF CYLINDER OIL STORAGE</t>
+          <t>TANK(95%) CYLINDER OIL CONSUMPTION(ABT. 5 DAYS) DEAD OIL OF CYLINDER OIL STORAGE TANK(ABT. 5%)_HIGH BN CYLINDER OIL MEASURING TANK (HIGH</t>
         </is>
       </c>
       <c r="E1058" s="2" t="inlineStr">
@@ -39615,12 +39615,12 @@
       </c>
       <c r="D1059" s="4" t="inlineStr">
         <is>
-          <t>TANK(95%) CYLINDER OIL CONSUMPTION(ABT. 5 DAYS) DEAD OIL OF CYLINDER OIL STORAGE TANK(ABT. 5%)_HIGH BN CYLINDER OIL MEASURING TANK (HIGH</t>
+          <t>DEAD OIL OF CYLINDER OIL STORAGE</t>
         </is>
       </c>
       <c r="E1059" s="4" t="inlineStr">
         <is>
-          <t>TALUSIA HR 140</t>
+          <t>TALUSIA HD 40</t>
         </is>
       </c>
       <c r="F1059" s="5" t="inlineStr">
@@ -39652,7 +39652,7 @@
       </c>
       <c r="D1060" s="2" t="inlineStr">
         <is>
-          <t>DEAD OIL OF CYLINDER OIL STORAGE</t>
+          <t>DEAD OIL OF CYLINDER OIL STORAGE TANK(ABT. 5%)_LOW BN CYLINDER OIL MEASURING TANK (LOW</t>
         </is>
       </c>
       <c r="E1060" s="2" t="inlineStr">
@@ -39689,12 +39689,12 @@
       </c>
       <c r="D1061" s="4" t="inlineStr">
         <is>
-          <t>DEAD OIL OF CYLINDER OIL STORAGE TANK(ABT. 5%)_LOW BN CYLINDER OIL MEASURING TANK (LOW</t>
+          <t>AUXILIARY BLOWER MOTOR</t>
         </is>
       </c>
       <c r="E1061" s="4" t="inlineStr">
         <is>
-          <t>TALUSIA HD 40</t>
+          <t>CERAN XM 220</t>
         </is>
       </c>
       <c r="F1061" s="5" t="inlineStr">
@@ -39726,12 +39726,12 @@
       </c>
       <c r="D1062" s="2" t="inlineStr">
         <is>
-          <t>AUXILIARY BLOWER MOTOR</t>
+          <t>GAS VALVE TESTER(HANMI)</t>
         </is>
       </c>
       <c r="E1062" s="2" t="inlineStr">
         <is>
-          <t>CERAN XM 220</t>
+          <t>VISGA 15</t>
         </is>
       </c>
       <c r="F1062" s="3" t="inlineStr">
@@ -39763,12 +39763,12 @@
       </c>
       <c r="D1063" s="4" t="inlineStr">
         <is>
-          <t>GAS VALVE TESTER(HANMI)</t>
+          <t>TURNING GEAR(GEAR)</t>
         </is>
       </c>
       <c r="E1063" s="4" t="inlineStr">
         <is>
-          <t>VISGA 15</t>
+          <t>EPONA Z 320</t>
         </is>
       </c>
       <c r="F1063" s="5" t="inlineStr">
@@ -39800,12 +39800,12 @@
       </c>
       <c r="D1064" s="2" t="inlineStr">
         <is>
-          <t>TURNING GEAR(GEAR)</t>
+          <t>TURNING GEAR(CHAIN)</t>
         </is>
       </c>
       <c r="E1064" s="2" t="inlineStr">
         <is>
-          <t>EPONA Z 320</t>
+          <t>CERAN XM 220</t>
         </is>
       </c>
       <c r="F1064" s="3" t="inlineStr">
@@ -39837,12 +39837,12 @@
       </c>
       <c r="D1065" s="4" t="inlineStr">
         <is>
-          <t>TURNING GEAR(CHAIN)</t>
+          <t>EGR CIRCULATION PUMP</t>
         </is>
       </c>
       <c r="E1065" s="4" t="inlineStr">
         <is>
-          <t>CERAN XM 220</t>
+          <t>ALTIS EM 2</t>
         </is>
       </c>
       <c r="F1065" s="5" t="inlineStr">
@@ -39874,12 +39874,12 @@
       </c>
       <c r="D1066" s="2" t="inlineStr">
         <is>
-          <t>EGR CIRCULATION PUMP</t>
+          <t>EGR CIRCULATION PUMP MOTOR FOR ELLECTRICALLY DRIVEMN</t>
         </is>
       </c>
       <c r="E1066" s="2" t="inlineStr">
         <is>
-          <t>ALTIS EM 2</t>
+          <t>MULTIS COMPLEX SHD 100</t>
         </is>
       </c>
       <c r="F1066" s="3" t="inlineStr">
@@ -39911,12 +39911,12 @@
       </c>
       <c r="D1067" s="4" t="inlineStr">
         <is>
-          <t>EGR CIRCULATION PUMP MOTOR FOR ELLECTRICALLY DRIVEMN</t>
+          <t>PUMP</t>
         </is>
       </c>
       <c r="E1067" s="4" t="inlineStr">
         <is>
-          <t>MULTIS COMPLEX SHD 100</t>
+          <t>MULTIS COMPLEX EP 3 [OR</t>
         </is>
       </c>
       <c r="F1067" s="5" t="inlineStr">
@@ -39948,12 +39948,12 @@
       </c>
       <c r="D1068" s="2" t="inlineStr">
         <is>
-          <t>PUMP</t>
+          <t>PUMP L.P BOOSTER PUMP</t>
         </is>
       </c>
       <c r="E1068" s="2" t="inlineStr">
         <is>
-          <t>MULTIS COMPLEX EP 3 [OR</t>
+          <t>MULTIS EP 3]</t>
         </is>
       </c>
       <c r="F1068" s="3" t="inlineStr">
@@ -39985,12 +39985,12 @@
       </c>
       <c r="D1069" s="4" t="inlineStr">
         <is>
-          <t>PUMP L.P BOOSTER PUMP</t>
+          <t>NAOH DOSING PUMP</t>
         </is>
       </c>
       <c r="E1069" s="4" t="inlineStr">
         <is>
-          <t>MULTIS EP 3]</t>
+          <t>TRANSELF TYPE B 80W90</t>
         </is>
       </c>
       <c r="F1069" s="5" t="inlineStr">
@@ -40022,12 +40022,12 @@
       </c>
       <c r="D1070" s="2" t="inlineStr">
         <is>
-          <t>NAOH DOSING PUMP</t>
+          <t>LDCL C.W. PUMP</t>
         </is>
       </c>
       <c r="E1070" s="2" t="inlineStr">
         <is>
-          <t>TRANSELF TYPE B 80W90</t>
+          <t>ALTIS EM 2</t>
         </is>
       </c>
       <c r="F1070" s="3" t="inlineStr">
@@ -40059,12 +40059,12 @@
       </c>
       <c r="D1071" s="4" t="inlineStr">
         <is>
-          <t>LDCL C.W. PUMP</t>
+          <t>FUEL VALVE TESTER</t>
         </is>
       </c>
       <c r="E1071" s="4" t="inlineStr">
         <is>
-          <t>ALTIS EM 2</t>
+          <t>VISGA 15</t>
         </is>
       </c>
       <c r="F1071" s="5" t="inlineStr">
@@ -40081,27 +40081,27 @@
     <row r="1072">
       <c r="A1072" s="2" t="inlineStr">
         <is>
-          <t>MAIN ENGINE</t>
+          <t>GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B1072" s="2" t="inlineStr">
         <is>
-          <t>HANWHA ENGINE HANMI HYDRAULIC</t>
+          <t>INDUSTRIES HYUNDAI HEAVY</t>
         </is>
       </c>
       <c r="C1072" s="2" t="inlineStr">
         <is>
-          <t>9G95ME-C10.5-LGIM-EGRTC</t>
+          <t>9H32DF-LM</t>
         </is>
       </c>
       <c r="D1072" s="2" t="inlineStr">
         <is>
-          <t>FUEL VALVE TESTER</t>
+          <t>L.O SUMP TANK &amp; LO COOLER</t>
         </is>
       </c>
       <c r="E1072" s="2" t="inlineStr">
         <is>
-          <t>VISGA 15</t>
+          <t>AURELIA TI 4040</t>
         </is>
       </c>
       <c r="F1072" s="3" t="inlineStr">
@@ -40138,7 +40138,7 @@
       </c>
       <c r="E1073" s="4" t="inlineStr">
         <is>
-          <t>AURELIA TI 4040</t>
+          <t>DISOLA M 4012</t>
         </is>
       </c>
       <c r="F1073" s="5" t="inlineStr">
@@ -40170,7 +40170,7 @@
       </c>
       <c r="D1074" s="2" t="inlineStr">
         <is>
-          <t>L.O SUMP TANK &amp; LO COOLER</t>
+          <t>LO CONSUMPTION (60DAYS X 1SET)</t>
         </is>
       </c>
       <c r="E1074" s="2" t="inlineStr">
@@ -40202,17 +40202,17 @@
       </c>
       <c r="C1075" s="4" t="inlineStr">
         <is>
-          <t>9H32DF-LM</t>
+          <t>7H32DF-LM</t>
         </is>
       </c>
       <c r="D1075" s="4" t="inlineStr">
         <is>
-          <t>LO CONSUMPTION (60DAYS X 1SET)</t>
+          <t>L.O SUMP TANK &amp; LO COOLER</t>
         </is>
       </c>
       <c r="E1075" s="4" t="inlineStr">
         <is>
-          <t>DISOLA M 4012</t>
+          <t>AURELIA TI 4040</t>
         </is>
       </c>
       <c r="F1075" s="5" t="inlineStr">
@@ -40249,7 +40249,7 @@
       </c>
       <c r="E1076" s="2" t="inlineStr">
         <is>
-          <t>AURELIA TI 4040</t>
+          <t>DISOLA M 4012</t>
         </is>
       </c>
       <c r="F1076" s="3" t="inlineStr">
@@ -40281,7 +40281,7 @@
       </c>
       <c r="D1077" s="4" t="inlineStr">
         <is>
-          <t>L.O SUMP TANK &amp; LO COOLER</t>
+          <t>LO CONSUMPTION (60DAYS X 1SET)</t>
         </is>
       </c>
       <c r="E1077" s="4" t="inlineStr">
@@ -40323,7 +40323,7 @@
       </c>
       <c r="E1078" s="2" t="inlineStr">
         <is>
-          <t>DISOLA M 4012</t>
+          <t>BAUER SPECIAL</t>
         </is>
       </c>
       <c r="F1078" s="3" t="inlineStr">
@@ -40345,22 +40345,22 @@
       </c>
       <c r="B1079" s="4" t="inlineStr">
         <is>
-          <t>INDUSTRIES HYUNDAI HEAVY</t>
+          <t>INDUSTRIES</t>
         </is>
       </c>
       <c r="C1079" s="4" t="inlineStr">
         <is>
-          <t>7H32DF-LM</t>
+          <t>H32DF-LM</t>
         </is>
       </c>
       <c r="D1079" s="4" t="inlineStr">
         <is>
-          <t>LO CONSUMPTION (60DAYS X 1SET)</t>
+          <t>N2 BOOSTER UNIT</t>
         </is>
       </c>
       <c r="E1079" s="4" t="inlineStr">
         <is>
-          <t>BAUER SPECIAL</t>
+          <t>COMPRESSOR</t>
         </is>
       </c>
       <c r="F1079" s="5" t="inlineStr">
@@ -40397,7 +40397,7 @@
       </c>
       <c r="E1080" s="2" t="inlineStr">
         <is>
-          <t>COMPRESSOR</t>
+          <t>OIL(SYNTHETIC OIL, N46641)</t>
         </is>
       </c>
       <c r="F1080" s="3" t="inlineStr">
@@ -40429,12 +40429,12 @@
       </c>
       <c r="D1081" s="4" t="inlineStr">
         <is>
-          <t>N2 BOOSTER UNIT</t>
+          <t>METHANOL-HIGH PRESSURE PUMP UNIT</t>
         </is>
       </c>
       <c r="E1081" s="4" t="inlineStr">
         <is>
-          <t>OIL(SYNTHETIC OIL, N46641)</t>
+          <t>VISGA 46</t>
         </is>
       </c>
       <c r="F1081" s="5" t="inlineStr">
@@ -40451,27 +40451,27 @@
     <row r="1082">
       <c r="A1082" s="2" t="inlineStr">
         <is>
-          <t>GENERATOR ENGINE</t>
+          <t>EMERGENCY GENSET</t>
         </is>
       </c>
       <c r="B1082" s="2" t="inlineStr">
         <is>
-          <t>INDUSTRIES</t>
+          <t>CMXD</t>
         </is>
       </c>
       <c r="C1082" s="2" t="inlineStr">
         <is>
-          <t>H32DF-LM</t>
+          <t>K19-DM</t>
         </is>
       </c>
       <c r="D1082" s="2" t="inlineStr">
         <is>
-          <t>METHANOL-HIGH PRESSURE PUMP UNIT</t>
+          <t>MAIN LO SYSTEM</t>
         </is>
       </c>
       <c r="E1082" s="2" t="inlineStr">
         <is>
-          <t>VISGA 46</t>
+          <t>DISOLA W 15W40</t>
         </is>
       </c>
       <c r="F1082" s="3" t="inlineStr">
@@ -40503,12 +40503,12 @@
       </c>
       <c r="D1083" s="4" t="inlineStr">
         <is>
-          <t>MAIN LO SYSTEM</t>
+          <t>MAIN LO SYSTEM HYDRAULIC STARTING UNIT_TANK &amp;</t>
         </is>
       </c>
       <c r="E1083" s="4" t="inlineStr">
         <is>
-          <t>DISOLA W 15W40</t>
+          <t>VISGA 32</t>
         </is>
       </c>
       <c r="F1083" s="5" t="inlineStr">
@@ -40525,27 +40525,27 @@
     <row r="1084">
       <c r="A1084" s="2" t="inlineStr">
         <is>
-          <t>EMERGENCY GENSET</t>
+          <t>H.F.O. PURIFIER</t>
         </is>
       </c>
       <c r="B1084" s="2" t="inlineStr">
         <is>
-          <t>CMXD</t>
+          <t>SAMGONG CO., LTD.</t>
         </is>
       </c>
       <c r="C1084" s="2" t="inlineStr">
         <is>
-          <t>K19-DM</t>
+          <t>SJ160HH</t>
         </is>
       </c>
       <c r="D1084" s="2" t="inlineStr">
         <is>
-          <t>MAIN LO SYSTEM HYDRAULIC STARTING UNIT_TANK &amp;</t>
+          <t>GEAR CASE</t>
         </is>
       </c>
       <c r="E1084" s="2" t="inlineStr">
         <is>
-          <t>VISGA 32</t>
+          <t>EPONA Z 150</t>
         </is>
       </c>
       <c r="F1084" s="3" t="inlineStr">
@@ -40577,7 +40577,7 @@
       </c>
       <c r="D1085" s="4" t="inlineStr">
         <is>
-          <t>GEAR CASE</t>
+          <t>FOR CONSUMPTION</t>
         </is>
       </c>
       <c r="E1085" s="4" t="inlineStr">
@@ -40599,7 +40599,7 @@
     <row r="1086">
       <c r="A1086" s="2" t="inlineStr">
         <is>
-          <t>H.F.O. PURIFIER</t>
+          <t>M.G.O. PURIFIER</t>
         </is>
       </c>
       <c r="B1086" s="2" t="inlineStr">
@@ -40609,12 +40609,12 @@
       </c>
       <c r="C1086" s="2" t="inlineStr">
         <is>
-          <t>SJ160HH</t>
+          <t>SJ60H</t>
         </is>
       </c>
       <c r="D1086" s="2" t="inlineStr">
         <is>
-          <t>FOR CONSUMPTION</t>
+          <t>GEAR CASE</t>
         </is>
       </c>
       <c r="E1086" s="2" t="inlineStr">
@@ -40651,7 +40651,7 @@
       </c>
       <c r="D1087" s="4" t="inlineStr">
         <is>
-          <t>GEAR CASE</t>
+          <t>FOR CONSUMPTION</t>
         </is>
       </c>
       <c r="E1087" s="4" t="inlineStr">
@@ -40673,7 +40673,7 @@
     <row r="1088">
       <c r="A1088" s="2" t="inlineStr">
         <is>
-          <t>M.G.O. PURIFIER</t>
+          <t>MAIN L.O. PURIFIER</t>
         </is>
       </c>
       <c r="B1088" s="2" t="inlineStr">
@@ -40683,7 +40683,7 @@
       </c>
       <c r="C1088" s="2" t="inlineStr">
         <is>
-          <t>SJ60H</t>
+          <t>SJ85H</t>
         </is>
       </c>
       <c r="D1088" s="2" t="inlineStr">
@@ -40725,7 +40725,7 @@
       </c>
       <c r="D1089" s="4" t="inlineStr">
         <is>
-          <t>FOR CONSUMPTION</t>
+          <t>GEAR CASE</t>
         </is>
       </c>
       <c r="E1089" s="4" t="inlineStr">
@@ -40747,17 +40747,17 @@
     <row r="1090">
       <c r="A1090" s="2" t="inlineStr">
         <is>
-          <t>MAIN L.O. PURIFIER</t>
+          <t>GE L.O. PURIFIER</t>
         </is>
       </c>
       <c r="B1090" s="2" t="inlineStr">
         <is>
-          <t>SAMGONG CO., LTD.</t>
+          <t>SAMGONG CO., LTD. J.P. SAUER &amp; SOHN</t>
         </is>
       </c>
       <c r="C1090" s="2" t="inlineStr">
         <is>
-          <t>SJ85H</t>
+          <t>SJ35H</t>
         </is>
       </c>
       <c r="D1090" s="2" t="inlineStr">
@@ -40799,7 +40799,7 @@
       </c>
       <c r="D1091" s="4" t="inlineStr">
         <is>
-          <t>GEAR CASE</t>
+          <t>FOR CONSUMPTION</t>
         </is>
       </c>
       <c r="E1091" s="4" t="inlineStr">
@@ -40821,27 +40821,27 @@
     <row r="1092">
       <c r="A1092" s="2" t="inlineStr">
         <is>
-          <t>GE L.O. PURIFIER</t>
+          <t>MAIN AIR COMPRESSOR SERVICE AIR COMPRESSOR(NEX-</t>
         </is>
       </c>
       <c r="B1092" s="2" t="inlineStr">
         <is>
-          <t>SAMGONG CO., LTD. J.P. SAUER &amp; SOHN</t>
+          <t>MASCHINENBAU GMBH</t>
         </is>
       </c>
       <c r="C1092" s="2" t="inlineStr">
         <is>
-          <t>SJ35H</t>
+          <t>WP460L</t>
         </is>
       </c>
       <c r="D1092" s="2" t="inlineStr">
         <is>
-          <t>FOR CONSUMPTION</t>
+          <t>CRANK CASE</t>
         </is>
       </c>
       <c r="E1092" s="2" t="inlineStr">
         <is>
-          <t>EPONA Z 150</t>
+          <t>DACNIS 100</t>
         </is>
       </c>
       <c r="F1092" s="3" t="inlineStr">
@@ -40873,7 +40873,7 @@
       </c>
       <c r="D1093" s="4" t="inlineStr">
         <is>
-          <t>CRANK CASE</t>
+          <t>FOR CONSUMPTION</t>
         </is>
       </c>
       <c r="E1093" s="4" t="inlineStr">
@@ -40895,27 +40895,27 @@
     <row r="1094">
       <c r="A1094" s="2" t="inlineStr">
         <is>
-          <t>MAIN AIR COMPRESSOR SERVICE AIR COMPRESSOR(NEX-</t>
+          <t>A/C PLANT</t>
         </is>
       </c>
       <c r="B1094" s="2" t="inlineStr">
         <is>
-          <t>MASCHINENBAU GMBH</t>
+          <t>HEINEN&amp;HOPMAN</t>
         </is>
       </c>
       <c r="C1094" s="2" t="inlineStr">
         <is>
-          <t>WP460L</t>
+          <t>DECK UNIT NO.1 &amp; 2</t>
         </is>
       </c>
       <c r="D1094" s="2" t="inlineStr">
         <is>
-          <t>FOR CONSUMPTION</t>
+          <t>COMPRESSOR</t>
         </is>
       </c>
       <c r="E1094" s="2" t="inlineStr">
         <is>
-          <t>DACNIS 100</t>
+          <t>[DANFOSS] POE 320SZ</t>
         </is>
       </c>
       <c r="F1094" s="3" t="inlineStr">
@@ -40932,7 +40932,7 @@
     <row r="1095">
       <c r="A1095" s="4" t="inlineStr">
         <is>
-          <t>A/C PLANT</t>
+          <t>PACKAGE TYPE UNIT COOLER</t>
         </is>
       </c>
       <c r="B1095" s="4" t="inlineStr">
@@ -40942,7 +40942,7 @@
       </c>
       <c r="C1095" s="4" t="inlineStr">
         <is>
-          <t>DECK UNIT NO.1 &amp; 2</t>
+          <t>GALLEY</t>
         </is>
       </c>
       <c r="D1095" s="4" t="inlineStr">
@@ -40952,7 +40952,7 @@
       </c>
       <c r="E1095" s="4" t="inlineStr">
         <is>
-          <t>[DANFOSS] POE 320SZ</t>
+          <t>[DANFOSS] POE RL32-3MAF</t>
         </is>
       </c>
       <c r="F1095" s="5" t="inlineStr">
@@ -40969,27 +40969,27 @@
     <row r="1096">
       <c r="A1096" s="2" t="inlineStr">
         <is>
-          <t>PACKAGE TYPE UNIT COOLER</t>
+          <t>NO.3) GENERATOR 5400KVA(NO.1 &amp;</t>
         </is>
       </c>
       <c r="B1096" s="2" t="inlineStr">
         <is>
-          <t>HEINEN&amp;HOPMAN</t>
+          <t>HDHE</t>
         </is>
       </c>
       <c r="C1096" s="2" t="inlineStr">
         <is>
-          <t>GALLEY</t>
+          <t>811-10P</t>
         </is>
       </c>
       <c r="D1096" s="2" t="inlineStr">
         <is>
-          <t>COMPRESSOR</t>
+          <t>NON-DRIVED END BEARING</t>
         </is>
       </c>
       <c r="E1096" s="2" t="inlineStr">
         <is>
-          <t>[DANFOSS] POE RL32-3MAF</t>
+          <t>AURELIA TI 4040</t>
         </is>
       </c>
       <c r="F1096" s="3" t="inlineStr">
@@ -41006,7 +41006,7 @@
     <row r="1097">
       <c r="A1097" s="4" t="inlineStr">
         <is>
-          <t>NO.3) GENERATOR 5400KVA(NO.1 &amp;</t>
+          <t>NO.4) GENERATOR 4200KVA(NO.2 &amp;</t>
         </is>
       </c>
       <c r="B1097" s="4" t="inlineStr">
@@ -41016,7 +41016,7 @@
       </c>
       <c r="C1097" s="4" t="inlineStr">
         <is>
-          <t>811-10P</t>
+          <t>805-10P</t>
         </is>
       </c>
       <c r="D1097" s="4" t="inlineStr">
@@ -41043,7 +41043,7 @@
     <row r="1098">
       <c r="A1098" s="2" t="inlineStr">
         <is>
-          <t>NO.4) GENERATOR 4200KVA(NO.2 &amp;</t>
+          <t>NO.3) GENERATOR 5400KVA(NO.1 &amp;</t>
         </is>
       </c>
       <c r="B1098" s="2" t="inlineStr">
@@ -41053,7 +41053,7 @@
       </c>
       <c r="C1098" s="2" t="inlineStr">
         <is>
-          <t>805-10P</t>
+          <t>811-10P</t>
         </is>
       </c>
       <c r="D1098" s="2" t="inlineStr">
@@ -41063,7 +41063,7 @@
       </c>
       <c r="E1098" s="2" t="inlineStr">
         <is>
-          <t>AURELIA TI 4040</t>
+          <t>DISOLA M 4012</t>
         </is>
       </c>
       <c r="F1098" s="3" t="inlineStr">
@@ -41080,27 +41080,27 @@
     <row r="1099">
       <c r="A1099" s="4" t="inlineStr">
         <is>
-          <t>NO.3) GENERATOR 5400KVA(NO.1 &amp;</t>
+          <t>AMP CABLE REEL</t>
         </is>
       </c>
       <c r="B1099" s="4" t="inlineStr">
         <is>
-          <t>HDHE</t>
+          <t>SAIERNICO</t>
         </is>
       </c>
       <c r="C1099" s="4" t="inlineStr">
         <is>
-          <t>811-10P</t>
+          <t>PORT</t>
         </is>
       </c>
       <c r="D1099" s="4" t="inlineStr">
         <is>
-          <t>NON-DRIVED END BEARING</t>
+          <t>REDUCER FOR REEL MOTOR</t>
         </is>
       </c>
       <c r="E1099" s="4" t="inlineStr">
         <is>
-          <t>DISOLA M 4012</t>
+          <t>TRAXIUM AXLE 7 80W90</t>
         </is>
       </c>
       <c r="F1099" s="5" t="inlineStr">
@@ -41132,12 +41132,12 @@
       </c>
       <c r="D1100" s="2" t="inlineStr">
         <is>
-          <t>REDUCER FOR REEL MOTOR</t>
+          <t>BEARING FOR ROTATE REEL</t>
         </is>
       </c>
       <c r="E1100" s="2" t="inlineStr">
         <is>
-          <t>TRAXIUM AXLE 7 80W90</t>
+          <t>CERAN XM 220</t>
         </is>
       </c>
       <c r="F1100" s="3" t="inlineStr">
@@ -41169,12 +41169,12 @@
       </c>
       <c r="D1101" s="4" t="inlineStr">
         <is>
-          <t>BEARING FOR ROTATE REEL</t>
+          <t>REDUCER FOR GUIDE MOTOR</t>
         </is>
       </c>
       <c r="E1101" s="4" t="inlineStr">
         <is>
-          <t>CERAN XM 220</t>
+          <t>TRAXIUM AXLE 7 80W90</t>
         </is>
       </c>
       <c r="F1101" s="5" t="inlineStr">
@@ -41206,12 +41206,12 @@
       </c>
       <c r="D1102" s="2" t="inlineStr">
         <is>
-          <t>REDUCER FOR GUIDE MOTOR</t>
+          <t>GEARS</t>
         </is>
       </c>
       <c r="E1102" s="2" t="inlineStr">
         <is>
-          <t>TRAXIUM AXLE 7 80W90</t>
+          <t>CERAN XM 220</t>
         </is>
       </c>
       <c r="F1102" s="3" t="inlineStr">
@@ -41233,22 +41233,22 @@
       </c>
       <c r="B1103" s="4" t="inlineStr">
         <is>
-          <t>SAIERNICO</t>
+          <t>SAIERNICO HD HYUNDAI</t>
         </is>
       </c>
       <c r="C1103" s="4" t="inlineStr">
         <is>
-          <t>PORT</t>
+          <t>STBD</t>
         </is>
       </c>
       <c r="D1103" s="4" t="inlineStr">
         <is>
-          <t>GEARS</t>
+          <t>REDUCER FOR REEL MOTOR</t>
         </is>
       </c>
       <c r="E1103" s="4" t="inlineStr">
         <is>
-          <t>CERAN XM 220</t>
+          <t>TRAXIUM AXLE 7 80W90</t>
         </is>
       </c>
       <c r="F1103" s="5" t="inlineStr">
@@ -41280,7 +41280,7 @@
       </c>
       <c r="D1104" s="2" t="inlineStr">
         <is>
-          <t>REDUCER FOR REEL MOTOR</t>
+          <t>REDUCER FOR GUIDE MOTOR</t>
         </is>
       </c>
       <c r="E1104" s="2" t="inlineStr">
@@ -41317,12 +41317,12 @@
       </c>
       <c r="D1105" s="4" t="inlineStr">
         <is>
-          <t>REDUCER FOR GUIDE MOTOR</t>
+          <t>GEARS</t>
         </is>
       </c>
       <c r="E1105" s="4" t="inlineStr">
         <is>
-          <t>TRAXIUM AXLE 7 80W90</t>
+          <t>CERAN XM 220</t>
         </is>
       </c>
       <c r="F1105" s="5" t="inlineStr">
@@ -41354,7 +41354,7 @@
       </c>
       <c r="D1106" s="2" t="inlineStr">
         <is>
-          <t>GEARS</t>
+          <t>BEARING FOR ROTATE REEL</t>
         </is>
       </c>
       <c r="E1106" s="2" t="inlineStr">
@@ -41368,43 +41368,6 @@
         </is>
       </c>
       <c r="G1106" s="2" t="inlineStr">
-        <is>
-          <t>SN2672 76 79 81 83 85 L.O chart(TOTAL)_HSHFO_rev.D_2025-09-19.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1107">
-      <c r="A1107" s="4" t="inlineStr">
-        <is>
-          <t>AMP CABLE REEL</t>
-        </is>
-      </c>
-      <c r="B1107" s="4" t="inlineStr">
-        <is>
-          <t>SAIERNICO HD HYUNDAI</t>
-        </is>
-      </c>
-      <c r="C1107" s="4" t="inlineStr">
-        <is>
-          <t>STBD</t>
-        </is>
-      </c>
-      <c r="D1107" s="4" t="inlineStr">
-        <is>
-          <t>BEARING FOR ROTATE REEL</t>
-        </is>
-      </c>
-      <c r="E1107" s="4" t="inlineStr">
-        <is>
-          <t>CERAN XM 220</t>
-        </is>
-      </c>
-      <c r="F1107" s="5" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1107" s="4" t="inlineStr">
         <is>
           <t>SN2672 76 79 81 83 85 L.O chart(TOTAL)_HSHFO_rev.D_2025-09-19.pdf</t>
         </is>

</xml_diff>

<commit_message>
data: update 2026-04-26 12:14
</commit_message>
<xml_diff>
--- a/output/nb_master.xlsx
+++ b/output/nb_master.xlsx
@@ -3938,7 +3938,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>TURNING GEAR</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -4654,7 +4654,7 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>HYDR. SYSTEM</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
@@ -4691,7 +4691,7 @@
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>HYDR.SYSTEM OIL</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E115" s="4" t="inlineStr">
@@ -4987,7 +4987,7 @@
       </c>
       <c r="D123" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E123" s="4" t="inlineStr">
@@ -5098,7 +5098,7 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>LUBE.OIL FOR GEARBOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
@@ -5172,7 +5172,7 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -5283,7 +5283,7 @@
       </c>
       <c r="D131" s="4" t="inlineStr">
         <is>
-          <t>HYDR. SYSTEM</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E131" s="4" t="inlineStr">
@@ -5320,7 +5320,7 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
@@ -5431,7 +5431,7 @@
       </c>
       <c r="D135" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E135" s="4" t="inlineStr">
@@ -5616,7 +5616,7 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="D143" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E143" s="4" t="inlineStr">
@@ -9801,7 +9801,7 @@
       </c>
       <c r="D253" s="4" t="inlineStr">
         <is>
-          <t>ENCLOSED GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E253" s="4" t="inlineStr">
@@ -9875,7 +9875,7 @@
       </c>
       <c r="D255" s="4" t="inlineStr">
         <is>
-          <t>HYDRAULIC OIL(SYSTEM OIL)</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E255" s="4" t="inlineStr">
@@ -9912,7 +9912,7 @@
       </c>
       <c r="D256" s="2" t="inlineStr">
         <is>
-          <t>ENCLOSED GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E256" s="2" t="inlineStr">
@@ -10023,7 +10023,7 @@
       </c>
       <c r="D259" s="4" t="inlineStr">
         <is>
-          <t>ENCLOSED GEAR-</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E259" s="4" t="inlineStr">
@@ -10504,7 +10504,7 @@
       </c>
       <c r="D272" s="2" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E272" s="2" t="inlineStr">
@@ -10985,7 +10985,7 @@
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t>TURNING GEAR</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E285" s="4" t="inlineStr">
@@ -11244,7 +11244,7 @@
       </c>
       <c r="D292" s="2" t="inlineStr">
         <is>
-          <t>TURNING GEAR</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E292" s="2" t="inlineStr">
@@ -11943,7 +11943,7 @@
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>GEAR OIL</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E311" s="4" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E323" s="4" t="inlineStr">
@@ -12494,7 +12494,7 @@
       </c>
       <c r="D326" s="2" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E326" s="2" t="inlineStr">
@@ -12605,7 +12605,7 @@
       </c>
       <c r="D329" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E329" s="4" t="inlineStr">
@@ -12790,7 +12790,7 @@
       </c>
       <c r="D334" s="2" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E334" s="2" t="inlineStr">
@@ -13012,7 +13012,7 @@
       </c>
       <c r="D340" s="2" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E340" s="2" t="inlineStr">
@@ -13123,7 +13123,7 @@
       </c>
       <c r="D343" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E343" s="4" t="inlineStr">
@@ -13419,7 +13419,7 @@
       </c>
       <c r="D351" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E351" s="4" t="inlineStr">
@@ -13900,7 +13900,7 @@
       </c>
       <c r="D364" s="2" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E364" s="2" t="inlineStr">
@@ -14344,7 +14344,7 @@
       </c>
       <c r="D376" s="2" t="inlineStr">
         <is>
-          <t>TURING GEAR</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E376" s="2" t="inlineStr">
@@ -15713,7 +15713,7 @@
       </c>
       <c r="D413" s="4" t="inlineStr">
         <is>
-          <t>HYDR. SYSTEM</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E413" s="4" t="inlineStr">
@@ -15935,7 +15935,7 @@
       </c>
       <c r="D419" s="4" t="inlineStr">
         <is>
-          <t>HYDR. SYSTEM</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E419" s="4" t="inlineStr">
@@ -16157,7 +16157,7 @@
       </c>
       <c r="D425" s="4" t="inlineStr">
         <is>
-          <t>HYDR. SYSTEM</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E425" s="4" t="inlineStr">
@@ -16453,7 +16453,7 @@
       </c>
       <c r="D433" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E433" s="4" t="inlineStr">
@@ -16564,7 +16564,7 @@
       </c>
       <c r="D436" s="2" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E436" s="2" t="inlineStr">
@@ -16786,7 +16786,7 @@
       </c>
       <c r="D442" s="2" t="inlineStr">
         <is>
-          <t>HYDR. SYSTEM</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E442" s="2" t="inlineStr">
@@ -16971,7 +16971,7 @@
       </c>
       <c r="D447" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E447" s="4" t="inlineStr">
@@ -17156,7 +17156,7 @@
       </c>
       <c r="D452" s="2" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E452" s="2" t="inlineStr">
@@ -17267,7 +17267,7 @@
       </c>
       <c r="D455" s="4" t="inlineStr">
         <is>
-          <t>HYDR. SYSTEM</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E455" s="4" t="inlineStr">
@@ -17489,7 +17489,7 @@
       </c>
       <c r="D461" s="4" t="inlineStr">
         <is>
-          <t>HYDR. SYSTEM</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E461" s="4" t="inlineStr">
@@ -17526,7 +17526,7 @@
       </c>
       <c r="D462" s="2" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E462" s="2" t="inlineStr">
@@ -18266,7 +18266,7 @@
       </c>
       <c r="D482" s="2" t="inlineStr">
         <is>
-          <t>HYDR. SYSTEM</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E482" s="2" t="inlineStr">
@@ -18562,7 +18562,7 @@
       </c>
       <c r="D490" s="2" t="inlineStr">
         <is>
-          <t>HYDR. SYSTEM</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E490" s="2" t="inlineStr">
@@ -22669,7 +22669,7 @@
       </c>
       <c r="D601" s="4" t="inlineStr">
         <is>
-          <t>GEAR</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E601" s="4" t="inlineStr">
@@ -23298,7 +23298,7 @@
       </c>
       <c r="D618" s="2" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E618" s="2" t="inlineStr">
@@ -23631,7 +23631,7 @@
       </c>
       <c r="D627" s="4" t="inlineStr">
         <is>
-          <t>ENCLOSED GEAR-</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E627" s="4" t="inlineStr">
@@ -23779,7 +23779,7 @@
       </c>
       <c r="D631" s="4" t="inlineStr">
         <is>
-          <t>ENCLOSED GEAR-</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E631" s="4" t="inlineStr">
@@ -24297,7 +24297,7 @@
       </c>
       <c r="D645" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>GEAR BOX-</t>
         </is>
       </c>
       <c r="E645" s="4" t="inlineStr">
@@ -24482,7 +24482,7 @@
       </c>
       <c r="D650" s="2" t="inlineStr">
         <is>
-          <t>GEAR</t>
+          <t>GEAR-</t>
         </is>
       </c>
       <c r="E650" s="2" t="inlineStr">
@@ -24889,7 +24889,7 @@
       </c>
       <c r="D661" s="4" t="inlineStr">
         <is>
-          <t>ENCLOSED GEAR-</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E661" s="4" t="inlineStr">
@@ -25259,7 +25259,7 @@
       </c>
       <c r="D671" s="4" t="inlineStr">
         <is>
-          <t>ENCLOSED GEARS</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E671" s="4" t="inlineStr">
@@ -25296,7 +25296,7 @@
       </c>
       <c r="D672" s="2" t="inlineStr">
         <is>
-          <t>ENCLOSED GEARS</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E672" s="2" t="inlineStr">
@@ -25407,7 +25407,7 @@
       </c>
       <c r="D675" s="4" t="inlineStr">
         <is>
-          <t>ENCLOSED GEAR-</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E675" s="4" t="inlineStr">
@@ -25925,7 +25925,7 @@
       </c>
       <c r="D689" s="4" t="inlineStr">
         <is>
-          <t>TURNING GEAR</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E689" s="4" t="inlineStr">
@@ -26850,7 +26850,7 @@
       </c>
       <c r="D714" s="2" t="inlineStr">
         <is>
-          <t>GEAR</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E714" s="2" t="inlineStr">
@@ -26887,7 +26887,7 @@
       </c>
       <c r="D715" s="4" t="inlineStr">
         <is>
-          <t>HYDR.OIL</t>
+          <t>HYDR. OIL</t>
         </is>
       </c>
       <c r="E715" s="4" t="inlineStr">
@@ -26998,7 +26998,7 @@
       </c>
       <c r="D718" s="2" t="inlineStr">
         <is>
-          <t>HYDR.OIL</t>
+          <t>HYDR. OIL</t>
         </is>
       </c>
       <c r="E718" s="2" t="inlineStr">
@@ -27146,7 +27146,7 @@
       </c>
       <c r="D722" s="2" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E722" s="2" t="inlineStr">
@@ -27294,7 +27294,7 @@
       </c>
       <c r="D726" s="2" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E726" s="2" t="inlineStr">
@@ -27368,7 +27368,7 @@
       </c>
       <c r="D728" s="2" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E728" s="2" t="inlineStr">
@@ -27479,7 +27479,7 @@
       </c>
       <c r="D731" s="4" t="inlineStr">
         <is>
-          <t>INCLOSED GEAR</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E731" s="4" t="inlineStr">
@@ -27590,7 +27590,7 @@
       </c>
       <c r="D734" s="2" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E734" s="2" t="inlineStr">
@@ -27775,7 +27775,7 @@
       </c>
       <c r="D739" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E739" s="4" t="inlineStr">
@@ -27849,7 +27849,7 @@
       </c>
       <c r="D741" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E741" s="4" t="inlineStr">
@@ -27997,7 +27997,7 @@
       </c>
       <c r="D745" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E745" s="4" t="inlineStr">
@@ -28404,7 +28404,7 @@
       </c>
       <c r="D756" s="2" t="inlineStr">
         <is>
-          <t>HYDR.OIL</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E756" s="2" t="inlineStr">
@@ -28441,7 +28441,7 @@
       </c>
       <c r="D757" s="4" t="inlineStr">
         <is>
-          <t>HYDR.OIL</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E757" s="4" t="inlineStr">
@@ -29181,7 +29181,7 @@
       </c>
       <c r="D777" s="4" t="inlineStr">
         <is>
-          <t>A.HYDRAULIC SYSTEM</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E777" s="4" t="inlineStr">
@@ -29292,7 +29292,7 @@
       </c>
       <c r="D780" s="2" t="inlineStr">
         <is>
-          <t>A.HYDRAULIC SYSTEM</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E780" s="2" t="inlineStr">
@@ -29440,7 +29440,7 @@
       </c>
       <c r="D784" s="2" t="inlineStr">
         <is>
-          <t>A.HYDRAULIC SYSTEM</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E784" s="2" t="inlineStr">
@@ -29514,7 +29514,7 @@
       </c>
       <c r="D786" s="2" t="inlineStr">
         <is>
-          <t>HYDRAULIC OIL</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E786" s="2" t="inlineStr">
@@ -29551,7 +29551,7 @@
       </c>
       <c r="D787" s="4" t="inlineStr">
         <is>
-          <t>ENCLOSED GEAR-</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E787" s="4" t="inlineStr">
@@ -29884,7 +29884,7 @@
       </c>
       <c r="D796" s="2" t="inlineStr">
         <is>
-          <t>B.LUBE. OIL FOR GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E796" s="2" t="inlineStr">
@@ -30772,7 +30772,7 @@
       </c>
       <c r="D820" s="2" t="inlineStr">
         <is>
-          <t>TURING GEAR</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E820" s="2" t="inlineStr">
@@ -32178,7 +32178,7 @@
       </c>
       <c r="D858" s="2" t="inlineStr">
         <is>
-          <t>GEAR OIL</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E858" s="2" t="inlineStr">
@@ -32437,7 +32437,7 @@
       </c>
       <c r="D865" s="4" t="inlineStr">
         <is>
-          <t>GEAR OIL</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E865" s="4" t="inlineStr">
@@ -32918,7 +32918,7 @@
       </c>
       <c r="D878" s="2" t="inlineStr">
         <is>
-          <t>ENCLOSE GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E878" s="2" t="inlineStr">
@@ -32992,7 +32992,7 @@
       </c>
       <c r="D880" s="2" t="inlineStr">
         <is>
-          <t>HYDRAULIC OIL (UNIT)</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E880" s="2" t="inlineStr">
@@ -33029,7 +33029,7 @@
       </c>
       <c r="D881" s="4" t="inlineStr">
         <is>
-          <t>HYDRAULIC OIL</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E881" s="4" t="inlineStr">
@@ -33066,7 +33066,7 @@
       </c>
       <c r="D882" s="2" t="inlineStr">
         <is>
-          <t>HYDRAULIC OIL</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E882" s="2" t="inlineStr">
@@ -33177,7 +33177,7 @@
       </c>
       <c r="D885" s="4" t="inlineStr">
         <is>
-          <t>ENCLOSE GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E885" s="4" t="inlineStr">
@@ -33214,7 +33214,7 @@
       </c>
       <c r="D886" s="2" t="inlineStr">
         <is>
-          <t>HYDRAULIC OIL</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E886" s="2" t="inlineStr">
@@ -33325,7 +33325,7 @@
       </c>
       <c r="D889" s="4" t="inlineStr">
         <is>
-          <t>ENCLOSE GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E889" s="4" t="inlineStr">
@@ -33584,7 +33584,7 @@
       </c>
       <c r="D896" s="2" t="inlineStr">
         <is>
-          <t>HYDRAULIC OIL</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E896" s="2" t="inlineStr">
@@ -33695,7 +33695,7 @@
       </c>
       <c r="D899" s="4" t="inlineStr">
         <is>
-          <t>ENCLOSE GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E899" s="4" t="inlineStr">
@@ -33769,7 +33769,7 @@
       </c>
       <c r="D901" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOX</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E901" s="4" t="inlineStr">
@@ -33954,7 +33954,7 @@
       </c>
       <c r="D906" s="2" t="inlineStr">
         <is>
-          <t>HYDR.OIL</t>
+          <t>HYDRAULIC SYSTEM</t>
         </is>
       </c>
       <c r="E906" s="2" t="inlineStr">
@@ -37765,7 +37765,7 @@
       </c>
       <c r="D1009" s="4" t="inlineStr">
         <is>
-          <t>TURNING GEAR</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E1009" s="4" t="inlineStr">
@@ -37876,7 +37876,7 @@
       </c>
       <c r="D1012" s="2" t="inlineStr">
         <is>
-          <t>TURNING GEAR</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E1012" s="2" t="inlineStr">
@@ -41206,7 +41206,7 @@
       </c>
       <c r="D1102" s="2" t="inlineStr">
         <is>
-          <t>GEARS</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E1102" s="2" t="inlineStr">
@@ -41317,7 +41317,7 @@
       </c>
       <c r="D1105" s="4" t="inlineStr">
         <is>
-          <t>GEARS</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E1105" s="4" t="inlineStr">

</xml_diff>

<commit_message>
data: update 2026-04-27 11:32
</commit_message>
<xml_diff>
--- a/output/nb_master.xlsx
+++ b/output/nb_master.xlsx
@@ -2842,8 +2842,7 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>D/G ENGINE
-&amp; GENERATOR</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
@@ -5928,8 +5927,7 @@
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>AUX. GENERATOR DIESEL
-ENGINE &amp; AC GENERATOR</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B149" s="4" t="inlineStr">
@@ -6867,7 +6865,7 @@
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>A/E</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
@@ -6904,7 +6902,7 @@
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>A/E</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
@@ -6941,7 +6939,7 @@
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>A/E</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
@@ -7163,7 +7161,7 @@
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>A/E</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
@@ -7200,7 +7198,7 @@
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>A/E</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B183" s="4" t="inlineStr">
@@ -7237,7 +7235,7 @@
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>A/E</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
@@ -7899,7 +7897,7 @@
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>GENERATOR ENGINE</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
@@ -7936,7 +7934,7 @@
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>GENERATOR ENGINE</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
@@ -7973,7 +7971,7 @@
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>GENERATOR ENGINE</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
@@ -22321,7 +22319,7 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>DIESEL GENERATOR 3 SETS</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B592" s="2" t="inlineStr">
@@ -25022,7 +25020,7 @@
     <row r="665">
       <c r="A665" s="4" t="inlineStr">
         <is>
-          <t>GENERATOR DIESEL ENGINE</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B665" s="4" t="inlineStr">
@@ -28167,7 +28165,7 @@
     <row r="750">
       <c r="A750" s="2" t="inlineStr">
         <is>
-          <t>A/E</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B750" s="2" t="inlineStr">
@@ -28204,7 +28202,7 @@
     <row r="751">
       <c r="A751" s="4" t="inlineStr">
         <is>
-          <t>A/E</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B751" s="4" t="inlineStr">
@@ -28241,7 +28239,7 @@
     <row r="752">
       <c r="A752" s="2" t="inlineStr">
         <is>
-          <t>A/E</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B752" s="2" t="inlineStr">
@@ -30646,7 +30644,7 @@
     <row r="817">
       <c r="A817" s="4" t="inlineStr">
         <is>
-          <t>AUXILIARY ENGINE</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B817" s="4" t="inlineStr">
@@ -30683,7 +30681,7 @@
     <row r="818">
       <c r="A818" s="2" t="inlineStr">
         <is>
-          <t>AUXILIARY ENGINE</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B818" s="2" t="inlineStr">
@@ -30720,7 +30718,7 @@
     <row r="819">
       <c r="A819" s="4" t="inlineStr">
         <is>
-          <t>AUXILIARY ENGINE</t>
+          <t>DIESEL GENERATOR ENGINE</t>
         </is>
       </c>
       <c r="B819" s="4" t="inlineStr">

</xml_diff>

<commit_message>
data: update 2026-04-27 11:49
</commit_message>
<xml_diff>
--- a/output/nb_master.xlsx
+++ b/output/nb_master.xlsx
@@ -785,7 +785,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>BEARINGS SPINDLE BOWL</t>
+          <t>BEARING SPINDLE BOWL</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>BEARINGS SPINDLE BOWL</t>
+          <t>BEARING SPINDLE BOWL</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -2820,7 +2820,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL - CYLINDER (CYL.O.STOR.TK, CONSUMPTION - GEAR BOX - SHAFT - BEARINGS - HYD.HIGH PRESSURE PUMP - FUEL VALVE TEST</t>
+          <t>SYSTEM OIL - CYLINDER (CYL.O.STOR.TK, CONSUMPTION - GEAR BOX - SHAFT - BEARING - HYD.HIGH PRESSURE PUMP - FUEL VALVE TEST</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -3044,7 +3044,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -3082,7 +3082,7 @@
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -4159,7 +4159,7 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>OIL LUBRICATION</t>
+          <t>OIL POINT</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -4196,7 +4196,7 @@
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E101" s="4" t="inlineStr">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -4270,7 +4270,7 @@
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E103" s="4" t="inlineStr">
@@ -4307,7 +4307,7 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -4344,7 +4344,7 @@
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E105" s="4" t="inlineStr">
@@ -4505,7 +4505,7 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>TRAVELING&amp;LIFTING GEARS BOX</t>
+          <t>TRAVELING&amp;LIFTING GEAR BOX</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
@@ -5905,7 +5905,7 @@
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL - CYLINDER (CYL.O.STOR.TK, CONSUMPTION - GEAR BOX - SHAFT - BEARINGS - HYD. HIGH PRESSURE PUMP - FUEL VALVE TEST - HYD.HIGH PRESSURE PUMP</t>
+          <t>SYSTEM OIL - CYLINDER (CYL.O.STOR.TK, CONSUMPTION - GEAR BOX - SHAFT - BEARING - HYD. HIGH PRESSURE PUMP - FUEL VALVE TEST - HYD.HIGH PRESSURE PUMP</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
@@ -6130,7 +6130,7 @@
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
@@ -6319,7 +6319,7 @@
       </c>
       <c r="D159" s="4" t="inlineStr">
         <is>
-          <t>MOTOR FOR PUMP - CYLINDER BODY SEALS - PISTON SEALS -END COVER SEALS - CYLINDER BODY SEALS - PISTON SEALS - END COVER SEALS - BEARING - BEARING - BEARING - BEARING</t>
+          <t>MOTOR FOR PUMP - CYLINDER BODY SEAL - PISTON SEAL -END COVER SEAL - CYLINDER BODY SEAL - PISTON SEAL - END COVER SEAL - BEARING - BEARING - BEARING - BEARING</t>
         </is>
       </c>
       <c r="E159" s="4" t="inlineStr">
@@ -6806,7 +6806,7 @@
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E172" s="2" t="inlineStr">
@@ -6880,7 +6880,7 @@
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E174" s="2" t="inlineStr">
@@ -7028,7 +7028,7 @@
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
@@ -7065,7 +7065,7 @@
       </c>
       <c r="D179" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E179" s="4" t="inlineStr">
@@ -7176,7 +7176,7 @@
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E182" s="2" t="inlineStr">
@@ -7357,7 +7357,7 @@
       </c>
       <c r="D187" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E187" s="4" t="inlineStr">
@@ -7912,7 +7912,7 @@
       </c>
       <c r="D202" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E202" s="2" t="inlineStr">
@@ -8504,7 +8504,7 @@
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E218" s="2" t="inlineStr">
@@ -8541,7 +8541,7 @@
       </c>
       <c r="D219" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E219" s="4" t="inlineStr">
@@ -8763,7 +8763,7 @@
       </c>
       <c r="D225" s="4" t="inlineStr">
         <is>
-          <t>BEARINGS</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="E225" s="4" t="inlineStr">
@@ -9651,7 +9651,7 @@
       </c>
       <c r="D249" s="4" t="inlineStr">
         <is>
-          <t>BEARINGS</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="E249" s="4" t="inlineStr">
@@ -9762,7 +9762,7 @@
       </c>
       <c r="D252" s="2" t="inlineStr">
         <is>
-          <t>BEARINGS</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="E252" s="2" t="inlineStr">
@@ -10021,7 +10021,7 @@
       </c>
       <c r="D259" s="4" t="inlineStr">
         <is>
-          <t>GREASE NIPPLE</t>
+          <t>GREASE POINT</t>
         </is>
       </c>
       <c r="E259" s="4" t="inlineStr">
@@ -10613,7 +10613,7 @@
       </c>
       <c r="D275" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E275" s="4" t="inlineStr">
@@ -11205,7 +11205,7 @@
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>/ HOISTING/TRAVELING GEARS BOX</t>
+          <t>/ HOISTING/TRAVELING GEAR BOX</t>
         </is>
       </c>
       <c r="E291" s="4" t="inlineStr">
@@ -11242,7 +11242,7 @@
       </c>
       <c r="D292" s="2" t="inlineStr">
         <is>
-          <t>ROLLING BEARINGS</t>
+          <t>ROLLING BEARING</t>
         </is>
       </c>
       <c r="E292" s="2" t="inlineStr">
@@ -12085,7 +12085,7 @@
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>WIRE ROPES &amp; OPEN GEAR</t>
+          <t>WIRE ROPE &amp; OPEN GEAR</t>
         </is>
       </c>
       <c r="E315" s="4" t="inlineStr">
@@ -12196,7 +12196,7 @@
       </c>
       <c r="D318" s="2" t="inlineStr">
         <is>
-          <t>WIRE ROPES-</t>
+          <t>WIRE ROPE</t>
         </is>
       </c>
       <c r="E318" s="2" t="inlineStr">
@@ -12492,7 +12492,7 @@
       </c>
       <c r="D326" s="2" t="inlineStr">
         <is>
-          <t>GREASE POINTS</t>
+          <t>GREASE POINT</t>
         </is>
       </c>
       <c r="E326" s="2" t="inlineStr">
@@ -12566,7 +12566,7 @@
       </c>
       <c r="D328" s="2" t="inlineStr">
         <is>
-          <t>GREASE POINTS</t>
+          <t>GREASE POINT</t>
         </is>
       </c>
       <c r="E328" s="2" t="inlineStr">
@@ -12640,7 +12640,7 @@
       </c>
       <c r="D330" s="2" t="inlineStr">
         <is>
-          <t>GREASE POINTS</t>
+          <t>GREASE POINT</t>
         </is>
       </c>
       <c r="E330" s="2" t="inlineStr">
@@ -12751,7 +12751,7 @@
       </c>
       <c r="D333" s="4" t="inlineStr">
         <is>
-          <t>GREASE POINTS</t>
+          <t>GREASE POINT</t>
         </is>
       </c>
       <c r="E333" s="4" t="inlineStr">
@@ -12899,7 +12899,7 @@
       </c>
       <c r="D337" s="4" t="inlineStr">
         <is>
-          <t>WIRE ROPES-</t>
+          <t>WIRE ROPE</t>
         </is>
       </c>
       <c r="E337" s="4" t="inlineStr">
@@ -13047,7 +13047,7 @@
       </c>
       <c r="D341" s="4" t="inlineStr">
         <is>
-          <t>GREASE POINTS</t>
+          <t>GREASE POINT</t>
         </is>
       </c>
       <c r="E341" s="4" t="inlineStr">
@@ -13676,7 +13676,7 @@
       </c>
       <c r="D358" s="2" t="inlineStr">
         <is>
-          <t>CRANK CASE AND BEARINGS</t>
+          <t>CRANK CASE AND BEARING</t>
         </is>
       </c>
       <c r="E358" s="2" t="inlineStr">
@@ -13824,7 +13824,7 @@
       </c>
       <c r="D362" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E362" s="2" t="inlineStr">
@@ -14342,7 +14342,7 @@
       </c>
       <c r="D376" s="2" t="inlineStr">
         <is>
-          <t>OIL LUBRICATION</t>
+          <t>OIL POINT</t>
         </is>
       </c>
       <c r="E376" s="2" t="inlineStr">
@@ -14379,7 +14379,7 @@
       </c>
       <c r="D377" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E377" s="4" t="inlineStr">
@@ -14490,7 +14490,7 @@
       </c>
       <c r="D380" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E380" s="2" t="inlineStr">
@@ -14527,7 +14527,7 @@
       </c>
       <c r="D381" s="4" t="inlineStr">
         <is>
-          <t>OIL LUBRICATION</t>
+          <t>OIL POINT</t>
         </is>
       </c>
       <c r="E381" s="4" t="inlineStr">
@@ -14564,7 +14564,7 @@
       </c>
       <c r="D382" s="2" t="inlineStr">
         <is>
-          <t>OIL LUBRICATION</t>
+          <t>OIL POINT</t>
         </is>
       </c>
       <c r="E382" s="2" t="inlineStr">
@@ -14601,7 +14601,7 @@
       </c>
       <c r="D383" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E383" s="4" t="inlineStr">
@@ -14638,7 +14638,7 @@
       </c>
       <c r="D384" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E384" s="2" t="inlineStr">
@@ -14675,7 +14675,7 @@
       </c>
       <c r="D385" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E385" s="4" t="inlineStr">
@@ -14712,7 +14712,7 @@
       </c>
       <c r="D386" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E386" s="2" t="inlineStr">
@@ -14749,7 +14749,7 @@
       </c>
       <c r="D387" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E387" s="4" t="inlineStr">
@@ -14786,7 +14786,7 @@
       </c>
       <c r="D388" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E388" s="2" t="inlineStr">
@@ -14860,7 +14860,7 @@
       </c>
       <c r="D390" s="2" t="inlineStr">
         <is>
-          <t>TURNING POINT,OPEN GEARS AND BEARING</t>
+          <t>TURNING POINT,OPEN GEAR AND BEARING</t>
         </is>
       </c>
       <c r="E390" s="2" t="inlineStr">
@@ -15119,7 +15119,7 @@
       </c>
       <c r="D397" s="4" t="inlineStr">
         <is>
-          <t>PUMP BEARING OIL POINTS</t>
+          <t>PUMP BEARING OIL POINT</t>
         </is>
       </c>
       <c r="E397" s="4" t="inlineStr">
@@ -16969,7 +16969,7 @@
       </c>
       <c r="D447" s="4" t="inlineStr">
         <is>
-          <t>AIR MOTOR OIL POINTS</t>
+          <t>AIR MOTOR OIL POINT</t>
         </is>
       </c>
       <c r="E447" s="4" t="inlineStr">
@@ -17080,7 +17080,7 @@
       </c>
       <c r="D450" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E450" s="2" t="inlineStr">
@@ -17413,7 +17413,7 @@
       </c>
       <c r="D459" s="4" t="inlineStr">
         <is>
-          <t>DEEPWELL PUMP MOTOR-ABB DRIVE END -</t>
+          <t>DEEPWELL PUMP MOTOR-ABB DRIVE END</t>
         </is>
       </c>
       <c r="E459" s="4" t="inlineStr">
@@ -17635,7 +17635,7 @@
       </c>
       <c r="D465" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E465" s="4" t="inlineStr">
@@ -17672,7 +17672,7 @@
       </c>
       <c r="D466" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E466" s="2" t="inlineStr">
@@ -17820,7 +17820,7 @@
       </c>
       <c r="D470" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E470" s="2" t="inlineStr">
@@ -17968,7 +17968,7 @@
       </c>
       <c r="D474" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E474" s="2" t="inlineStr">
@@ -18005,7 +18005,7 @@
       </c>
       <c r="D475" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E475" s="4" t="inlineStr">
@@ -18042,7 +18042,7 @@
       </c>
       <c r="D476" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E476" s="2" t="inlineStr">
@@ -18930,7 +18930,7 @@
       </c>
       <c r="D500" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E500" s="2" t="inlineStr">
@@ -19189,7 +19189,7 @@
       </c>
       <c r="D507" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E507" s="4" t="inlineStr">
@@ -19226,7 +19226,7 @@
       </c>
       <c r="D508" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E508" s="2" t="inlineStr">
@@ -19263,7 +19263,7 @@
       </c>
       <c r="D509" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E509" s="4" t="inlineStr">
@@ -19300,7 +19300,7 @@
       </c>
       <c r="D510" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E510" s="2" t="inlineStr">
@@ -20447,7 +20447,7 @@
       </c>
       <c r="D541" s="4" t="inlineStr">
         <is>
-          <t>BEARINGS</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="E541" s="4" t="inlineStr">
@@ -20484,7 +20484,7 @@
       </c>
       <c r="D542" s="2" t="inlineStr">
         <is>
-          <t>OILER</t>
+          <t>OIL POINT</t>
         </is>
       </c>
       <c r="E542" s="2" t="inlineStr">
@@ -20706,7 +20706,7 @@
       </c>
       <c r="D548" s="2" t="inlineStr">
         <is>
-          <t>BEARINGS</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="E548" s="2" t="inlineStr">
@@ -20743,7 +20743,7 @@
       </c>
       <c r="D549" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E549" s="4" t="inlineStr">
@@ -20891,7 +20891,7 @@
       </c>
       <c r="D553" s="4" t="inlineStr">
         <is>
-          <t>BEARINGS</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="E553" s="4" t="inlineStr">
@@ -20928,7 +20928,7 @@
       </c>
       <c r="D554" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E554" s="2" t="inlineStr">
@@ -21076,7 +21076,7 @@
       </c>
       <c r="D558" s="2" t="inlineStr">
         <is>
-          <t>BEARINGS</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="E558" s="2" t="inlineStr">
@@ -21113,7 +21113,7 @@
       </c>
       <c r="D559" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E559" s="4" t="inlineStr">
@@ -21483,7 +21483,7 @@
       </c>
       <c r="D569" s="4" t="inlineStr">
         <is>
-          <t>HYDRAULIC CYLINDERS</t>
+          <t>HYDRAULIC CYLINDER</t>
         </is>
       </c>
       <c r="E569" s="4" t="inlineStr">
@@ -22149,7 +22149,7 @@
       </c>
       <c r="D587" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E587" s="4" t="inlineStr">
@@ -22334,7 +22334,7 @@
       </c>
       <c r="D592" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS &amp;</t>
+          <t>CYLINDER &amp; BEARING &amp;</t>
         </is>
       </c>
       <c r="E592" s="2" t="inlineStr">
@@ -22519,7 +22519,7 @@
       </c>
       <c r="D597" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E597" s="4" t="inlineStr">
@@ -22556,7 +22556,7 @@
       </c>
       <c r="D598" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E598" s="2" t="inlineStr">
@@ -22593,7 +22593,7 @@
       </c>
       <c r="D599" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E599" s="4" t="inlineStr">
@@ -22630,7 +22630,7 @@
       </c>
       <c r="D600" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E600" s="2" t="inlineStr">
@@ -22963,7 +22963,7 @@
       </c>
       <c r="D609" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E609" s="4" t="inlineStr">
@@ -23000,7 +23000,7 @@
       </c>
       <c r="D610" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E610" s="2" t="inlineStr">
@@ -23037,7 +23037,7 @@
       </c>
       <c r="D611" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E611" s="4" t="inlineStr">
@@ -23074,7 +23074,7 @@
       </c>
       <c r="D612" s="2" t="inlineStr">
         <is>
-          <t>MOTO BEARING-</t>
+          <t>MOTO BEARING</t>
         </is>
       </c>
       <c r="E612" s="2" t="inlineStr">
@@ -23111,7 +23111,7 @@
       </c>
       <c r="D613" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E613" s="4" t="inlineStr">
@@ -23148,7 +23148,7 @@
       </c>
       <c r="D614" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E614" s="2" t="inlineStr">
@@ -23222,7 +23222,7 @@
       </c>
       <c r="D616" s="2" t="inlineStr">
         <is>
-          <t>OPEN GEAR &amp;WIRE ROPE-</t>
+          <t>OPEN GEAR &amp;WIRE ROPE</t>
         </is>
       </c>
       <c r="E616" s="2" t="inlineStr">
@@ -23296,7 +23296,7 @@
       </c>
       <c r="D618" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E618" s="2" t="inlineStr">
@@ -23370,7 +23370,7 @@
       </c>
       <c r="D620" s="2" t="inlineStr">
         <is>
-          <t>OPEN GEAR&amp;WIRE ROPES-</t>
+          <t>OPEN GEAR&amp;WIRE ROPE</t>
         </is>
       </c>
       <c r="E620" s="2" t="inlineStr">
@@ -23407,7 +23407,7 @@
       </c>
       <c r="D621" s="4" t="inlineStr">
         <is>
-          <t>BEARINGS &amp; CHAIN</t>
+          <t>BEARING &amp; CHAIN</t>
         </is>
       </c>
       <c r="E621" s="4" t="inlineStr">
@@ -23481,7 +23481,7 @@
       </c>
       <c r="D623" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOXES FOR WINCH-</t>
+          <t>GEAR BOXES FOR WINCH</t>
         </is>
       </c>
       <c r="E623" s="4" t="inlineStr">
@@ -23629,7 +23629,7 @@
       </c>
       <c r="D627" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOXES FOR WINCH-</t>
+          <t>GEAR BOXES FOR WINCH</t>
         </is>
       </c>
       <c r="E627" s="4" t="inlineStr">
@@ -23740,7 +23740,7 @@
       </c>
       <c r="D630" s="2" t="inlineStr">
         <is>
-          <t>ENGINE GEAR BOX -</t>
+          <t>ENGINE GEAR BOX</t>
         </is>
       </c>
       <c r="E630" s="2" t="inlineStr">
@@ -23851,7 +23851,7 @@
       </c>
       <c r="D633" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOX-</t>
+          <t>GEAR BOX</t>
         </is>
       </c>
       <c r="E633" s="4" t="inlineStr">
@@ -23962,7 +23962,7 @@
       </c>
       <c r="D636" s="2" t="inlineStr">
         <is>
-          <t>WIRE ROPES-</t>
+          <t>WIRE ROPE</t>
         </is>
       </c>
       <c r="E636" s="2" t="inlineStr">
@@ -23999,7 +23999,7 @@
       </c>
       <c r="D637" s="4" t="inlineStr">
         <is>
-          <t>PULLEY &amp; BLOCK-</t>
+          <t>PULLEY &amp; BLOCK</t>
         </is>
       </c>
       <c r="E637" s="4" t="inlineStr">
@@ -24036,7 +24036,7 @@
       </c>
       <c r="D638" s="2" t="inlineStr">
         <is>
-          <t>GEAR-</t>
+          <t>GEAR</t>
         </is>
       </c>
       <c r="E638" s="2" t="inlineStr">
@@ -24073,7 +24073,7 @@
       </c>
       <c r="D639" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E639" s="4" t="inlineStr">
@@ -24147,7 +24147,7 @@
       </c>
       <c r="D641" s="4" t="inlineStr">
         <is>
-          <t>WIRE ROPES-</t>
+          <t>WIRE ROPE</t>
         </is>
       </c>
       <c r="E641" s="4" t="inlineStr">
@@ -24184,7 +24184,7 @@
       </c>
       <c r="D642" s="2" t="inlineStr">
         <is>
-          <t>BEARINGS</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="E642" s="2" t="inlineStr">
@@ -24295,7 +24295,7 @@
       </c>
       <c r="D645" s="4" t="inlineStr">
         <is>
-          <t>WIRE ROPES-</t>
+          <t>WIRE ROPE</t>
         </is>
       </c>
       <c r="E645" s="4" t="inlineStr">
@@ -24369,7 +24369,7 @@
       </c>
       <c r="D647" s="4" t="inlineStr">
         <is>
-          <t>BEARINGS</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="E647" s="4" t="inlineStr">
@@ -24480,7 +24480,7 @@
       </c>
       <c r="D650" s="2" t="inlineStr">
         <is>
-          <t>WIRE ROPES-</t>
+          <t>WIRE ROPE</t>
         </is>
       </c>
       <c r="E650" s="2" t="inlineStr">
@@ -24776,7 +24776,7 @@
       </c>
       <c r="D658" s="2" t="inlineStr">
         <is>
-          <t>BEARINGS AND OIL FILLING</t>
+          <t>BEARING AND OIL FILLING</t>
         </is>
       </c>
       <c r="E658" s="2" t="inlineStr">
@@ -24887,7 +24887,7 @@
       </c>
       <c r="D661" s="4" t="inlineStr">
         <is>
-          <t>ENCLOSED GEARS AND BEARINGS</t>
+          <t>ENCLOSED GEAR AND BEARING</t>
         </is>
       </c>
       <c r="E661" s="4" t="inlineStr">
@@ -24924,7 +24924,7 @@
       </c>
       <c r="D662" s="2" t="inlineStr">
         <is>
-          <t>ENCLOSED GEARS AND BEARINGS</t>
+          <t>ENCLOSED GEAR AND BEARING</t>
         </is>
       </c>
       <c r="E662" s="2" t="inlineStr">
@@ -25072,7 +25072,7 @@
       </c>
       <c r="D666" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E666" s="2" t="inlineStr">
@@ -25109,7 +25109,7 @@
       </c>
       <c r="D667" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E667" s="4" t="inlineStr">
@@ -25146,7 +25146,7 @@
       </c>
       <c r="D668" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E668" s="2" t="inlineStr">
@@ -25183,7 +25183,7 @@
       </c>
       <c r="D669" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E669" s="4" t="inlineStr">
@@ -25405,7 +25405,7 @@
       </c>
       <c r="D675" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E675" s="4" t="inlineStr">
@@ -26182,7 +26182,7 @@
       </c>
       <c r="D696" s="2" t="inlineStr">
         <is>
-          <t>GREASE NIPPLE POINTS</t>
+          <t>GREASE NIPPLE POINT</t>
         </is>
       </c>
       <c r="E696" s="2" t="inlineStr">
@@ -26367,7 +26367,7 @@
       </c>
       <c r="D701" s="4" t="inlineStr">
         <is>
-          <t>BLOCKS/TOLLEYS GEAR AND ELECTIRC HOIST</t>
+          <t>BLOCK/TOLLEYS GEAR AND ELECTIRC HOIST</t>
         </is>
       </c>
       <c r="E701" s="4" t="inlineStr">
@@ -26626,7 +26626,7 @@
       </c>
       <c r="D708" s="2" t="inlineStr">
         <is>
-          <t>GREASE FOR -RUDDER TRUNK FILLING -SHAFT SEALS -ROLLER/SLIDE BEARING -RAM BOLTS</t>
+          <t>GREASE FOR -RUDDER TRUNK FILLING -SHAFT SEAL -ROLLER/SLIDE BEARING -RAM BOLT</t>
         </is>
       </c>
       <c r="E708" s="2" t="inlineStr">
@@ -26811,7 +26811,7 @@
       </c>
       <c r="D713" s="4" t="inlineStr">
         <is>
-          <t>GREASE NIPPLE</t>
+          <t>GREASE POINT</t>
         </is>
       </c>
       <c r="E713" s="4" t="inlineStr">
@@ -26996,7 +26996,7 @@
       </c>
       <c r="D718" s="2" t="inlineStr">
         <is>
-          <t>GREASE NIPPLE POINTS</t>
+          <t>GREASE NIPPLE POINT</t>
         </is>
       </c>
       <c r="E718" s="2" t="inlineStr">
@@ -27884,7 +27884,7 @@
       </c>
       <c r="D742" s="2" t="inlineStr">
         <is>
-          <t>GEAR ANF BEARINGS</t>
+          <t>GEAR ANF BEARING</t>
         </is>
       </c>
       <c r="E742" s="2" t="inlineStr">
@@ -28069,7 +28069,7 @@
       </c>
       <c r="D747" s="4" t="inlineStr">
         <is>
-          <t>B.CYLINDERS</t>
+          <t>B.CYLINDER</t>
         </is>
       </c>
       <c r="E747" s="4" t="inlineStr">
@@ -28106,7 +28106,7 @@
       </c>
       <c r="D748" s="2" t="inlineStr">
         <is>
-          <t>C.TURNING GEAR ENCLOSED GEARS</t>
+          <t>C.TURNING GEAR ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E748" s="2" t="inlineStr">
@@ -28254,7 +28254,7 @@
       </c>
       <c r="D752" s="2" t="inlineStr">
         <is>
-          <t>C.ALTERNATOR BEARINGS</t>
+          <t>C.ALTERNATOR BEARING</t>
         </is>
       </c>
       <c r="E752" s="2" t="inlineStr">
@@ -28328,7 +28328,7 @@
       </c>
       <c r="D754" s="2" t="inlineStr">
         <is>
-          <t>ENCLOSED BEARINGS</t>
+          <t>ENCLOSED BEARING</t>
         </is>
       </c>
       <c r="E754" s="2" t="inlineStr">
@@ -28365,7 +28365,7 @@
       </c>
       <c r="D755" s="4" t="inlineStr">
         <is>
-          <t>ENCLOSED BEARINGS</t>
+          <t>ENCLOSED BEARING</t>
         </is>
       </c>
       <c r="E755" s="4" t="inlineStr">
@@ -28439,7 +28439,7 @@
       </c>
       <c r="D757" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E757" s="4" t="inlineStr">
@@ -28476,7 +28476,7 @@
       </c>
       <c r="D758" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E758" s="2" t="inlineStr">
@@ -28883,7 +28883,7 @@
       </c>
       <c r="D769" s="4" t="inlineStr">
         <is>
-          <t>B.ENCLOSED GEARS</t>
+          <t>B.ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E769" s="4" t="inlineStr">
@@ -28920,7 +28920,7 @@
       </c>
       <c r="D770" s="2" t="inlineStr">
         <is>
-          <t>C.OPEN GEARS</t>
+          <t>C.OPEN GEAR</t>
         </is>
       </c>
       <c r="E770" s="2" t="inlineStr">
@@ -28957,7 +28957,7 @@
       </c>
       <c r="D771" s="4" t="inlineStr">
         <is>
-          <t>D.GREASE NIPPLES</t>
+          <t>D.GREASE NIPPLE</t>
         </is>
       </c>
       <c r="E771" s="4" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="D773" s="4" t="inlineStr">
         <is>
-          <t>B.LUBRICANT GREASE FOR NIPPLES</t>
+          <t>B.LUBRICANT GREASE FOR NIPPLE</t>
         </is>
       </c>
       <c r="E773" s="4" t="inlineStr">
@@ -29993,7 +29993,7 @@
       </c>
       <c r="D799" s="4" t="inlineStr">
         <is>
-          <t>C.BEARINGS AND LUBRICANT NIPPLES</t>
+          <t>C.BEARING AND LUBRICANT NIPPLE</t>
         </is>
       </c>
       <c r="E799" s="4" t="inlineStr">
@@ -30104,7 +30104,7 @@
       </c>
       <c r="D802" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E802" s="2" t="inlineStr">
@@ -30141,7 +30141,7 @@
       </c>
       <c r="D803" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E803" s="4" t="inlineStr">
@@ -30585,7 +30585,7 @@
       </c>
       <c r="D815" s="4" t="inlineStr">
         <is>
-          <t>STERN SEALS</t>
+          <t>STERN SEAL</t>
         </is>
       </c>
       <c r="E815" s="4" t="inlineStr">
@@ -30881,7 +30881,7 @@
       </c>
       <c r="D823" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E823" s="4" t="inlineStr">
@@ -30918,7 +30918,7 @@
       </c>
       <c r="D824" s="2" t="inlineStr">
         <is>
-          <t>WEARING PARTS SUCH AS:VALVES, SYLINDER LINERS AND CRANK BEARINGS, PISTON GUDGEON PINS ETC.</t>
+          <t>WEARING PARTS SUCH AS:VALVE, SYLINDER LINERS AND CRANK BEARING, PISTON GUDGEON PINS ETC.</t>
         </is>
       </c>
       <c r="E824" s="2" t="inlineStr">
@@ -32065,7 +32065,7 @@
       </c>
       <c r="D855" s="4" t="inlineStr">
         <is>
-          <t>GEAR BOXES FOR WINCH-</t>
+          <t>GEAR BOXES FOR WINCH</t>
         </is>
       </c>
       <c r="E855" s="4" t="inlineStr">
@@ -33064,7 +33064,7 @@
       </c>
       <c r="D882" s="2" t="inlineStr">
         <is>
-          <t>USED FOR NIPPLES &amp; SHAFT</t>
+          <t>USED FOR NIPPLE &amp; SHAFT</t>
         </is>
       </c>
       <c r="E882" s="2" t="inlineStr">
@@ -33582,7 +33582,7 @@
       </c>
       <c r="D896" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E896" s="2" t="inlineStr">
@@ -33989,7 +33989,7 @@
       </c>
       <c r="D907" s="4" t="inlineStr">
         <is>
-          <t>GENERAL GREASE UP POINTS</t>
+          <t>GENERAL GREASE UP POINT</t>
         </is>
       </c>
       <c r="E907" s="4" t="inlineStr">
@@ -34470,7 +34470,7 @@
       </c>
       <c r="D920" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E920" s="2" t="inlineStr">
@@ -34507,7 +34507,7 @@
       </c>
       <c r="D921" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E921" s="4" t="inlineStr">
@@ -35728,7 +35728,7 @@
       </c>
       <c r="D954" s="2" t="inlineStr">
         <is>
-          <t>BEARINGS</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="E954" s="2" t="inlineStr">
@@ -35765,7 +35765,7 @@
       </c>
       <c r="D955" s="4" t="inlineStr">
         <is>
-          <t>OILER</t>
+          <t>OIL POINT</t>
         </is>
       </c>
       <c r="E955" s="4" t="inlineStr">
@@ -35950,7 +35950,7 @@
       </c>
       <c r="D960" s="2" t="inlineStr">
         <is>
-          <t>BEARINGS</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="E960" s="2" t="inlineStr">
@@ -35987,7 +35987,7 @@
       </c>
       <c r="D961" s="4" t="inlineStr">
         <is>
-          <t>OILER</t>
+          <t>OIL POINT</t>
         </is>
       </c>
       <c r="E961" s="4" t="inlineStr">
@@ -36764,7 +36764,7 @@
       </c>
       <c r="D982" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E982" s="2" t="inlineStr">
@@ -37060,7 +37060,7 @@
       </c>
       <c r="D990" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E990" s="2" t="inlineStr">
@@ -37208,7 +37208,7 @@
       </c>
       <c r="D994" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E994" s="2" t="inlineStr">
@@ -37319,7 +37319,7 @@
       </c>
       <c r="D997" s="4" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E997" s="4" t="inlineStr">
@@ -37356,7 +37356,7 @@
       </c>
       <c r="D998" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E998" s="2" t="inlineStr">
@@ -37393,7 +37393,7 @@
       </c>
       <c r="D999" s="4" t="inlineStr">
         <is>
-          <t>BEARINGS</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="E999" s="4" t="inlineStr">
@@ -37467,7 +37467,7 @@
       </c>
       <c r="D1001" s="4" t="inlineStr">
         <is>
-          <t>BEARINGS</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="E1001" s="4" t="inlineStr">
@@ -37578,7 +37578,7 @@
       </c>
       <c r="D1004" s="2" t="inlineStr">
         <is>
-          <t>BEARINGS</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="E1004" s="2" t="inlineStr">
@@ -38651,7 +38651,7 @@
       </c>
       <c r="D1033" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM OIL</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="E1033" s="4" t="inlineStr">
@@ -40242,7 +40242,7 @@
       </c>
       <c r="D1076" s="2" t="inlineStr">
         <is>
-          <t>CYLINDERS &amp; BEARINGS</t>
+          <t>CYLINDER &amp; BEARING</t>
         </is>
       </c>
       <c r="E1076" s="2" t="inlineStr">

</xml_diff>

<commit_message>
data: update 2026-04-27 12:04
</commit_message>
<xml_diff>
--- a/output/nb_master.xlsx
+++ b/output/nb_master.xlsx
@@ -10788,7 +10788,7 @@
       </c>
       <c r="B280" s="2" t="inlineStr">
         <is>
-          <t>WARTSILA &amp;</t>
+          <t>WARTSILA</t>
         </is>
       </c>
       <c r="C280" s="2" t="inlineStr">
@@ -10825,7 +10825,7 @@
       </c>
       <c r="B281" s="4" t="inlineStr">
         <is>
-          <t>WARTSILA &amp;</t>
+          <t>WARTSILA</t>
         </is>
       </c>
       <c r="C281" s="4" t="inlineStr">
@@ -10862,7 +10862,7 @@
       </c>
       <c r="B282" s="2" t="inlineStr">
         <is>
-          <t>WARTSILA &amp;</t>
+          <t>WARTSILA</t>
         </is>
       </c>
       <c r="C282" s="2" t="inlineStr">
@@ -10899,7 +10899,7 @@
       </c>
       <c r="B283" s="4" t="inlineStr">
         <is>
-          <t>WARTSILA &amp;</t>
+          <t>WARTSILA</t>
         </is>
       </c>
       <c r="C283" s="4" t="inlineStr">
@@ -10936,7 +10936,7 @@
       </c>
       <c r="B284" s="2" t="inlineStr">
         <is>
-          <t>WARTSILA &amp;</t>
+          <t>WARTSILA</t>
         </is>
       </c>
       <c r="C284" s="2" t="inlineStr">
@@ -10973,7 +10973,7 @@
       </c>
       <c r="B285" s="4" t="inlineStr">
         <is>
-          <t>WARTSILA &amp;</t>
+          <t>WARTSILA</t>
         </is>
       </c>
       <c r="C285" s="4" t="inlineStr">
@@ -11010,7 +11010,7 @@
       </c>
       <c r="B286" s="2" t="inlineStr">
         <is>
-          <t>WARTSILA &amp;</t>
+          <t>WARTSILA</t>
         </is>
       </c>
       <c r="C286" s="2" t="inlineStr">

</xml_diff>

<commit_message>
data: update 2026-04-27 15:21
</commit_message>
<xml_diff>
--- a/output/nb_master.xlsx
+++ b/output/nb_master.xlsx
@@ -861,7 +861,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -937,7 +937,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2124,7 +2124,7 @@
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
@@ -2161,7 +2161,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -3840,7 +3840,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -5067,7 +5067,7 @@
       </c>
       <c r="D125" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E125" s="4" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
@@ -6251,7 +6251,7 @@
       </c>
       <c r="D157" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E157" s="4" t="inlineStr">
@@ -9063,7 +9063,7 @@
       </c>
       <c r="D233" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E233" s="4" t="inlineStr">
@@ -9100,7 +9100,7 @@
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E234" s="2" t="inlineStr">
@@ -9137,7 +9137,7 @@
       </c>
       <c r="D235" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E235" s="4" t="inlineStr">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E236" s="2" t="inlineStr">
@@ -9211,7 +9211,7 @@
       </c>
       <c r="D237" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E237" s="4" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="D238" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E238" s="2" t="inlineStr">
@@ -12097,7 +12097,7 @@
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E315" s="4" t="inlineStr">
@@ -12134,7 +12134,7 @@
       </c>
       <c r="D316" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E316" s="2" t="inlineStr">
@@ -12282,7 +12282,7 @@
       </c>
       <c r="D320" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E320" s="2" t="inlineStr">
@@ -12430,7 +12430,7 @@
       </c>
       <c r="D324" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E324" s="2" t="inlineStr">
@@ -12467,7 +12467,7 @@
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E325" s="4" t="inlineStr">
@@ -12504,7 +12504,7 @@
       </c>
       <c r="D326" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E326" s="2" t="inlineStr">
@@ -13651,7 +13651,7 @@
       </c>
       <c r="D357" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E357" s="4" t="inlineStr">
@@ -13688,7 +13688,7 @@
       </c>
       <c r="D358" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E358" s="2" t="inlineStr">
@@ -13725,7 +13725,7 @@
       </c>
       <c r="D359" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E359" s="4" t="inlineStr">
@@ -13762,7 +13762,7 @@
       </c>
       <c r="D360" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E360" s="2" t="inlineStr">
@@ -16981,7 +16981,7 @@
       </c>
       <c r="D447" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E447" s="4" t="inlineStr">
@@ -17018,7 +17018,7 @@
       </c>
       <c r="D448" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E448" s="2" t="inlineStr">
@@ -17055,7 +17055,7 @@
       </c>
       <c r="D449" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E449" s="4" t="inlineStr">
@@ -17092,7 +17092,7 @@
       </c>
       <c r="D450" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E450" s="2" t="inlineStr">
@@ -17425,7 +17425,7 @@
       </c>
       <c r="D459" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E459" s="4" t="inlineStr">
@@ -17462,7 +17462,7 @@
       </c>
       <c r="D460" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E460" s="2" t="inlineStr">
@@ -19497,7 +19497,7 @@
       </c>
       <c r="D515" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E515" s="4" t="inlineStr">
@@ -19534,7 +19534,7 @@
       </c>
       <c r="D516" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E516" s="2" t="inlineStr">
@@ -19571,7 +19571,7 @@
       </c>
       <c r="D517" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E517" s="4" t="inlineStr">
@@ -19608,7 +19608,7 @@
       </c>
       <c r="D518" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E518" s="2" t="inlineStr">
@@ -22864,7 +22864,7 @@
       </c>
       <c r="D606" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E606" s="2" t="inlineStr">
@@ -22901,7 +22901,7 @@
       </c>
       <c r="D607" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E607" s="4" t="inlineStr">
@@ -24529,7 +24529,7 @@
       </c>
       <c r="D651" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E651" s="4" t="inlineStr">
@@ -24566,7 +24566,7 @@
       </c>
       <c r="D652" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E652" s="2" t="inlineStr">
@@ -25306,7 +25306,7 @@
       </c>
       <c r="D672" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E672" s="2" t="inlineStr">
@@ -28895,7 +28895,7 @@
       </c>
       <c r="D769" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E769" s="4" t="inlineStr">
@@ -28932,7 +28932,7 @@
       </c>
       <c r="D770" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E770" s="2" t="inlineStr">
@@ -31744,7 +31744,7 @@
       </c>
       <c r="D846" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E846" s="2" t="inlineStr">
@@ -31781,7 +31781,7 @@
       </c>
       <c r="D847" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E847" s="4" t="inlineStr">
@@ -34667,7 +34667,7 @@
       </c>
       <c r="D925" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E925" s="4" t="inlineStr">
@@ -36147,7 +36147,7 @@
       </c>
       <c r="D965" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E965" s="4" t="inlineStr">
@@ -36184,7 +36184,7 @@
       </c>
       <c r="D966" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E966" s="2" t="inlineStr">
@@ -38219,7 +38219,7 @@
       </c>
       <c r="D1021" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E1021" s="4" t="inlineStr">
@@ -38256,7 +38256,7 @@
       </c>
       <c r="D1022" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E1022" s="2" t="inlineStr">
@@ -38293,7 +38293,7 @@
       </c>
       <c r="D1023" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E1023" s="4" t="inlineStr">
@@ -38589,7 +38589,7 @@
       </c>
       <c r="D1031" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E1031" s="4" t="inlineStr">
@@ -38626,7 +38626,7 @@
       </c>
       <c r="D1032" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E1032" s="2" t="inlineStr">
@@ -38663,7 +38663,7 @@
       </c>
       <c r="D1033" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>CYLINDERS &amp; BEARINGS</t>
         </is>
       </c>
       <c r="E1033" s="4" t="inlineStr">
@@ -39438,11 +39438,7 @@
           <t>SRP 4040 LSU FP</t>
         </is>
       </c>
-      <c r="D1054" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D1054" s="2" t="inlineStr"/>
       <c r="E1054" s="2" t="inlineStr">
         <is>
           <t>SHIPOWNER AFTER DELIVERY.</t>
@@ -40022,12 +40018,12 @@
       </c>
       <c r="B1070" s="2" t="inlineStr">
         <is>
-          <t>HYUNDAI-MAN B&amp;W</t>
+          <t>HYUNDAI-WINGD</t>
         </is>
       </c>
       <c r="C1070" s="2" t="inlineStr">
         <is>
-          <t>6G60ME-C9.5-GIE-HPSCR</t>
+          <t>5X72DF-2.2</t>
         </is>
       </c>
       <c r="D1070" s="2" t="inlineStr">
@@ -40037,7 +40033,7 @@
       </c>
       <c r="E1070" s="2" t="inlineStr">
         <is>
-          <t>ATLANTA MARINE D 3005</t>
+          <t>ATLANTA MARINE D 3005 A1</t>
         </is>
       </c>
       <c r="F1070" s="3" t="inlineStr">
@@ -40047,7 +40043,7 @@
       </c>
       <c r="G1070" s="2" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
@@ -40059,12 +40055,12 @@
       </c>
       <c r="B1071" s="4" t="inlineStr">
         <is>
-          <t>HYUNDAI-MAN B&amp;W</t>
+          <t>HYUNDAI-WINGD</t>
         </is>
       </c>
       <c r="C1071" s="4" t="inlineStr">
         <is>
-          <t>6G60ME-C9.5-GIE-HPSCR</t>
+          <t>5X72DF-2.2</t>
         </is>
       </c>
       <c r="D1071" s="4" t="inlineStr">
@@ -40084,7 +40080,7 @@
       </c>
       <c r="G1071" s="4" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
@@ -40096,22 +40092,22 @@
       </c>
       <c r="B1072" s="2" t="inlineStr">
         <is>
-          <t>HYUNDAI-MAN B&amp;W</t>
+          <t>HYUNDAI-WINGD</t>
         </is>
       </c>
       <c r="C1072" s="2" t="inlineStr">
         <is>
-          <t>6G60ME-C9.5-GIE-HPSCR</t>
+          <t>5X72DF-2.2</t>
         </is>
       </c>
       <c r="D1072" s="2" t="inlineStr">
         <is>
-          <t>FUEL VALVE TEST DEVICE OIL TANK</t>
+          <t>ENCLOSED GEAR</t>
         </is>
       </c>
       <c r="E1072" s="2" t="inlineStr">
         <is>
-          <t>VISGA 15</t>
+          <t>EPONA Z 220</t>
         </is>
       </c>
       <c r="F1072" s="3" t="inlineStr">
@@ -40121,7 +40117,7 @@
       </c>
       <c r="G1072" s="2" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
@@ -40133,22 +40129,22 @@
       </c>
       <c r="B1073" s="4" t="inlineStr">
         <is>
-          <t>HYUNDAI-MAN B&amp;W</t>
+          <t>HYUNDAI-WINGD</t>
         </is>
       </c>
       <c r="C1073" s="4" t="inlineStr">
         <is>
-          <t>6G60ME-C9.5-GIE-HPSCR</t>
+          <t>5X72DF-2.2</t>
         </is>
       </c>
       <c r="D1073" s="4" t="inlineStr">
         <is>
-          <t>PNEUMATIC HYD. H.P. PUMP</t>
+          <t>TURNING GEAR GREASE</t>
         </is>
       </c>
       <c r="E1073" s="4" t="inlineStr">
         <is>
-          <t>VISGA 15</t>
+          <t>CERAN XM 220</t>
         </is>
       </c>
       <c r="F1073" s="5" t="inlineStr">
@@ -40158,7 +40154,7 @@
       </c>
       <c r="G1073" s="4" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
@@ -40170,22 +40166,22 @@
       </c>
       <c r="B1074" s="2" t="inlineStr">
         <is>
-          <t>HYUNDAI-MAN B&amp;W</t>
+          <t>HYUNDAI-WINGD</t>
         </is>
       </c>
       <c r="C1074" s="2" t="inlineStr">
         <is>
-          <t>6G60ME-C9.5-GIE-HPSCR</t>
+          <t>5X72DF-2.2</t>
         </is>
       </c>
       <c r="D1074" s="2" t="inlineStr">
         <is>
-          <t>TURNING ENCLOSED GEAR</t>
+          <t>AUX. BLOWER MOTOR BEARING</t>
         </is>
       </c>
       <c r="E1074" s="2" t="inlineStr">
         <is>
-          <t>EPONA Z 320</t>
+          <t>MULTIS EP 2</t>
         </is>
       </c>
       <c r="F1074" s="3" t="inlineStr">
@@ -40195,7 +40191,7 @@
       </c>
       <c r="G1074" s="2" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
@@ -40207,22 +40203,22 @@
       </c>
       <c r="B1075" s="4" t="inlineStr">
         <is>
-          <t>HYUNDAI-MAN B&amp;W</t>
+          <t>HYUNDAI-WINGD</t>
         </is>
       </c>
       <c r="C1075" s="4" t="inlineStr">
         <is>
-          <t>6G60ME-C9.5-GIE-HPSCR</t>
+          <t>5X72DF-2.2</t>
         </is>
       </c>
       <c r="D1075" s="4" t="inlineStr">
         <is>
-          <t>OPEN GEAR</t>
+          <t>FUEL VALVE TEST DEVICE</t>
         </is>
       </c>
       <c r="E1075" s="4" t="inlineStr">
         <is>
-          <t>CERAN XM 220</t>
+          <t>SHELL CALIBRATION FLUID S.9365</t>
         </is>
       </c>
       <c r="F1075" s="5" t="inlineStr">
@@ -40232,7 +40228,7 @@
       </c>
       <c r="G1075" s="4" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
@@ -40244,22 +40240,22 @@
       </c>
       <c r="B1076" s="2" t="inlineStr">
         <is>
-          <t>HYUNDAI-MAN B&amp;W</t>
+          <t>HYUNDAI-WINGD</t>
         </is>
       </c>
       <c r="C1076" s="2" t="inlineStr">
         <is>
-          <t>6G60ME-C9.5-GIE-HPSCR</t>
+          <t>5X72DF-2.2</t>
         </is>
       </c>
       <c r="D1076" s="2" t="inlineStr">
         <is>
-          <t>AUX. BLOWER GREASE POINT</t>
+          <t>AIR DRIVEN HIGH PRESS. PUMP</t>
         </is>
       </c>
       <c r="E1076" s="2" t="inlineStr">
         <is>
-          <t>MULTIS MS 2</t>
+          <t>VISGA 32</t>
         </is>
       </c>
       <c r="F1076" s="3" t="inlineStr">
@@ -40269,7 +40265,7 @@
       </c>
       <c r="G1076" s="2" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
@@ -40281,22 +40277,22 @@
       </c>
       <c r="B1077" s="4" t="inlineStr">
         <is>
-          <t>HYUNDAI-MAN B&amp;W</t>
+          <t>HYUNDAI-WINGD</t>
         </is>
       </c>
       <c r="C1077" s="4" t="inlineStr">
         <is>
-          <t>6G60ME-C9.5-GIE-HPSCR</t>
+          <t>5X72DF-2.2</t>
         </is>
       </c>
       <c r="D1077" s="4" t="inlineStr">
         <is>
-          <t>GAS VALVE TEST DEVICE</t>
+          <t>WTS SEPARATOR</t>
         </is>
       </c>
       <c r="E1077" s="4" t="inlineStr">
         <is>
-          <t>VISGA 32</t>
+          <t>EPONA Z 150</t>
         </is>
       </c>
       <c r="F1077" s="5" t="inlineStr">
@@ -40306,7 +40302,7 @@
       </c>
       <c r="G1077" s="4" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
@@ -40318,22 +40314,22 @@
       </c>
       <c r="B1078" s="2" t="inlineStr">
         <is>
-          <t>HYUNDAI-MAN B&amp;W</t>
+          <t>HYUNDAI-WINGD</t>
         </is>
       </c>
       <c r="C1078" s="2" t="inlineStr">
         <is>
-          <t>6G60ME-C9.5-GIE-HPSCR</t>
+          <t>5X72DF-2.2</t>
         </is>
       </c>
       <c r="D1078" s="2" t="inlineStr">
         <is>
-          <t>M/E HYD. TOP BRACING OIL CHAMBER</t>
+          <t>EGC BUTTERFLY VALVE</t>
         </is>
       </c>
       <c r="E1078" s="2" t="inlineStr">
         <is>
-          <t>VISGA 32</t>
+          <t>MULTIS EP 2</t>
         </is>
       </c>
       <c r="F1078" s="3" t="inlineStr">
@@ -40343,34 +40339,34 @@
       </c>
       <c r="G1078" s="2" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
     <row r="1079">
       <c r="A1079" s="4" t="inlineStr">
         <is>
-          <t>DIESEL GENERATOR ENGINE</t>
+          <t>MAIN ENGINE</t>
         </is>
       </c>
       <c r="B1079" s="4" t="inlineStr">
         <is>
-          <t>HYUNDAI-HIMSEN</t>
+          <t>HYUNDAI-WINGD</t>
         </is>
       </c>
       <c r="C1079" s="4" t="inlineStr">
         <is>
-          <t>8H25/33</t>
+          <t>5X72DF-2.2</t>
         </is>
       </c>
       <c r="D1079" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM</t>
+          <t>H-MOMENT COMPENSATOR</t>
         </is>
       </c>
       <c r="E1079" s="4" t="inlineStr">
         <is>
-          <t>AURELIA TI 4020</t>
+          <t>EPONA Z 150</t>
         </is>
       </c>
       <c r="F1079" s="5" t="inlineStr">
@@ -40380,34 +40376,34 @@
       </c>
       <c r="G1079" s="4" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
     <row r="1080">
       <c r="A1080" s="2" t="inlineStr">
         <is>
-          <t>DIESEL GENERATOR ENGINE</t>
+          <t>INCINERATOR</t>
         </is>
       </c>
       <c r="B1080" s="2" t="inlineStr">
         <is>
-          <t>HYUNDAI-HIMSEN</t>
+          <t>HMMCO</t>
         </is>
       </c>
       <c r="C1080" s="2" t="inlineStr">
         <is>
-          <t>8H25/33</t>
+          <t>MAXI T150SL WS</t>
         </is>
       </c>
       <c r="D1080" s="2" t="inlineStr">
         <is>
-          <t>GOVERNOR</t>
+          <t>GEAR BOX FOR W.O.DOSING PUMP</t>
         </is>
       </c>
       <c r="E1080" s="2" t="inlineStr">
         <is>
-          <t>AURELIA TI 4020</t>
+          <t>EPONA Z 220</t>
         </is>
       </c>
       <c r="F1080" s="3" t="inlineStr">
@@ -40417,34 +40413,34 @@
       </c>
       <c r="G1080" s="2" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
     <row r="1081">
       <c r="A1081" s="4" t="inlineStr">
         <is>
-          <t>G/E L.P. SCR</t>
+          <t>INCINERATOR</t>
         </is>
       </c>
       <c r="B1081" s="4" t="inlineStr">
         <is>
-          <t>HYUNDAI EMD</t>
+          <t>HMMCO</t>
         </is>
       </c>
       <c r="C1081" s="4" t="inlineStr">
         <is>
-          <t>BY-PASS VALVE</t>
+          <t>MAXI T150SL WS</t>
         </is>
       </c>
       <c r="D1081" s="4" t="inlineStr">
         <is>
-          <t>SHAFT BEARING GEAR BOX</t>
+          <t>MILL PUMP SEAL BOX</t>
         </is>
       </c>
       <c r="E1081" s="4" t="inlineStr">
         <is>
-          <t>R100 TECTYL G182 TECTYL G182</t>
+          <t>VISGA 46</t>
         </is>
       </c>
       <c r="F1081" s="5" t="inlineStr">
@@ -40454,34 +40450,34 @@
       </c>
       <c r="G1081" s="4" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
     <row r="1082">
       <c r="A1082" s="2" t="inlineStr">
         <is>
-          <t>AUXILIARY BOILER</t>
+          <t>ELECTRIC BALANCER</t>
         </is>
       </c>
       <c r="B1082" s="2" t="inlineStr">
         <is>
-          <t>ALFA LAVAL</t>
+          <t>COMPENSATOR</t>
         </is>
       </c>
       <c r="C1082" s="2" t="inlineStr">
         <is>
-          <t>AUXILIARY BOILER</t>
+          <t>(EMC-400VD 2SETS)</t>
         </is>
       </c>
       <c r="D1082" s="2" t="inlineStr">
         <is>
-          <t>SAFETY VALVE- LIFTING FORK, LEVER REMOTE PULL FOR SAFETY VALVE -WIRE, SHACKLE, PULLY REMOTE PULL FOR LEVEL GAUGE -WIRE, SHACKLE, PULLY FEED WATER CONTROL VALVE - SPINDLE, STUFFING BOX PACKING FD FANS- BEARING, GREASE NIPPLE FEED WATER CONTROL VALVE- GEAR ACTUATOR</t>
+          <t>BEARING, GEAR</t>
         </is>
       </c>
       <c r="E1082" s="2" t="inlineStr">
         <is>
-          <t>CERAN XM 220 CERAN AD PLUS CERAN AD PLUS CERAN XM 220 CERAN XM 220 CERAN XM 220</t>
+          <t>EPONA Z 100</t>
         </is>
       </c>
       <c r="F1082" s="3" t="inlineStr">
@@ -40491,34 +40487,34 @@
       </c>
       <c r="G1082" s="2" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
     <row r="1083">
       <c r="A1083" s="4" t="inlineStr">
         <is>
-          <t>PISTON TYPE AIR COMPRESSOR</t>
+          <t>STERN TUBE SYSTEM</t>
         </is>
       </c>
       <c r="B1083" s="4" t="inlineStr">
         <is>
-          <t>DONGHWA PNEUTEC</t>
+          <t>KEMEL</t>
         </is>
       </c>
       <c r="C1083" s="4" t="inlineStr">
         <is>
-          <t>MAIN AIR COMPRESSOR</t>
+          <t>AFT(AX-670), FWD(AX-670)</t>
         </is>
       </c>
       <c r="D1083" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>FWD/AFT SEAL CHAMBER</t>
         </is>
       </c>
       <c r="E1083" s="4" t="inlineStr">
         <is>
-          <t>DACNIS 100</t>
+          <t>ATLANTA MARINE D 3005</t>
         </is>
       </c>
       <c r="F1083" s="5" t="inlineStr">
@@ -40528,34 +40524,34 @@
       </c>
       <c r="G1083" s="4" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
     <row r="1084">
       <c r="A1084" s="2" t="inlineStr">
         <is>
-          <t>PISTON TYPE AIR COMPRESSOR</t>
+          <t>STERN TUBE SYSTEM</t>
         </is>
       </c>
       <c r="B1084" s="2" t="inlineStr">
         <is>
-          <t>DONGHWA PNEUTEC</t>
+          <t>KEMEL</t>
         </is>
       </c>
       <c r="C1084" s="2" t="inlineStr">
         <is>
-          <t>MAIN AIR COMPRESSOR</t>
+          <t>AFT(AX-670), FWD(AX-670)</t>
         </is>
       </c>
       <c r="D1084" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>S/T INSIDE</t>
         </is>
       </c>
       <c r="E1084" s="2" t="inlineStr">
         <is>
-          <t>MULTIS COMPLEX S2A</t>
+          <t>ATLANTA MARINE D 3005</t>
         </is>
       </c>
       <c r="F1084" s="3" t="inlineStr">
@@ -40565,34 +40561,34 @@
       </c>
       <c r="G1084" s="2" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
     <row r="1085">
       <c r="A1085" s="4" t="inlineStr">
         <is>
-          <t>SCREW TYPE AIR COMPRESSOR</t>
+          <t>STERN TUBE SYSTEM</t>
         </is>
       </c>
       <c r="B1085" s="4" t="inlineStr">
         <is>
-          <t>MAEKR : DONGHWA PNEUTEC</t>
+          <t>KEMEL</t>
         </is>
       </c>
       <c r="C1085" s="4" t="inlineStr">
         <is>
-          <t>NEX-45ABS</t>
+          <t>AFT(AX-670), FWD(AX-670)</t>
         </is>
       </c>
       <c r="D1085" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>FWD SEAL TANK</t>
         </is>
       </c>
       <c r="E1085" s="4" t="inlineStr">
         <is>
-          <t>DACNIS 46</t>
+          <t>ATLANTA MARINE D 3005</t>
         </is>
       </c>
       <c r="F1085" s="5" t="inlineStr">
@@ -40602,34 +40598,34 @@
       </c>
       <c r="G1085" s="4" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
     <row r="1086">
       <c r="A1086" s="2" t="inlineStr">
         <is>
-          <t>SCREW TYPE AIR COMPRESSOR</t>
+          <t>STERN TUBE SYSTEM</t>
         </is>
       </c>
       <c r="B1086" s="2" t="inlineStr">
         <is>
-          <t>MAEKR : DONGHWA PNEUTEC</t>
+          <t>KEMEL</t>
         </is>
       </c>
       <c r="C1086" s="2" t="inlineStr">
         <is>
-          <t>NEX-45ABS</t>
+          <t>AFT(AX-670), FWD(AX-670)</t>
         </is>
       </c>
       <c r="D1086" s="2" t="inlineStr">
         <is>
-          <t>CYLINDER &amp; BEARING</t>
+          <t>S/T L.O. TANK</t>
         </is>
       </c>
       <c r="E1086" s="2" t="inlineStr">
         <is>
-          <t>MULTIS COMPLEX S2A</t>
+          <t>ATLANTA MARINE D 3005</t>
         </is>
       </c>
       <c r="F1086" s="3" t="inlineStr">
@@ -40639,34 +40635,34 @@
       </c>
       <c r="G1086" s="2" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
     <row r="1087">
       <c r="A1087" s="4" t="inlineStr">
         <is>
-          <t>CENTRIFUGAL PUMP</t>
+          <t>STERN TUBE SYSTEM</t>
         </is>
       </c>
       <c r="B1087" s="4" t="inlineStr">
         <is>
-          <t>SHINKO IND. LTD.</t>
+          <t>KEMEL</t>
         </is>
       </c>
       <c r="C1087" s="4" t="inlineStr">
         <is>
-          <t>W.SPRAY PUMP (GVD300-3M)</t>
+          <t>AFT(AX-670), FWD(AX-670)</t>
         </is>
       </c>
       <c r="D1087" s="4" t="inlineStr">
         <is>
-          <t>COUPLING SIDE BEARING</t>
+          <t>S/T L.O. SUMP. TK</t>
         </is>
       </c>
       <c r="E1087" s="4" t="inlineStr">
         <is>
-          <t>CERAN XM 220</t>
+          <t>ATLANTA MARINE D 3005</t>
         </is>
       </c>
       <c r="F1087" s="5" t="inlineStr">
@@ -40676,34 +40672,34 @@
       </c>
       <c r="G1087" s="4" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
     <row r="1088">
       <c r="A1088" s="2" t="inlineStr">
         <is>
-          <t>CENTRIFUGAL PUMP</t>
+          <t>STERN TUBE SYSTEM</t>
         </is>
       </c>
       <c r="B1088" s="2" t="inlineStr">
         <is>
-          <t>SHINKO IND. LTD.</t>
+          <t>KEMEL</t>
         </is>
       </c>
       <c r="C1088" s="2" t="inlineStr">
         <is>
-          <t>W.SPRAY PUMP (GVD300-3M)</t>
+          <t>AFT(AX-670), FWD(AX-670)</t>
         </is>
       </c>
       <c r="D1088" s="2" t="inlineStr">
         <is>
-          <t>BEARING HOUSING</t>
+          <t>PIPE LINE</t>
         </is>
       </c>
       <c r="E1088" s="2" t="inlineStr">
         <is>
-          <t>PRESLIA 68</t>
+          <t>ATLANTA MARINE D 3005</t>
         </is>
       </c>
       <c r="F1088" s="3" t="inlineStr">
@@ -40713,34 +40709,34 @@
       </c>
       <c r="G1088" s="2" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
     <row r="1089">
       <c r="A1089" s="4" t="inlineStr">
         <is>
-          <t>CENTRIFUGAL PUMP</t>
+          <t>GREASE PUMP FOR RUDDER CARRIER</t>
         </is>
       </c>
       <c r="B1089" s="4" t="inlineStr">
         <is>
-          <t>SHINKO IND. LTD.</t>
+          <t>3K</t>
         </is>
       </c>
       <c r="C1089" s="4" t="inlineStr">
         <is>
-          <t>W.SPRAY PUMP (GVD300-3M)</t>
+          <t>INDUSTRY</t>
         </is>
       </c>
       <c r="D1089" s="4" t="inlineStr">
         <is>
-          <t>MOTOR DRIVE END BEARING</t>
+          <t>GREASE PUMP &amp; MANUAL FILLING PUMP</t>
         </is>
       </c>
       <c r="E1089" s="4" t="inlineStr">
         <is>
-          <t>MULTIS COMPLEX S2A</t>
+          <t>BIOMULTIS EP0</t>
         </is>
       </c>
       <c r="F1089" s="5" t="inlineStr">
@@ -40750,34 +40746,34 @@
       </c>
       <c r="G1089" s="4" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
     <row r="1090">
       <c r="A1090" s="2" t="inlineStr">
         <is>
-          <t>CENTRIFUGAL PUMP</t>
+          <t>AIR COND. PLANT</t>
         </is>
       </c>
       <c r="B1090" s="2" t="inlineStr">
         <is>
-          <t>SHINKO IND. LTD.</t>
+          <t>R-407C CONDENSING UNIT</t>
         </is>
       </c>
       <c r="C1090" s="2" t="inlineStr">
         <is>
-          <t>W.SPRAY PUMP (GVD300-3M)</t>
+          <t>(OSK8551/502320</t>
         </is>
       </c>
       <c r="D1090" s="2" t="inlineStr">
         <is>
-          <t>MOTOR NON-DRIVE END BEARING</t>
+          <t>OIL SEPARATOR</t>
         </is>
       </c>
       <c r="E1090" s="2" t="inlineStr">
         <is>
-          <t>MULTIS COMPLEX S2A</t>
+          <t>BITZER BSE 170</t>
         </is>
       </c>
       <c r="F1090" s="3" t="inlineStr">
@@ -40787,34 +40783,34 @@
       </c>
       <c r="G1090" s="2" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
     <row r="1091">
       <c r="A1091" s="4" t="inlineStr">
         <is>
-          <t>L.F.O. PURIFIER UNIT</t>
+          <t>AIR COND. PLANT</t>
         </is>
       </c>
       <c r="B1091" s="4" t="inlineStr">
         <is>
-          <t>SAMGONG 2 GEAR CASE</t>
+          <t>R-407C CONDENSING UNIT</t>
         </is>
       </c>
       <c r="C1091" s="4" t="inlineStr">
         <is>
-          <t>* NOTE) OIL REPLACEMENT INTERVALS</t>
+          <t>(OSK8551/502320</t>
         </is>
       </c>
       <c r="D1091" s="4" t="inlineStr">
         <is>
-          <t>GEAR CASE</t>
+          <t>REPLACEMENT OIL</t>
         </is>
       </c>
       <c r="E1091" s="4" t="inlineStr">
         <is>
-          <t>EPONA Z 150</t>
+          <t>BITZER BSE 170</t>
         </is>
       </c>
       <c r="F1091" s="5" t="inlineStr">
@@ -40824,34 +40820,34 @@
       </c>
       <c r="G1091" s="4" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
     <row r="1092">
       <c r="A1092" s="2" t="inlineStr">
         <is>
-          <t>INCINERATOR</t>
+          <t>PROV. REF. PLANT</t>
         </is>
       </c>
       <c r="B1092" s="2" t="inlineStr">
         <is>
-          <t>HYUNDAI MARINE MACHINERY CO.,</t>
+          <t>R-407C CONDENSING UNIT</t>
         </is>
       </c>
       <c r="C1092" s="2" t="inlineStr">
         <is>
-          <t>LTD.</t>
+          <t>(4T.2/221014)</t>
         </is>
       </c>
       <c r="D1092" s="2" t="inlineStr">
         <is>
-          <t>W.O. DOSING PUMP GEAR BOX</t>
+          <t>COMPRESSOR CRANKCASE</t>
         </is>
       </c>
       <c r="E1092" s="2" t="inlineStr">
         <is>
-          <t>EPONA Z 220</t>
+          <t>BITZER BSE 55</t>
         </is>
       </c>
       <c r="F1092" s="3" t="inlineStr">
@@ -40861,34 +40857,34 @@
       </c>
       <c r="G1092" s="2" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
     <row r="1093">
       <c r="A1093" s="4" t="inlineStr">
         <is>
-          <t>INCINERATOR</t>
+          <t>PROV. REF. PLANT</t>
         </is>
       </c>
       <c r="B1093" s="4" t="inlineStr">
         <is>
-          <t>HYUNDAI MARINE MACHINERY CO.,</t>
+          <t>R-407C CONDENSING UNIT</t>
         </is>
       </c>
       <c r="C1093" s="4" t="inlineStr">
         <is>
-          <t>LTD.</t>
+          <t>(4T.2/221014)</t>
         </is>
       </c>
       <c r="D1093" s="4" t="inlineStr">
         <is>
-          <t>MILL PUMP SEAL BOX</t>
+          <t>REPLACEMENT OIL</t>
         </is>
       </c>
       <c r="E1093" s="4" t="inlineStr">
         <is>
-          <t>VISGA 46</t>
+          <t>BITZER BSE 55</t>
         </is>
       </c>
       <c r="F1093" s="5" t="inlineStr">
@@ -40898,997 +40894,997 @@
       </c>
       <c r="G1093" s="4" t="inlineStr">
         <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
         </is>
       </c>
     </row>
     <row r="1094">
       <c r="A1094" s="2" t="inlineStr">
         <is>
+          <t>EM'CY GEN. ENGINE</t>
+        </is>
+      </c>
+      <c r="B1094" s="2" t="inlineStr">
+        <is>
+          <t>GPC - BAUDOUIN</t>
+        </is>
+      </c>
+      <c r="C1094" s="2" t="inlineStr">
+        <is>
+          <t>(12M33)</t>
+        </is>
+      </c>
+      <c r="D1094" s="2" t="inlineStr">
+        <is>
+          <t>MAIN LO SYSTEM</t>
+        </is>
+      </c>
+      <c r="E1094" s="2" t="inlineStr">
+        <is>
+          <t>DISOLA W 15W-40</t>
+        </is>
+      </c>
+      <c r="F1094" s="3" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1094" s="2" t="inlineStr">
+        <is>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" s="4" t="inlineStr">
+        <is>
+          <t>EM'CY GEN. ENGINE</t>
+        </is>
+      </c>
+      <c r="B1095" s="4" t="inlineStr">
+        <is>
+          <t>GPC - BAUDOUIN</t>
+        </is>
+      </c>
+      <c r="C1095" s="4" t="inlineStr">
+        <is>
+          <t>(12M33)</t>
+        </is>
+      </c>
+      <c r="D1095" s="4" t="inlineStr">
+        <is>
+          <t>HYDRO STARTING UNIT</t>
+        </is>
+      </c>
+      <c r="E1095" s="4" t="inlineStr">
+        <is>
+          <t>VISGA 32</t>
+        </is>
+      </c>
+      <c r="F1095" s="5" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1095" s="4" t="inlineStr">
+        <is>
+          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" s="2" t="inlineStr">
+        <is>
+          <t>MAIN ENGINE</t>
+        </is>
+      </c>
+      <c r="B1096" s="2" t="inlineStr">
+        <is>
+          <t>HYUNDAI-MAN B&amp;W</t>
+        </is>
+      </c>
+      <c r="C1096" s="2" t="inlineStr">
+        <is>
+          <t>6G60ME-C9.5-GIE-HPSCR</t>
+        </is>
+      </c>
+      <c r="D1096" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM OIL</t>
+        </is>
+      </c>
+      <c r="E1096" s="2" t="inlineStr">
+        <is>
+          <t>ATLANTA MARINE D 3005</t>
+        </is>
+      </c>
+      <c r="F1096" s="3" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1096" s="2" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" s="4" t="inlineStr">
+        <is>
+          <t>MAIN ENGINE</t>
+        </is>
+      </c>
+      <c r="B1097" s="4" t="inlineStr">
+        <is>
+          <t>HYUNDAI-MAN B&amp;W</t>
+        </is>
+      </c>
+      <c r="C1097" s="4" t="inlineStr">
+        <is>
+          <t>6G60ME-C9.5-GIE-HPSCR</t>
+        </is>
+      </c>
+      <c r="D1097" s="4" t="inlineStr">
+        <is>
+          <t>CYLINDER OIL</t>
+        </is>
+      </c>
+      <c r="E1097" s="4" t="inlineStr">
+        <is>
+          <t>TALUSIA HD 40</t>
+        </is>
+      </c>
+      <c r="F1097" s="5" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1097" s="4" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" s="2" t="inlineStr">
+        <is>
+          <t>MAIN ENGINE</t>
+        </is>
+      </c>
+      <c r="B1098" s="2" t="inlineStr">
+        <is>
+          <t>HYUNDAI-MAN B&amp;W</t>
+        </is>
+      </c>
+      <c r="C1098" s="2" t="inlineStr">
+        <is>
+          <t>6G60ME-C9.5-GIE-HPSCR</t>
+        </is>
+      </c>
+      <c r="D1098" s="2" t="inlineStr">
+        <is>
+          <t>FUEL VALVE TEST DEVICE OIL TANK</t>
+        </is>
+      </c>
+      <c r="E1098" s="2" t="inlineStr">
+        <is>
+          <t>VISGA 15</t>
+        </is>
+      </c>
+      <c r="F1098" s="3" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1098" s="2" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" s="4" t="inlineStr">
+        <is>
+          <t>MAIN ENGINE</t>
+        </is>
+      </c>
+      <c r="B1099" s="4" t="inlineStr">
+        <is>
+          <t>HYUNDAI-MAN B&amp;W</t>
+        </is>
+      </c>
+      <c r="C1099" s="4" t="inlineStr">
+        <is>
+          <t>6G60ME-C9.5-GIE-HPSCR</t>
+        </is>
+      </c>
+      <c r="D1099" s="4" t="inlineStr">
+        <is>
+          <t>PNEUMATIC HYD. H.P. PUMP</t>
+        </is>
+      </c>
+      <c r="E1099" s="4" t="inlineStr">
+        <is>
+          <t>VISGA 15</t>
+        </is>
+      </c>
+      <c r="F1099" s="5" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1099" s="4" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" s="2" t="inlineStr">
+        <is>
+          <t>MAIN ENGINE</t>
+        </is>
+      </c>
+      <c r="B1100" s="2" t="inlineStr">
+        <is>
+          <t>HYUNDAI-MAN B&amp;W</t>
+        </is>
+      </c>
+      <c r="C1100" s="2" t="inlineStr">
+        <is>
+          <t>6G60ME-C9.5-GIE-HPSCR</t>
+        </is>
+      </c>
+      <c r="D1100" s="2" t="inlineStr">
+        <is>
+          <t>TURNING ENCLOSED GEAR</t>
+        </is>
+      </c>
+      <c r="E1100" s="2" t="inlineStr">
+        <is>
+          <t>EPONA Z 320</t>
+        </is>
+      </c>
+      <c r="F1100" s="3" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1100" s="2" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" s="4" t="inlineStr">
+        <is>
+          <t>MAIN ENGINE</t>
+        </is>
+      </c>
+      <c r="B1101" s="4" t="inlineStr">
+        <is>
+          <t>HYUNDAI-MAN B&amp;W</t>
+        </is>
+      </c>
+      <c r="C1101" s="4" t="inlineStr">
+        <is>
+          <t>6G60ME-C9.5-GIE-HPSCR</t>
+        </is>
+      </c>
+      <c r="D1101" s="4" t="inlineStr">
+        <is>
+          <t>OPEN GEAR</t>
+        </is>
+      </c>
+      <c r="E1101" s="4" t="inlineStr">
+        <is>
+          <t>CERAN XM 220</t>
+        </is>
+      </c>
+      <c r="F1101" s="5" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1101" s="4" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" s="2" t="inlineStr">
+        <is>
+          <t>MAIN ENGINE</t>
+        </is>
+      </c>
+      <c r="B1102" s="2" t="inlineStr">
+        <is>
+          <t>HYUNDAI-MAN B&amp;W</t>
+        </is>
+      </c>
+      <c r="C1102" s="2" t="inlineStr">
+        <is>
+          <t>6G60ME-C9.5-GIE-HPSCR</t>
+        </is>
+      </c>
+      <c r="D1102" s="2" t="inlineStr">
+        <is>
+          <t>AUX. BLOWER GREASE POINT</t>
+        </is>
+      </c>
+      <c r="E1102" s="2" t="inlineStr">
+        <is>
+          <t>MULTIS MS 2</t>
+        </is>
+      </c>
+      <c r="F1102" s="3" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1102" s="2" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" s="4" t="inlineStr">
+        <is>
+          <t>MAIN ENGINE</t>
+        </is>
+      </c>
+      <c r="B1103" s="4" t="inlineStr">
+        <is>
+          <t>HYUNDAI-MAN B&amp;W</t>
+        </is>
+      </c>
+      <c r="C1103" s="4" t="inlineStr">
+        <is>
+          <t>6G60ME-C9.5-GIE-HPSCR</t>
+        </is>
+      </c>
+      <c r="D1103" s="4" t="inlineStr">
+        <is>
+          <t>GAS VALVE TEST DEVICE</t>
+        </is>
+      </c>
+      <c r="E1103" s="4" t="inlineStr">
+        <is>
+          <t>VISGA 32</t>
+        </is>
+      </c>
+      <c r="F1103" s="5" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1103" s="4" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" s="2" t="inlineStr">
+        <is>
+          <t>MAIN ENGINE</t>
+        </is>
+      </c>
+      <c r="B1104" s="2" t="inlineStr">
+        <is>
+          <t>HYUNDAI-MAN B&amp;W</t>
+        </is>
+      </c>
+      <c r="C1104" s="2" t="inlineStr">
+        <is>
+          <t>6G60ME-C9.5-GIE-HPSCR</t>
+        </is>
+      </c>
+      <c r="D1104" s="2" t="inlineStr">
+        <is>
+          <t>M/E HYD. TOP BRACING OIL CHAMBER</t>
+        </is>
+      </c>
+      <c r="E1104" s="2" t="inlineStr">
+        <is>
+          <t>VISGA 32</t>
+        </is>
+      </c>
+      <c r="F1104" s="3" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1104" s="2" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" s="4" t="inlineStr">
+        <is>
+          <t>D/G ENGINE</t>
+        </is>
+      </c>
+      <c r="B1105" s="4" t="inlineStr">
+        <is>
+          <t>HYUNDAI-HIMSEN</t>
+        </is>
+      </c>
+      <c r="C1105" s="4" t="inlineStr">
+        <is>
+          <t>8H25/33</t>
+        </is>
+      </c>
+      <c r="D1105" s="4" t="inlineStr">
+        <is>
+          <t>SYSTEM OIL</t>
+        </is>
+      </c>
+      <c r="E1105" s="4" t="inlineStr">
+        <is>
+          <t>AURELIA TI 4020</t>
+        </is>
+      </c>
+      <c r="F1105" s="5" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1105" s="4" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" s="2" t="inlineStr">
+        <is>
+          <t>D/G ENGINE</t>
+        </is>
+      </c>
+      <c r="B1106" s="2" t="inlineStr">
+        <is>
+          <t>HYUNDAI-HIMSEN</t>
+        </is>
+      </c>
+      <c r="C1106" s="2" t="inlineStr">
+        <is>
+          <t>8H25/33</t>
+        </is>
+      </c>
+      <c r="D1106" s="2" t="inlineStr">
+        <is>
+          <t>GOVERNOR</t>
+        </is>
+      </c>
+      <c r="E1106" s="2" t="inlineStr">
+        <is>
+          <t>AURELIA TI 4020</t>
+        </is>
+      </c>
+      <c r="F1106" s="3" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1106" s="2" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" s="4" t="inlineStr">
+        <is>
+          <t>G/E L.P. SCR</t>
+        </is>
+      </c>
+      <c r="B1107" s="4" t="inlineStr">
+        <is>
+          <t>HYUNDAI EMD</t>
+        </is>
+      </c>
+      <c r="C1107" s="4" t="inlineStr">
+        <is>
+          <t>BY-PASS VALVE</t>
+        </is>
+      </c>
+      <c r="D1107" s="4" t="inlineStr">
+        <is>
+          <t>SHAFT BEARING GEAR BOX</t>
+        </is>
+      </c>
+      <c r="E1107" s="4" t="inlineStr">
+        <is>
+          <t>R100 TECTYL G182 TECTYL G182</t>
+        </is>
+      </c>
+      <c r="F1107" s="5" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1107" s="4" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" s="2" t="inlineStr">
+        <is>
+          <t>AUXILIARY BOILER</t>
+        </is>
+      </c>
+      <c r="B1108" s="2" t="inlineStr">
+        <is>
+          <t>ALFA LAVAL</t>
+        </is>
+      </c>
+      <c r="C1108" s="2" t="inlineStr">
+        <is>
+          <t>AUXILIARY BOILER</t>
+        </is>
+      </c>
+      <c r="D1108" s="2" t="inlineStr">
+        <is>
+          <t>SAFETY VALVES- LIFTING FORK, LEVER REMOTE PULL FOR SAFETY VALVE -WIRE, SHACKLE, PULLY REMOTE PULL FOR LEVEL GAUGE -WIRE, SHACKLE, PULLY FEED WATER CONTROL VALVES - SPINDLE, STUFFING BOX PACKING FD FANS- BEARING, GREASE NIPPLE FEED WATER CONTROL VALVES- GEAR ACTUATOR</t>
+        </is>
+      </c>
+      <c r="E1108" s="2" t="inlineStr">
+        <is>
+          <t>CERAN XM 220 CERAN AD PLUS CERAN AD PLUS CERAN XM 220 CERAN XM 220 CERAN XM 220</t>
+        </is>
+      </c>
+      <c r="F1108" s="3" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1108" s="2" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" s="4" t="inlineStr">
+        <is>
+          <t>PISTON TYPE AIR COMPRESSOR</t>
+        </is>
+      </c>
+      <c r="B1109" s="4" t="inlineStr">
+        <is>
+          <t>DONGHWA PNEUTEC</t>
+        </is>
+      </c>
+      <c r="C1109" s="4" t="inlineStr">
+        <is>
+          <t>MAIN AIR COMPRESSOR</t>
+        </is>
+      </c>
+      <c r="D1109" s="4" t="inlineStr">
+        <is>
+          <t>CYLINDERS &amp; BEARINGS</t>
+        </is>
+      </c>
+      <c r="E1109" s="4" t="inlineStr">
+        <is>
+          <t>DACNIS 100</t>
+        </is>
+      </c>
+      <c r="F1109" s="5" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1109" s="4" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" s="2" t="inlineStr">
+        <is>
+          <t>PISTON TYPE AIR COMPRESSOR</t>
+        </is>
+      </c>
+      <c r="B1110" s="2" t="inlineStr">
+        <is>
+          <t>DONGHWA PNEUTEC</t>
+        </is>
+      </c>
+      <c r="C1110" s="2" t="inlineStr">
+        <is>
+          <t>MAIN AIR COMPRESSOR</t>
+        </is>
+      </c>
+      <c r="D1110" s="2" t="inlineStr">
+        <is>
+          <t>CYLINDERS &amp; BEARINGS</t>
+        </is>
+      </c>
+      <c r="E1110" s="2" t="inlineStr">
+        <is>
+          <t>MULTIS COMPLEX S2A</t>
+        </is>
+      </c>
+      <c r="F1110" s="3" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1110" s="2" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" s="4" t="inlineStr">
+        <is>
+          <t>SCREW TYPE AIR COMPRESSOR</t>
+        </is>
+      </c>
+      <c r="B1111" s="4" t="inlineStr">
+        <is>
+          <t>MAEKR : DONGHWA PNEUTEC</t>
+        </is>
+      </c>
+      <c r="C1111" s="4" t="inlineStr">
+        <is>
+          <t>NEX-45ABS</t>
+        </is>
+      </c>
+      <c r="D1111" s="4" t="inlineStr">
+        <is>
+          <t>CYLINDERS &amp; BEARINGS</t>
+        </is>
+      </c>
+      <c r="E1111" s="4" t="inlineStr">
+        <is>
+          <t>DACNIS 46</t>
+        </is>
+      </c>
+      <c r="F1111" s="5" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1111" s="4" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" s="2" t="inlineStr">
+        <is>
+          <t>SCREW TYPE AIR COMPRESSOR</t>
+        </is>
+      </c>
+      <c r="B1112" s="2" t="inlineStr">
+        <is>
+          <t>MAEKR : DONGHWA PNEUTEC</t>
+        </is>
+      </c>
+      <c r="C1112" s="2" t="inlineStr">
+        <is>
+          <t>NEX-45ABS</t>
+        </is>
+      </c>
+      <c r="D1112" s="2" t="inlineStr">
+        <is>
+          <t>CYLINDERS &amp; BEARINGS</t>
+        </is>
+      </c>
+      <c r="E1112" s="2" t="inlineStr">
+        <is>
+          <t>MULTIS COMPLEX S2A</t>
+        </is>
+      </c>
+      <c r="F1112" s="3" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1112" s="2" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" s="4" t="inlineStr">
+        <is>
+          <t>CENTRIFUGAL PUMP</t>
+        </is>
+      </c>
+      <c r="B1113" s="4" t="inlineStr">
+        <is>
+          <t>SHINKO IND. LTD.</t>
+        </is>
+      </c>
+      <c r="C1113" s="4" t="inlineStr">
+        <is>
+          <t>W.SPRAY PUMP (GVD300-3M)</t>
+        </is>
+      </c>
+      <c r="D1113" s="4" t="inlineStr">
+        <is>
+          <t>COUPLING SIDE BEARING</t>
+        </is>
+      </c>
+      <c r="E1113" s="4" t="inlineStr">
+        <is>
+          <t>CERAN XM 220</t>
+        </is>
+      </c>
+      <c r="F1113" s="5" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1113" s="4" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" s="2" t="inlineStr">
+        <is>
+          <t>CENTRIFUGAL PUMP</t>
+        </is>
+      </c>
+      <c r="B1114" s="2" t="inlineStr">
+        <is>
+          <t>SHINKO IND. LTD.</t>
+        </is>
+      </c>
+      <c r="C1114" s="2" t="inlineStr">
+        <is>
+          <t>W.SPRAY PUMP (GVD300-3M)</t>
+        </is>
+      </c>
+      <c r="D1114" s="2" t="inlineStr">
+        <is>
+          <t>BEARING HOUSING</t>
+        </is>
+      </c>
+      <c r="E1114" s="2" t="inlineStr">
+        <is>
+          <t>PRESLIA 68</t>
+        </is>
+      </c>
+      <c r="F1114" s="3" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1114" s="2" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" s="4" t="inlineStr">
+        <is>
+          <t>CENTRIFUGAL PUMP</t>
+        </is>
+      </c>
+      <c r="B1115" s="4" t="inlineStr">
+        <is>
+          <t>SHINKO IND. LTD.</t>
+        </is>
+      </c>
+      <c r="C1115" s="4" t="inlineStr">
+        <is>
+          <t>W.SPRAY PUMP (GVD300-3M)</t>
+        </is>
+      </c>
+      <c r="D1115" s="4" t="inlineStr">
+        <is>
+          <t>MOTOR DRIVE END BEARING</t>
+        </is>
+      </c>
+      <c r="E1115" s="4" t="inlineStr">
+        <is>
+          <t>MULTIS COMPLEX S2A</t>
+        </is>
+      </c>
+      <c r="F1115" s="5" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1115" s="4" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" s="2" t="inlineStr">
+        <is>
+          <t>CENTRIFUGAL PUMP</t>
+        </is>
+      </c>
+      <c r="B1116" s="2" t="inlineStr">
+        <is>
+          <t>SHINKO IND. LTD.</t>
+        </is>
+      </c>
+      <c r="C1116" s="2" t="inlineStr">
+        <is>
+          <t>W.SPRAY PUMP (GVD300-3M)</t>
+        </is>
+      </c>
+      <c r="D1116" s="2" t="inlineStr">
+        <is>
+          <t>MOTOR NON-DRIVE END BEARING</t>
+        </is>
+      </c>
+      <c r="E1116" s="2" t="inlineStr">
+        <is>
+          <t>MULTIS COMPLEX S2A</t>
+        </is>
+      </c>
+      <c r="F1116" s="3" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1116" s="2" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" s="4" t="inlineStr">
+        <is>
+          <t>L.F.O. PURIFIER UNIT</t>
+        </is>
+      </c>
+      <c r="B1117" s="4" t="inlineStr">
+        <is>
+          <t>SAMGONG 2 GEAR CASE</t>
+        </is>
+      </c>
+      <c r="C1117" s="4" t="inlineStr">
+        <is>
+          <t>* NOTE) OIL REPLACEMENT INTERVALS</t>
+        </is>
+      </c>
+      <c r="D1117" s="4" t="inlineStr">
+        <is>
+          <t>GEAR CASE</t>
+        </is>
+      </c>
+      <c r="E1117" s="4" t="inlineStr">
+        <is>
+          <t>EPONA Z 150</t>
+        </is>
+      </c>
+      <c r="F1117" s="5" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1117" s="4" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" s="2" t="inlineStr">
+        <is>
+          <t>INCINERATOR</t>
+        </is>
+      </c>
+      <c r="B1118" s="2" t="inlineStr">
+        <is>
+          <t>HYUNDAI MARINE MACHINERY CO.,</t>
+        </is>
+      </c>
+      <c r="C1118" s="2" t="inlineStr">
+        <is>
+          <t>LTD.</t>
+        </is>
+      </c>
+      <c r="D1118" s="2" t="inlineStr">
+        <is>
+          <t>W.O. DOSING PUMP GEAR BOX</t>
+        </is>
+      </c>
+      <c r="E1118" s="2" t="inlineStr">
+        <is>
+          <t>EPONA Z 220</t>
+        </is>
+      </c>
+      <c r="F1118" s="3" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1118" s="2" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" s="4" t="inlineStr">
+        <is>
+          <t>INCINERATOR</t>
+        </is>
+      </c>
+      <c r="B1119" s="4" t="inlineStr">
+        <is>
+          <t>HYUNDAI MARINE MACHINERY CO.,</t>
+        </is>
+      </c>
+      <c r="C1119" s="4" t="inlineStr">
+        <is>
+          <t>LTD.</t>
+        </is>
+      </c>
+      <c r="D1119" s="4" t="inlineStr">
+        <is>
+          <t>MILL PUMP SEAL BOX</t>
+        </is>
+      </c>
+      <c r="E1119" s="4" t="inlineStr">
+        <is>
+          <t>VISGA 46</t>
+        </is>
+      </c>
+      <c r="F1119" s="5" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="G1119" s="4" t="inlineStr">
+        <is>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" s="2" t="inlineStr">
+        <is>
           <t>VENTILATION FAN
 FOR MACHINERY OUTFITTING SPACE</t>
         </is>
       </c>
-      <c r="B1094" s="2" t="inlineStr">
+      <c r="B1120" s="2" t="inlineStr">
         <is>
           <t>HI AIR KOREA</t>
         </is>
       </c>
-      <c r="C1094" s="2" t="inlineStr">
+      <c r="C1120" s="2" t="inlineStr">
         <is>
           <t>PNEU. CLOSING DAMPER FOR NO.1~4</t>
         </is>
       </c>
-      <c r="D1094" s="2" t="inlineStr">
+      <c r="D1120" s="2" t="inlineStr">
         <is>
           <t>GREASE NIPPLE FOR SHAFT</t>
         </is>
       </c>
-      <c r="E1094" s="2" t="inlineStr">
+      <c r="E1120" s="2" t="inlineStr">
         <is>
           <t>CERAN XM 220</t>
-        </is>
-      </c>
-      <c r="F1094" s="3" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1094" s="2" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1095">
-      <c r="A1095" s="4" t="inlineStr">
-        <is>
-          <t>ENGINE ROOM OVERHEAD CRANE</t>
-        </is>
-      </c>
-      <c r="B1095" s="4" t="inlineStr">
-        <is>
-          <t>ORIENTAL</t>
-        </is>
-      </c>
-      <c r="C1095" s="4" t="inlineStr">
-        <is>
-          <t>S.W.L. 4.0 TON</t>
-        </is>
-      </c>
-      <c r="D1095" s="4" t="inlineStr">
-        <is>
-          <t>HOISTING GEAR BOX</t>
-        </is>
-      </c>
-      <c r="E1095" s="4" t="inlineStr">
-        <is>
-          <t>EPONA Z 220</t>
-        </is>
-      </c>
-      <c r="F1095" s="5" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1095" s="4" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1096">
-      <c r="A1096" s="2" t="inlineStr">
-        <is>
-          <t>ENGINE ROOM OVERHEAD CRANE</t>
-        </is>
-      </c>
-      <c r="B1096" s="2" t="inlineStr">
-        <is>
-          <t>ORIENTAL</t>
-        </is>
-      </c>
-      <c r="C1096" s="2" t="inlineStr">
-        <is>
-          <t>S.W.L. 4.0 TON</t>
-        </is>
-      </c>
-      <c r="D1096" s="2" t="inlineStr">
-        <is>
-          <t>WIRE ROPE</t>
-        </is>
-      </c>
-      <c r="E1096" s="2" t="inlineStr">
-        <is>
-          <t>CERAN AD PLUS</t>
-        </is>
-      </c>
-      <c r="F1096" s="3" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1096" s="2" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1097">
-      <c r="A1097" s="4" t="inlineStr">
-        <is>
-          <t>ENGINE ROOM OVERHEAD CRANE</t>
-        </is>
-      </c>
-      <c r="B1097" s="4" t="inlineStr">
-        <is>
-          <t>ORIENTAL</t>
-        </is>
-      </c>
-      <c r="C1097" s="4" t="inlineStr">
-        <is>
-          <t>S.W.L. 4.0 TON</t>
-        </is>
-      </c>
-      <c r="D1097" s="4" t="inlineStr">
-        <is>
-          <t>OPEN GEAR</t>
-        </is>
-      </c>
-      <c r="E1097" s="4" t="inlineStr">
-        <is>
-          <t>CERAN AD PLUS</t>
-        </is>
-      </c>
-      <c r="F1097" s="5" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1097" s="4" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1098">
-      <c r="A1098" s="2" t="inlineStr">
-        <is>
-          <t>ENGINE ROOM OVERHEAD CRANE</t>
-        </is>
-      </c>
-      <c r="B1098" s="2" t="inlineStr">
-        <is>
-          <t>ORIENTAL</t>
-        </is>
-      </c>
-      <c r="C1098" s="2" t="inlineStr">
-        <is>
-          <t>S.W.L. 4.0 TON</t>
-        </is>
-      </c>
-      <c r="D1098" s="2" t="inlineStr">
-        <is>
-          <t>TRAVERSING GEAR BOX</t>
-        </is>
-      </c>
-      <c r="E1098" s="2" t="inlineStr">
-        <is>
-          <t>CERAN XM 220</t>
-        </is>
-      </c>
-      <c r="F1098" s="3" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1098" s="2" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1099">
-      <c r="A1099" s="4" t="inlineStr">
-        <is>
-          <t>ENGINE ROOM OVERHEAD CRANE</t>
-        </is>
-      </c>
-      <c r="B1099" s="4" t="inlineStr">
-        <is>
-          <t>ORIENTAL</t>
-        </is>
-      </c>
-      <c r="C1099" s="4" t="inlineStr">
-        <is>
-          <t>S.W.L. 4.0 TON</t>
-        </is>
-      </c>
-      <c r="D1099" s="4" t="inlineStr">
-        <is>
-          <t>HOOK BLOCK</t>
-        </is>
-      </c>
-      <c r="E1099" s="4" t="inlineStr">
-        <is>
-          <t>CERAN XM 220</t>
-        </is>
-      </c>
-      <c r="F1099" s="5" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1099" s="4" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1100">
-      <c r="A1100" s="2" t="inlineStr">
-        <is>
-          <t>WORKSHOP MACHINERY</t>
-        </is>
-      </c>
-      <c r="B1100" s="2" t="inlineStr">
-        <is>
-          <t>TMS SOLUTION</t>
-        </is>
-      </c>
-      <c r="C1100" s="2" t="inlineStr">
-        <is>
-          <t>LATHE (TYC510)</t>
-        </is>
-      </c>
-      <c r="D1100" s="2" t="inlineStr">
-        <is>
-          <t>DRILLING MACHINE- SLEEVE</t>
-        </is>
-      </c>
-      <c r="E1100" s="2" t="inlineStr">
-        <is>
-          <t>VISGA 32</t>
-        </is>
-      </c>
-      <c r="F1100" s="3" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1100" s="2" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1101">
-      <c r="A1101" s="4" t="inlineStr">
-        <is>
-          <t>WORKSHOP MACHINERY</t>
-        </is>
-      </c>
-      <c r="B1101" s="4" t="inlineStr">
-        <is>
-          <t>TMS SOLUTION</t>
-        </is>
-      </c>
-      <c r="C1101" s="4" t="inlineStr">
-        <is>
-          <t>LATHE (TYC510)</t>
-        </is>
-      </c>
-      <c r="D1101" s="4" t="inlineStr">
-        <is>
-          <t>DRILLING MACHINE- BAND GEAR BOX</t>
-        </is>
-      </c>
-      <c r="E1101" s="4" t="inlineStr">
-        <is>
-          <t>CERAN XM 220</t>
-        </is>
-      </c>
-      <c r="F1101" s="5" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1101" s="4" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1102">
-      <c r="A1102" s="2" t="inlineStr">
-        <is>
-          <t>WORKSHOP MACHINERY</t>
-        </is>
-      </c>
-      <c r="B1102" s="2" t="inlineStr">
-        <is>
-          <t>TMS SOLUTION</t>
-        </is>
-      </c>
-      <c r="C1102" s="2" t="inlineStr">
-        <is>
-          <t>LATHE (TYC510)</t>
-        </is>
-      </c>
-      <c r="D1102" s="2" t="inlineStr">
-        <is>
-          <t>DRILLING MACHINE- SPINDLE</t>
-        </is>
-      </c>
-      <c r="E1102" s="2" t="inlineStr">
-        <is>
-          <t>VISGA 32</t>
-        </is>
-      </c>
-      <c r="F1102" s="3" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1102" s="2" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1103">
-      <c r="A1103" s="4" t="inlineStr">
-        <is>
-          <t>WORKSHOP MACHINERY</t>
-        </is>
-      </c>
-      <c r="B1103" s="4" t="inlineStr">
-        <is>
-          <t>TMS SOLUTION</t>
-        </is>
-      </c>
-      <c r="C1103" s="4" t="inlineStr">
-        <is>
-          <t>LATHE (TYC510)</t>
-        </is>
-      </c>
-      <c r="D1103" s="4" t="inlineStr">
-        <is>
-          <t>DRILLING MACHINE- HEAD GEAR</t>
-        </is>
-      </c>
-      <c r="E1103" s="4" t="inlineStr">
-        <is>
-          <t>VISGA 32</t>
-        </is>
-      </c>
-      <c r="F1103" s="5" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1103" s="4" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1104">
-      <c r="A1104" s="2" t="inlineStr">
-        <is>
-          <t>WORKSHOP MACHINERY</t>
-        </is>
-      </c>
-      <c r="B1104" s="2" t="inlineStr">
-        <is>
-          <t>TMS SOLUTION</t>
-        </is>
-      </c>
-      <c r="C1104" s="2" t="inlineStr">
-        <is>
-          <t>LATHE (TYC510)</t>
-        </is>
-      </c>
-      <c r="D1104" s="2" t="inlineStr">
-        <is>
-          <t>DRILLING MACHINE- COLUMN GEAR</t>
-        </is>
-      </c>
-      <c r="E1104" s="2" t="inlineStr">
-        <is>
-          <t>CERAN XM 220</t>
-        </is>
-      </c>
-      <c r="F1104" s="3" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1104" s="2" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1105">
-      <c r="A1105" s="4" t="inlineStr">
-        <is>
-          <t>WORKSHOP MACHINERY</t>
-        </is>
-      </c>
-      <c r="B1105" s="4" t="inlineStr">
-        <is>
-          <t>TMS SOLUTION</t>
-        </is>
-      </c>
-      <c r="C1105" s="4" t="inlineStr">
-        <is>
-          <t>LATHE (TYC510)</t>
-        </is>
-      </c>
-      <c r="D1105" s="4" t="inlineStr">
-        <is>
-          <t>LATHE- HEAD STOCK</t>
-        </is>
-      </c>
-      <c r="E1105" s="4" t="inlineStr">
-        <is>
-          <t>VISGA 32</t>
-        </is>
-      </c>
-      <c r="F1105" s="5" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1105" s="4" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1106">
-      <c r="A1106" s="2" t="inlineStr">
-        <is>
-          <t>WORKSHOP MACHINERY</t>
-        </is>
-      </c>
-      <c r="B1106" s="2" t="inlineStr">
-        <is>
-          <t>TMS SOLUTION</t>
-        </is>
-      </c>
-      <c r="C1106" s="2" t="inlineStr">
-        <is>
-          <t>LATHE (TYC510)</t>
-        </is>
-      </c>
-      <c r="D1106" s="2" t="inlineStr">
-        <is>
-          <t>LATHE- FEED BOX</t>
-        </is>
-      </c>
-      <c r="E1106" s="2" t="inlineStr">
-        <is>
-          <t>VISGA 32</t>
-        </is>
-      </c>
-      <c r="F1106" s="3" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1106" s="2" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1107">
-      <c r="A1107" s="4" t="inlineStr">
-        <is>
-          <t>WORKSHOP MACHINERY</t>
-        </is>
-      </c>
-      <c r="B1107" s="4" t="inlineStr">
-        <is>
-          <t>TMS SOLUTION</t>
-        </is>
-      </c>
-      <c r="C1107" s="4" t="inlineStr">
-        <is>
-          <t>LATHE (TYC510)</t>
-        </is>
-      </c>
-      <c r="D1107" s="4" t="inlineStr">
-        <is>
-          <t>LATHE- APRON</t>
-        </is>
-      </c>
-      <c r="E1107" s="4" t="inlineStr">
-        <is>
-          <t>VISGA 32</t>
-        </is>
-      </c>
-      <c r="F1107" s="5" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1107" s="4" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1108">
-      <c r="A1108" s="2" t="inlineStr">
-        <is>
-          <t>WORKSHOP MACHINERY</t>
-        </is>
-      </c>
-      <c r="B1108" s="2" t="inlineStr">
-        <is>
-          <t>TMS SOLUTION</t>
-        </is>
-      </c>
-      <c r="C1108" s="2" t="inlineStr">
-        <is>
-          <t>LATHE (TYC510)</t>
-        </is>
-      </c>
-      <c r="D1108" s="2" t="inlineStr">
-        <is>
-          <t>LATHE- OIL POINTER</t>
-        </is>
-      </c>
-      <c r="E1108" s="2" t="inlineStr">
-        <is>
-          <t>VISGA 32</t>
-        </is>
-      </c>
-      <c r="F1108" s="3" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1108" s="2" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1109">
-      <c r="A1109" s="4" t="inlineStr">
-        <is>
-          <t>WORKSHOP MACHINERY</t>
-        </is>
-      </c>
-      <c r="B1109" s="4" t="inlineStr">
-        <is>
-          <t>TMS SOLUTION</t>
-        </is>
-      </c>
-      <c r="C1109" s="4" t="inlineStr">
-        <is>
-          <t>LATHE (TYC510)</t>
-        </is>
-      </c>
-      <c r="D1109" s="4" t="inlineStr">
-        <is>
-          <t>LATHE- CHANGE GEAR</t>
-        </is>
-      </c>
-      <c r="E1109" s="4" t="inlineStr">
-        <is>
-          <t>VISGA 32</t>
-        </is>
-      </c>
-      <c r="F1109" s="5" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1109" s="4" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1110">
-      <c r="A1110" s="2" t="inlineStr">
-        <is>
-          <t>WORKSHOP MACHINERY</t>
-        </is>
-      </c>
-      <c r="B1110" s="2" t="inlineStr">
-        <is>
-          <t>TMS SOLUTION</t>
-        </is>
-      </c>
-      <c r="C1110" s="2" t="inlineStr">
-        <is>
-          <t>LATHE (TYC510)</t>
-        </is>
-      </c>
-      <c r="D1110" s="2" t="inlineStr">
-        <is>
-          <t>LATHE- ACTION BAR</t>
-        </is>
-      </c>
-      <c r="E1110" s="2" t="inlineStr">
-        <is>
-          <t>VISGA 32</t>
-        </is>
-      </c>
-      <c r="F1110" s="3" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1110" s="2" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1111">
-      <c r="A1111" s="4" t="inlineStr">
-        <is>
-          <t>WORKSHOP MACHINERY</t>
-        </is>
-      </c>
-      <c r="B1111" s="4" t="inlineStr">
-        <is>
-          <t>TMS SOLUTION</t>
-        </is>
-      </c>
-      <c r="C1111" s="4" t="inlineStr">
-        <is>
-          <t>LATHE (TYC510)</t>
-        </is>
-      </c>
-      <c r="D1111" s="4" t="inlineStr">
-        <is>
-          <t>LATHE- TAILSTOCK</t>
-        </is>
-      </c>
-      <c r="E1111" s="4" t="inlineStr">
-        <is>
-          <t>VISGA 32</t>
-        </is>
-      </c>
-      <c r="F1111" s="5" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1111" s="4" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1112">
-      <c r="A1112" s="2" t="inlineStr">
-        <is>
-          <t>WORKSHOP MACHINERY</t>
-        </is>
-      </c>
-      <c r="B1112" s="2" t="inlineStr">
-        <is>
-          <t>TMS SOLUTION</t>
-        </is>
-      </c>
-      <c r="C1112" s="2" t="inlineStr">
-        <is>
-          <t>LATHE (TYC510)</t>
-        </is>
-      </c>
-      <c r="D1112" s="2" t="inlineStr">
-        <is>
-          <t>LATHE- CARRIAGE</t>
-        </is>
-      </c>
-      <c r="E1112" s="2" t="inlineStr">
-        <is>
-          <t>VISGA 32</t>
-        </is>
-      </c>
-      <c r="F1112" s="3" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1112" s="2" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1113">
-      <c r="A1113" s="4" t="inlineStr">
-        <is>
-          <t>ENGINE ROOM PUMP</t>
-        </is>
-      </c>
-      <c r="B1113" s="4" t="inlineStr">
-        <is>
-          <t>IMO</t>
-        </is>
-      </c>
-      <c r="C1113" s="4" t="inlineStr">
-        <is>
-          <t>IINO KAI</t>
-        </is>
-      </c>
-      <c r="D1113" s="4" t="inlineStr">
-        <is>
-          <t>M.G.O. TRANSFER PUMP</t>
-        </is>
-      </c>
-      <c r="E1113" s="4" t="inlineStr">
-        <is>
-          <t>MULTIS EP 3</t>
-        </is>
-      </c>
-      <c r="F1113" s="5" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1113" s="4" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1114">
-      <c r="A1114" s="2" t="inlineStr">
-        <is>
-          <t>ENGINE ROOM PUMP</t>
-        </is>
-      </c>
-      <c r="B1114" s="2" t="inlineStr">
-        <is>
-          <t>IMO</t>
-        </is>
-      </c>
-      <c r="C1114" s="2" t="inlineStr">
-        <is>
-          <t>IINO KAI</t>
-        </is>
-      </c>
-      <c r="D1114" s="2" t="inlineStr">
-        <is>
-          <t>L.F.O. TRANSFER PUMP</t>
-        </is>
-      </c>
-      <c r="E1114" s="2" t="inlineStr">
-        <is>
-          <t>MULTIS EP 3</t>
-        </is>
-      </c>
-      <c r="F1114" s="3" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1114" s="2" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1115">
-      <c r="A1115" s="4" t="inlineStr">
-        <is>
-          <t>ENGINE ROOM PUMP</t>
-        </is>
-      </c>
-      <c r="B1115" s="4" t="inlineStr">
-        <is>
-          <t>IMO</t>
-        </is>
-      </c>
-      <c r="C1115" s="4" t="inlineStr">
-        <is>
-          <t>IINO KAI</t>
-        </is>
-      </c>
-      <c r="D1115" s="4" t="inlineStr">
-        <is>
-          <t>FWD L.F.O. TRANSFER PUMP</t>
-        </is>
-      </c>
-      <c r="E1115" s="4" t="inlineStr">
-        <is>
-          <t>MULTIS EP 3</t>
-        </is>
-      </c>
-      <c r="F1115" s="5" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1115" s="4" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1116">
-      <c r="A1116" s="2" t="inlineStr">
-        <is>
-          <t>ENGINE ROOM PUMP</t>
-        </is>
-      </c>
-      <c r="B1116" s="2" t="inlineStr">
-        <is>
-          <t>IMO</t>
-        </is>
-      </c>
-      <c r="C1116" s="2" t="inlineStr">
-        <is>
-          <t>IINO KAI</t>
-        </is>
-      </c>
-      <c r="D1116" s="2" t="inlineStr">
-        <is>
-          <t>OILY BILGE PUMP</t>
-        </is>
-      </c>
-      <c r="E1116" s="2" t="inlineStr">
-        <is>
-          <t>EPONA Z 460</t>
-        </is>
-      </c>
-      <c r="F1116" s="3" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1116" s="2" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1117">
-      <c r="A1117" s="4" t="inlineStr">
-        <is>
-          <t>ENGINE ROOM PUMP</t>
-        </is>
-      </c>
-      <c r="B1117" s="4" t="inlineStr">
-        <is>
-          <t>IMO</t>
-        </is>
-      </c>
-      <c r="C1117" s="4" t="inlineStr">
-        <is>
-          <t>IINO KAI</t>
-        </is>
-      </c>
-      <c r="D1117" s="4" t="inlineStr">
-        <is>
-          <t>BILGE CIRC. PUMP</t>
-        </is>
-      </c>
-      <c r="E1117" s="4" t="inlineStr">
-        <is>
-          <t>EPONA Z 460</t>
-        </is>
-      </c>
-      <c r="F1117" s="5" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1117" s="4" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1118">
-      <c r="A1118" s="2" t="inlineStr">
-        <is>
-          <t>ENGINE ROOM PUMP</t>
-        </is>
-      </c>
-      <c r="B1118" s="2" t="inlineStr">
-        <is>
-          <t>IMO</t>
-        </is>
-      </c>
-      <c r="C1118" s="2" t="inlineStr">
-        <is>
-          <t>IINO KAI</t>
-        </is>
-      </c>
-      <c r="D1118" s="2" t="inlineStr">
-        <is>
-          <t>SLUDGE PUMP</t>
-        </is>
-      </c>
-      <c r="E1118" s="2" t="inlineStr">
-        <is>
-          <t>EPONA Z 460</t>
-        </is>
-      </c>
-      <c r="F1118" s="3" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1118" s="2" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1119">
-      <c r="A1119" s="4" t="inlineStr">
-        <is>
-          <t>STEERING GEAR</t>
-        </is>
-      </c>
-      <c r="B1119" s="4" t="inlineStr">
-        <is>
-          <t>YOOWON-MITSUBISHI</t>
-        </is>
-      </c>
-      <c r="C1119" s="4" t="inlineStr">
-        <is>
-          <t>YDFT-200-2</t>
-        </is>
-      </c>
-      <c r="D1119" s="4" t="inlineStr">
-        <is>
-          <t>HYD. OIL STOR. TK</t>
-        </is>
-      </c>
-      <c r="E1119" s="4" t="inlineStr">
-        <is>
-          <t>PRESLIA 68</t>
-        </is>
-      </c>
-      <c r="F1119" s="5" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="G1119" s="4" t="inlineStr">
-        <is>
-          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="1120">
-      <c r="A1120" s="2" t="inlineStr">
-        <is>
-          <t>STEERING GEAR</t>
-        </is>
-      </c>
-      <c r="B1120" s="2" t="inlineStr">
-        <is>
-          <t>YOOWON-MITSUBISHI</t>
-        </is>
-      </c>
-      <c r="C1120" s="2" t="inlineStr">
-        <is>
-          <t>YDFT-200-2</t>
-        </is>
-      </c>
-      <c r="D1120" s="2" t="inlineStr">
-        <is>
-          <t>PUMP, CYLINDER, PIPE</t>
-        </is>
-      </c>
-      <c r="E1120" s="2" t="inlineStr">
-        <is>
-          <t>PRESLIA 68</t>
         </is>
       </c>
       <c r="F1120" s="3" t="inlineStr">
@@ -41905,27 +41901,27 @@
     <row r="1121">
       <c r="A1121" s="4" t="inlineStr">
         <is>
-          <t>STERN TUBE SYSTEM</t>
+          <t>ENGINE ROOM OVERHEAD CRANE</t>
         </is>
       </c>
       <c r="B1121" s="4" t="inlineStr">
         <is>
-          <t>KEMEL</t>
+          <t>ORIENTAL</t>
         </is>
       </c>
       <c r="C1121" s="4" t="inlineStr">
         <is>
-          <t>AFT/FWD : AX-630</t>
+          <t>S.W.L. 4.0 TON</t>
         </is>
       </c>
       <c r="D1121" s="4" t="inlineStr">
         <is>
-          <t>S/T L.O. TANK</t>
+          <t>HOISTING GEAR BOX</t>
         </is>
       </c>
       <c r="E1121" s="4" t="inlineStr">
         <is>
-          <t>ATLANTA MARINE D 3005</t>
+          <t>EPONA Z 220</t>
         </is>
       </c>
       <c r="F1121" s="5" t="inlineStr">
@@ -41942,27 +41938,27 @@
     <row r="1122">
       <c r="A1122" s="2" t="inlineStr">
         <is>
-          <t>STERN TUBE SYSTEM</t>
+          <t>ENGINE ROOM OVERHEAD CRANE</t>
         </is>
       </c>
       <c r="B1122" s="2" t="inlineStr">
         <is>
-          <t>KEMEL</t>
+          <t>ORIENTAL</t>
         </is>
       </c>
       <c r="C1122" s="2" t="inlineStr">
         <is>
-          <t>AFT/FWD : AX-630</t>
+          <t>S.W.L. 4.0 TON</t>
         </is>
       </c>
       <c r="D1122" s="2" t="inlineStr">
         <is>
-          <t>FWD SEAL TANK</t>
+          <t>WIRE ROPE</t>
         </is>
       </c>
       <c r="E1122" s="2" t="inlineStr">
         <is>
-          <t>ATLANTA MARINE D 3005</t>
+          <t>CERAN AD PLUS</t>
         </is>
       </c>
       <c r="F1122" s="3" t="inlineStr">
@@ -41979,27 +41975,27 @@
     <row r="1123">
       <c r="A1123" s="4" t="inlineStr">
         <is>
-          <t>STERN TUBE SYSTEM</t>
+          <t>ENGINE ROOM OVERHEAD CRANE</t>
         </is>
       </c>
       <c r="B1123" s="4" t="inlineStr">
         <is>
-          <t>KEMEL</t>
+          <t>ORIENTAL</t>
         </is>
       </c>
       <c r="C1123" s="4" t="inlineStr">
         <is>
-          <t>AFT/FWD : AX-630</t>
+          <t>S.W.L. 4.0 TON</t>
         </is>
       </c>
       <c r="D1123" s="4" t="inlineStr">
         <is>
-          <t>S/T LO SUMP TANK</t>
+          <t>OPEN GEAR</t>
         </is>
       </c>
       <c r="E1123" s="4" t="inlineStr">
         <is>
-          <t>ATLANTA MARINE D 3005</t>
+          <t>CERAN AD PLUS</t>
         </is>
       </c>
       <c r="F1123" s="5" t="inlineStr">
@@ -42016,27 +42012,27 @@
     <row r="1124">
       <c r="A1124" s="2" t="inlineStr">
         <is>
-          <t>STERN TUBE SYSTEM</t>
+          <t>ENGINE ROOM OVERHEAD CRANE</t>
         </is>
       </c>
       <c r="B1124" s="2" t="inlineStr">
         <is>
-          <t>KEMEL</t>
+          <t>ORIENTAL</t>
         </is>
       </c>
       <c r="C1124" s="2" t="inlineStr">
         <is>
-          <t>AFT/FWD : AX-630</t>
+          <t>S.W.L. 4.0 TON</t>
         </is>
       </c>
       <c r="D1124" s="2" t="inlineStr">
         <is>
-          <t>S/T LO PIPE LINE</t>
+          <t>TRAVERSING GEAR BOX</t>
         </is>
       </c>
       <c r="E1124" s="2" t="inlineStr">
         <is>
-          <t>ATLANTA MARINE D 3005</t>
+          <t>CERAN XM 220</t>
         </is>
       </c>
       <c r="F1124" s="3" t="inlineStr">
@@ -42053,27 +42049,27 @@
     <row r="1125">
       <c r="A1125" s="4" t="inlineStr">
         <is>
-          <t>STERN TUBE SYSTEM</t>
+          <t>ENGINE ROOM OVERHEAD CRANE</t>
         </is>
       </c>
       <c r="B1125" s="4" t="inlineStr">
         <is>
-          <t>KEMEL</t>
+          <t>ORIENTAL</t>
         </is>
       </c>
       <c r="C1125" s="4" t="inlineStr">
         <is>
-          <t>AFT/FWD : AX-630</t>
+          <t>S.W.L. 4.0 TON</t>
         </is>
       </c>
       <c r="D1125" s="4" t="inlineStr">
         <is>
-          <t>AFT &amp; FWD SEAL CHAMBER</t>
+          <t>HOOK BLOCK</t>
         </is>
       </c>
       <c r="E1125" s="4" t="inlineStr">
         <is>
-          <t>ATLANTA MARINE D 3005</t>
+          <t>CERAN XM 220</t>
         </is>
       </c>
       <c r="F1125" s="5" t="inlineStr">
@@ -42090,27 +42086,27 @@
     <row r="1126">
       <c r="A1126" s="2" t="inlineStr">
         <is>
-          <t>STERN TUBE SYSTEM</t>
+          <t>WORKSHOP MACHINERY</t>
         </is>
       </c>
       <c r="B1126" s="2" t="inlineStr">
         <is>
-          <t>KEMEL</t>
+          <t>TMS SOLUTION</t>
         </is>
       </c>
       <c r="C1126" s="2" t="inlineStr">
         <is>
-          <t>AFT/FWD : AX-630</t>
+          <t>LATHE (TYC510)</t>
         </is>
       </c>
       <c r="D1126" s="2" t="inlineStr">
         <is>
-          <t>S/T INSIDE</t>
+          <t>DRILLING MACHINE- SLEEVE</t>
         </is>
       </c>
       <c r="E1126" s="2" t="inlineStr">
         <is>
-          <t>ATLANTA MARINE D 3005</t>
+          <t>VISGA 32</t>
         </is>
       </c>
       <c r="F1126" s="3" t="inlineStr">
@@ -42127,27 +42123,27 @@
     <row r="1127">
       <c r="A1127" s="4" t="inlineStr">
         <is>
-          <t>INTER. SHAFT BEARING</t>
+          <t>WORKSHOP MACHINERY</t>
         </is>
       </c>
       <c r="B1127" s="4" t="inlineStr">
         <is>
-          <t>KEMEL</t>
+          <t>TMS SOLUTION</t>
         </is>
       </c>
       <c r="C1127" s="4" t="inlineStr">
         <is>
-          <t>KMS-620</t>
+          <t>LATHE (TYC510)</t>
         </is>
       </c>
       <c r="D1127" s="4" t="inlineStr">
         <is>
-          <t>INTER. SHAFT BEARING</t>
+          <t>DRILLING MACHINE- BAND GEAR BOX</t>
         </is>
       </c>
       <c r="E1127" s="4" t="inlineStr">
         <is>
-          <t>ATLANTA MARINE D 3005</t>
+          <t>CERAN XM 220</t>
         </is>
       </c>
       <c r="F1127" s="5" t="inlineStr">
@@ -42164,27 +42160,27 @@
     <row r="1128">
       <c r="A1128" s="2" t="inlineStr">
         <is>
-          <t>GREASE PUMP FOR RUDDER CARRIER</t>
+          <t>WORKSHOP MACHINERY</t>
         </is>
       </c>
       <c r="B1128" s="2" t="inlineStr">
         <is>
-          <t>3K INDUSTRY</t>
+          <t>TMS SOLUTION</t>
         </is>
       </c>
       <c r="C1128" s="2" t="inlineStr">
         <is>
-          <t>MSK-602-T5M / OK 92DH</t>
+          <t>LATHE (TYC510)</t>
         </is>
       </c>
       <c r="D1128" s="2" t="inlineStr">
         <is>
-          <t>MOTOR DRIVEN GREASE PUMP &amp; MANUAL FILLING PUMP</t>
+          <t>DRILLING MACHINE- SPINDLE</t>
         </is>
       </c>
       <c r="E1128" s="2" t="inlineStr">
         <is>
-          <t>BIOMULTIS EP0</t>
+          <t>VISGA 32</t>
         </is>
       </c>
       <c r="F1128" s="3" t="inlineStr">
@@ -42201,27 +42197,27 @@
     <row r="1129">
       <c r="A1129" s="4" t="inlineStr">
         <is>
-          <t>AIR CONDITIONING PLANT</t>
+          <t>WORKSHOP MACHINERY</t>
         </is>
       </c>
       <c r="B1129" s="4" t="inlineStr">
         <is>
-          <t>HI AIR KOREA</t>
+          <t>TMS SOLUTION</t>
         </is>
       </c>
       <c r="C1129" s="4" t="inlineStr">
         <is>
-          <t>OSK7451/CRKT501917</t>
+          <t>LATHE (TYC510)</t>
         </is>
       </c>
       <c r="D1129" s="4" t="inlineStr">
         <is>
-          <t>OIL SEPARATOR</t>
+          <t>DRILLING MACHINE- HEAD GEAR</t>
         </is>
       </c>
       <c r="E1129" s="4" t="inlineStr">
         <is>
-          <t>CPI SOLEST 170</t>
+          <t>VISGA 32</t>
         </is>
       </c>
       <c r="F1129" s="5" t="inlineStr">
@@ -42238,27 +42234,27 @@
     <row r="1130">
       <c r="A1130" s="2" t="inlineStr">
         <is>
-          <t>PROVISION REFRIGERATING PLANT</t>
+          <t>WORKSHOP MACHINERY</t>
         </is>
       </c>
       <c r="B1130" s="2" t="inlineStr">
         <is>
-          <t>HI AIR KOREA</t>
+          <t>TMS SOLUTION</t>
         </is>
       </c>
       <c r="C1130" s="2" t="inlineStr">
         <is>
-          <t>2N.2./CRKT221016</t>
+          <t>LATHE (TYC510)</t>
         </is>
       </c>
       <c r="D1130" s="2" t="inlineStr">
         <is>
-          <t>COMPRESSOR CRANKCASE</t>
+          <t>DRILLING MACHINE- COLUMN GEAR</t>
         </is>
       </c>
       <c r="E1130" s="2" t="inlineStr">
         <is>
-          <t>CPI SOLEST 68</t>
+          <t>CERAN XM 220</t>
         </is>
       </c>
       <c r="F1130" s="3" t="inlineStr">
@@ -42275,27 +42271,27 @@
     <row r="1131">
       <c r="A1131" s="4" t="inlineStr">
         <is>
-          <t>EM'CY GEN. ENGINE</t>
+          <t>WORKSHOP MACHINERY</t>
         </is>
       </c>
       <c r="B1131" s="4" t="inlineStr">
         <is>
-          <t>GPC-HD HYUNDAI INFRACORE</t>
+          <t>TMS SOLUTION</t>
         </is>
       </c>
       <c r="C1131" s="4" t="inlineStr">
         <is>
-          <t>4AD126TIS</t>
+          <t>LATHE (TYC510)</t>
         </is>
       </c>
       <c r="D1131" s="4" t="inlineStr">
         <is>
-          <t>MAIN LO SYSTEM</t>
+          <t>LATHE- HEAD STOCK</t>
         </is>
       </c>
       <c r="E1131" s="4" t="inlineStr">
         <is>
-          <t>DISOLA W 15W40</t>
+          <t>VISGA 32</t>
         </is>
       </c>
       <c r="F1131" s="5" t="inlineStr">
@@ -42312,22 +42308,22 @@
     <row r="1132">
       <c r="A1132" s="2" t="inlineStr">
         <is>
-          <t>EM'CY GEN. ENGINE</t>
+          <t>WORKSHOP MACHINERY</t>
         </is>
       </c>
       <c r="B1132" s="2" t="inlineStr">
         <is>
-          <t>GPC-HD HYUNDAI INFRACORE</t>
+          <t>TMS SOLUTION</t>
         </is>
       </c>
       <c r="C1132" s="2" t="inlineStr">
         <is>
-          <t>4AD126TIS</t>
+          <t>LATHE (TYC510)</t>
         </is>
       </c>
       <c r="D1132" s="2" t="inlineStr">
         <is>
-          <t>HYDRO STARTING UNIT</t>
+          <t>LATHE- FEED BOX</t>
         </is>
       </c>
       <c r="E1132" s="2" t="inlineStr">
@@ -42349,27 +42345,27 @@
     <row r="1133">
       <c r="A1133" s="4" t="inlineStr">
         <is>
-          <t>MAIN GENERATOR</t>
+          <t>WORKSHOP MACHINERY</t>
         </is>
       </c>
       <c r="B1133" s="4" t="inlineStr">
         <is>
-          <t>HDHE</t>
+          <t>TMS SOLUTION</t>
         </is>
       </c>
       <c r="C1133" s="4" t="inlineStr">
         <is>
-          <t>HFC7 716-08P</t>
+          <t>LATHE (TYC510)</t>
         </is>
       </c>
       <c r="D1133" s="4" t="inlineStr">
         <is>
-          <t>SLEEVE BEARING</t>
+          <t>LATHE- APRON</t>
         </is>
       </c>
       <c r="E1133" s="4" t="inlineStr">
         <is>
-          <t>VISGA 68</t>
+          <t>VISGA 32</t>
         </is>
       </c>
       <c r="F1133" s="5" t="inlineStr">
@@ -42386,27 +42382,27 @@
     <row r="1134">
       <c r="A1134" s="2" t="inlineStr">
         <is>
-          <t>MAIN ENGINE</t>
+          <t>WORKSHOP MACHINERY</t>
         </is>
       </c>
       <c r="B1134" s="2" t="inlineStr">
         <is>
-          <t>HYUNDAI-WINGD</t>
+          <t>TMS SOLUTION</t>
         </is>
       </c>
       <c r="C1134" s="2" t="inlineStr">
         <is>
-          <t>5X72DF-2.2</t>
+          <t>LATHE (TYC510)</t>
         </is>
       </c>
       <c r="D1134" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM</t>
+          <t>LATHE- OIL POINTER</t>
         </is>
       </c>
       <c r="E1134" s="2" t="inlineStr">
         <is>
-          <t>ATLANTA MARINE D 3005 A1</t>
+          <t>VISGA 32</t>
         </is>
       </c>
       <c r="F1134" s="3" t="inlineStr">
@@ -42416,34 +42412,34 @@
       </c>
       <c r="G1134" s="2" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
     <row r="1135">
       <c r="A1135" s="4" t="inlineStr">
         <is>
-          <t>MAIN ENGINE</t>
+          <t>WORKSHOP MACHINERY</t>
         </is>
       </c>
       <c r="B1135" s="4" t="inlineStr">
         <is>
-          <t>HYUNDAI-WINGD</t>
+          <t>TMS SOLUTION</t>
         </is>
       </c>
       <c r="C1135" s="4" t="inlineStr">
         <is>
-          <t>5X72DF-2.2</t>
+          <t>LATHE (TYC510)</t>
         </is>
       </c>
       <c r="D1135" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER OIL</t>
+          <t>LATHE- CHANGE GEAR</t>
         </is>
       </c>
       <c r="E1135" s="4" t="inlineStr">
         <is>
-          <t>TALUSIA HD 40</t>
+          <t>VISGA 32</t>
         </is>
       </c>
       <c r="F1135" s="5" t="inlineStr">
@@ -42453,34 +42449,34 @@
       </c>
       <c r="G1135" s="4" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
     <row r="1136">
       <c r="A1136" s="2" t="inlineStr">
         <is>
-          <t>MAIN ENGINE</t>
+          <t>WORKSHOP MACHINERY</t>
         </is>
       </c>
       <c r="B1136" s="2" t="inlineStr">
         <is>
-          <t>HYUNDAI-WINGD</t>
+          <t>TMS SOLUTION</t>
         </is>
       </c>
       <c r="C1136" s="2" t="inlineStr">
         <is>
-          <t>5X72DF-2.2</t>
+          <t>LATHE (TYC510)</t>
         </is>
       </c>
       <c r="D1136" s="2" t="inlineStr">
         <is>
-          <t>ENCLOSED GEAR</t>
+          <t>LATHE- ACTION BAR</t>
         </is>
       </c>
       <c r="E1136" s="2" t="inlineStr">
         <is>
-          <t>EPONA Z 220</t>
+          <t>VISGA 32</t>
         </is>
       </c>
       <c r="F1136" s="3" t="inlineStr">
@@ -42490,34 +42486,34 @@
       </c>
       <c r="G1136" s="2" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
     <row r="1137">
       <c r="A1137" s="4" t="inlineStr">
         <is>
-          <t>MAIN ENGINE</t>
+          <t>WORKSHOP MACHINERY</t>
         </is>
       </c>
       <c r="B1137" s="4" t="inlineStr">
         <is>
-          <t>HYUNDAI-WINGD</t>
+          <t>TMS SOLUTION</t>
         </is>
       </c>
       <c r="C1137" s="4" t="inlineStr">
         <is>
-          <t>5X72DF-2.2</t>
+          <t>LATHE (TYC510)</t>
         </is>
       </c>
       <c r="D1137" s="4" t="inlineStr">
         <is>
-          <t>TURNING GEAR GREASE</t>
+          <t>LATHE- TAILSTOCK</t>
         </is>
       </c>
       <c r="E1137" s="4" t="inlineStr">
         <is>
-          <t>CERAN XM 220</t>
+          <t>VISGA 32</t>
         </is>
       </c>
       <c r="F1137" s="5" t="inlineStr">
@@ -42527,34 +42523,34 @@
       </c>
       <c r="G1137" s="4" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
     <row r="1138">
       <c r="A1138" s="2" t="inlineStr">
         <is>
-          <t>MAIN ENGINE</t>
+          <t>WORKSHOP MACHINERY</t>
         </is>
       </c>
       <c r="B1138" s="2" t="inlineStr">
         <is>
-          <t>HYUNDAI-WINGD</t>
+          <t>TMS SOLUTION</t>
         </is>
       </c>
       <c r="C1138" s="2" t="inlineStr">
         <is>
-          <t>5X72DF-2.2</t>
+          <t>LATHE (TYC510)</t>
         </is>
       </c>
       <c r="D1138" s="2" t="inlineStr">
         <is>
-          <t>AUX. BLOWER MOTOR BEARING</t>
+          <t>LATHE- CARRIAGE</t>
         </is>
       </c>
       <c r="E1138" s="2" t="inlineStr">
         <is>
-          <t>MULTIS EP 2</t>
+          <t>VISGA 32</t>
         </is>
       </c>
       <c r="F1138" s="3" t="inlineStr">
@@ -42564,34 +42560,34 @@
       </c>
       <c r="G1138" s="2" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
     <row r="1139">
       <c r="A1139" s="4" t="inlineStr">
         <is>
-          <t>MAIN ENGINE</t>
+          <t>ENGINE ROOM PUMP</t>
         </is>
       </c>
       <c r="B1139" s="4" t="inlineStr">
         <is>
-          <t>HYUNDAI-WINGD</t>
+          <t>IMO</t>
         </is>
       </c>
       <c r="C1139" s="4" t="inlineStr">
         <is>
-          <t>5X72DF-2.2</t>
+          <t>IINO KAI</t>
         </is>
       </c>
       <c r="D1139" s="4" t="inlineStr">
         <is>
-          <t>FUEL VALVE TEST DEVICE</t>
+          <t>M.G.O. TRANSFER PUMP</t>
         </is>
       </c>
       <c r="E1139" s="4" t="inlineStr">
         <is>
-          <t>SHELL CALIBRATION FLUID S.9365</t>
+          <t>MULTIS EP 3</t>
         </is>
       </c>
       <c r="F1139" s="5" t="inlineStr">
@@ -42601,34 +42597,34 @@
       </c>
       <c r="G1139" s="4" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
     <row r="1140">
       <c r="A1140" s="2" t="inlineStr">
         <is>
-          <t>MAIN ENGINE</t>
+          <t>ENGINE ROOM PUMP</t>
         </is>
       </c>
       <c r="B1140" s="2" t="inlineStr">
         <is>
-          <t>HYUNDAI-WINGD</t>
+          <t>IMO</t>
         </is>
       </c>
       <c r="C1140" s="2" t="inlineStr">
         <is>
-          <t>5X72DF-2.2</t>
+          <t>IINO KAI</t>
         </is>
       </c>
       <c r="D1140" s="2" t="inlineStr">
         <is>
-          <t>AIR DRIVEN HIGH PRESS. PUMP</t>
+          <t>L.F.O. TRANSFER PUMP</t>
         </is>
       </c>
       <c r="E1140" s="2" t="inlineStr">
         <is>
-          <t>VISGA 32</t>
+          <t>MULTIS EP 3</t>
         </is>
       </c>
       <c r="F1140" s="3" t="inlineStr">
@@ -42638,34 +42634,34 @@
       </c>
       <c r="G1140" s="2" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
     <row r="1141">
       <c r="A1141" s="4" t="inlineStr">
         <is>
-          <t>MAIN ENGINE</t>
+          <t>ENGINE ROOM PUMP</t>
         </is>
       </c>
       <c r="B1141" s="4" t="inlineStr">
         <is>
-          <t>HYUNDAI-WINGD</t>
+          <t>IMO</t>
         </is>
       </c>
       <c r="C1141" s="4" t="inlineStr">
         <is>
-          <t>5X72DF-2.2</t>
+          <t>IINO KAI</t>
         </is>
       </c>
       <c r="D1141" s="4" t="inlineStr">
         <is>
-          <t>WTS SEPARATOR</t>
+          <t>FWD L.F.O. TRANSFER PUMP</t>
         </is>
       </c>
       <c r="E1141" s="4" t="inlineStr">
         <is>
-          <t>EPONA Z 150</t>
+          <t>MULTIS EP 3</t>
         </is>
       </c>
       <c r="F1141" s="5" t="inlineStr">
@@ -42675,34 +42671,34 @@
       </c>
       <c r="G1141" s="4" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
     <row r="1142">
       <c r="A1142" s="2" t="inlineStr">
         <is>
-          <t>MAIN ENGINE</t>
+          <t>ENGINE ROOM PUMP</t>
         </is>
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>HYUNDAI-WINGD</t>
+          <t>IMO</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
         <is>
-          <t>5X72DF-2.2</t>
+          <t>IINO KAI</t>
         </is>
       </c>
       <c r="D1142" s="2" t="inlineStr">
         <is>
-          <t>EGC BUTTERFLY VALVE</t>
+          <t>OILY BILGE PUMP</t>
         </is>
       </c>
       <c r="E1142" s="2" t="inlineStr">
         <is>
-          <t>MULTIS EP 2</t>
+          <t>EPONA Z 460</t>
         </is>
       </c>
       <c r="F1142" s="3" t="inlineStr">
@@ -42712,34 +42708,34 @@
       </c>
       <c r="G1142" s="2" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
     <row r="1143">
       <c r="A1143" s="4" t="inlineStr">
         <is>
-          <t>MAIN ENGINE</t>
+          <t>ENGINE ROOM PUMP</t>
         </is>
       </c>
       <c r="B1143" s="4" t="inlineStr">
         <is>
-          <t>HYUNDAI-WINGD</t>
+          <t>IMO</t>
         </is>
       </c>
       <c r="C1143" s="4" t="inlineStr">
         <is>
-          <t>5X72DF-2.2</t>
+          <t>IINO KAI</t>
         </is>
       </c>
       <c r="D1143" s="4" t="inlineStr">
         <is>
-          <t>H-MOMENT COMPENSATOR</t>
+          <t>BILGE CIRC. PUMP</t>
         </is>
       </c>
       <c r="E1143" s="4" t="inlineStr">
         <is>
-          <t>EPONA Z 150</t>
+          <t>EPONA Z 460</t>
         </is>
       </c>
       <c r="F1143" s="5" t="inlineStr">
@@ -42749,34 +42745,34 @@
       </c>
       <c r="G1143" s="4" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
     <row r="1144">
       <c r="A1144" s="2" t="inlineStr">
         <is>
-          <t>INCINERATOR</t>
+          <t>ENGINE ROOM PUMP</t>
         </is>
       </c>
       <c r="B1144" s="2" t="inlineStr">
         <is>
-          <t>HMMCO</t>
+          <t>IMO</t>
         </is>
       </c>
       <c r="C1144" s="2" t="inlineStr">
         <is>
-          <t>MAXI T150SL WS</t>
+          <t>IINO KAI</t>
         </is>
       </c>
       <c r="D1144" s="2" t="inlineStr">
         <is>
-          <t>GEAR BOX FOR W.O.DOSING PUMP</t>
+          <t>SLUDGE PUMP</t>
         </is>
       </c>
       <c r="E1144" s="2" t="inlineStr">
         <is>
-          <t>EPONA Z 220</t>
+          <t>EPONA Z 460</t>
         </is>
       </c>
       <c r="F1144" s="3" t="inlineStr">
@@ -42786,34 +42782,34 @@
       </c>
       <c r="G1144" s="2" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
     <row r="1145">
       <c r="A1145" s="4" t="inlineStr">
         <is>
-          <t>INCINERATOR</t>
+          <t>STEERING GEAR</t>
         </is>
       </c>
       <c r="B1145" s="4" t="inlineStr">
         <is>
-          <t>HMMCO</t>
+          <t>YOOWON-MITSUBISHI</t>
         </is>
       </c>
       <c r="C1145" s="4" t="inlineStr">
         <is>
-          <t>MAXI T150SL WS</t>
+          <t>YDFT-200-2</t>
         </is>
       </c>
       <c r="D1145" s="4" t="inlineStr">
         <is>
-          <t>MILL PUMP SEAL BOX</t>
+          <t>HYD. OIL STOR. TK</t>
         </is>
       </c>
       <c r="E1145" s="4" t="inlineStr">
         <is>
-          <t>VISGA 46</t>
+          <t>PRESLIA 68</t>
         </is>
       </c>
       <c r="F1145" s="5" t="inlineStr">
@@ -42823,34 +42819,34 @@
       </c>
       <c r="G1145" s="4" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
     <row r="1146">
       <c r="A1146" s="2" t="inlineStr">
         <is>
-          <t>ELECTRIC BALANCER</t>
+          <t>STEERING GEAR</t>
         </is>
       </c>
       <c r="B1146" s="2" t="inlineStr">
         <is>
-          <t>COMPENSATOR</t>
+          <t>YOOWON-MITSUBISHI</t>
         </is>
       </c>
       <c r="C1146" s="2" t="inlineStr">
         <is>
-          <t>(EMC-400VD 2SETS)</t>
+          <t>YDFT-200-2</t>
         </is>
       </c>
       <c r="D1146" s="2" t="inlineStr">
         <is>
-          <t>BEARING, GEAR</t>
+          <t>PUMP, CYLINDER, PIPE</t>
         </is>
       </c>
       <c r="E1146" s="2" t="inlineStr">
         <is>
-          <t>EPONA Z 100</t>
+          <t>PRESLIA 68</t>
         </is>
       </c>
       <c r="F1146" s="3" t="inlineStr">
@@ -42860,7 +42856,7 @@
       </c>
       <c r="G1146" s="2" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
@@ -42877,12 +42873,12 @@
       </c>
       <c r="C1147" s="4" t="inlineStr">
         <is>
-          <t>AFT(AX-670), FWD(AX-670)</t>
+          <t>AFT/FWD : AX-630</t>
         </is>
       </c>
       <c r="D1147" s="4" t="inlineStr">
         <is>
-          <t>FWD/AFT SEAL CHAMBER</t>
+          <t>S/T L.O. TANK</t>
         </is>
       </c>
       <c r="E1147" s="4" t="inlineStr">
@@ -42897,7 +42893,7 @@
       </c>
       <c r="G1147" s="4" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
@@ -42914,12 +42910,12 @@
       </c>
       <c r="C1148" s="2" t="inlineStr">
         <is>
-          <t>AFT(AX-670), FWD(AX-670)</t>
+          <t>AFT/FWD : AX-630</t>
         </is>
       </c>
       <c r="D1148" s="2" t="inlineStr">
         <is>
-          <t>S/T INSIDE</t>
+          <t>FWD SEAL TANK</t>
         </is>
       </c>
       <c r="E1148" s="2" t="inlineStr">
@@ -42934,7 +42930,7 @@
       </c>
       <c r="G1148" s="2" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
@@ -42951,12 +42947,12 @@
       </c>
       <c r="C1149" s="4" t="inlineStr">
         <is>
-          <t>AFT(AX-670), FWD(AX-670)</t>
+          <t>AFT/FWD : AX-630</t>
         </is>
       </c>
       <c r="D1149" s="4" t="inlineStr">
         <is>
-          <t>FWD SEAL TANK</t>
+          <t>S/T LO SUMP TANK</t>
         </is>
       </c>
       <c r="E1149" s="4" t="inlineStr">
@@ -42971,7 +42967,7 @@
       </c>
       <c r="G1149" s="4" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
@@ -42988,12 +42984,12 @@
       </c>
       <c r="C1150" s="2" t="inlineStr">
         <is>
-          <t>AFT(AX-670), FWD(AX-670)</t>
+          <t>AFT/FWD : AX-630</t>
         </is>
       </c>
       <c r="D1150" s="2" t="inlineStr">
         <is>
-          <t>S/T L.O. TANK</t>
+          <t>S/T LO PIPE LINE</t>
         </is>
       </c>
       <c r="E1150" s="2" t="inlineStr">
@@ -43008,7 +43004,7 @@
       </c>
       <c r="G1150" s="2" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
@@ -43025,12 +43021,12 @@
       </c>
       <c r="C1151" s="4" t="inlineStr">
         <is>
-          <t>AFT(AX-670), FWD(AX-670)</t>
+          <t>AFT/FWD : AX-630</t>
         </is>
       </c>
       <c r="D1151" s="4" t="inlineStr">
         <is>
-          <t>S/T L.O. SUMP. TK</t>
+          <t>AFT &amp; FWD SEAL CHAMBER</t>
         </is>
       </c>
       <c r="E1151" s="4" t="inlineStr">
@@ -43045,7 +43041,7 @@
       </c>
       <c r="G1151" s="4" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
@@ -43062,12 +43058,12 @@
       </c>
       <c r="C1152" s="2" t="inlineStr">
         <is>
-          <t>AFT(AX-670), FWD(AX-670)</t>
+          <t>AFT/FWD : AX-630</t>
         </is>
       </c>
       <c r="D1152" s="2" t="inlineStr">
         <is>
-          <t>PIPE LINE</t>
+          <t>S/T INSIDE</t>
         </is>
       </c>
       <c r="E1152" s="2" t="inlineStr">
@@ -43082,34 +43078,34 @@
       </c>
       <c r="G1152" s="2" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
     <row r="1153">
       <c r="A1153" s="4" t="inlineStr">
         <is>
-          <t>GREASE PUMP FOR RUDDER CARRIER</t>
+          <t>INTER. SHAFT BEARING</t>
         </is>
       </c>
       <c r="B1153" s="4" t="inlineStr">
         <is>
-          <t>3K</t>
+          <t>KEMEL</t>
         </is>
       </c>
       <c r="C1153" s="4" t="inlineStr">
         <is>
-          <t>INDUSTRY</t>
+          <t>KMS-620</t>
         </is>
       </c>
       <c r="D1153" s="4" t="inlineStr">
         <is>
-          <t>GREASE PUMP &amp; MANUAL FILLING PUMP</t>
+          <t>INTER. SHAFT BEARING</t>
         </is>
       </c>
       <c r="E1153" s="4" t="inlineStr">
         <is>
-          <t>BIOMULTIS EP0</t>
+          <t>ATLANTA MARINE D 3005</t>
         </is>
       </c>
       <c r="F1153" s="5" t="inlineStr">
@@ -43119,34 +43115,34 @@
       </c>
       <c r="G1153" s="4" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
     <row r="1154">
       <c r="A1154" s="2" t="inlineStr">
         <is>
-          <t>AIR COND. PLANT</t>
+          <t>GREASE PUMP FOR RUDDER CARRIER</t>
         </is>
       </c>
       <c r="B1154" s="2" t="inlineStr">
         <is>
-          <t>R-407C CONDENSING UNIT</t>
+          <t>3K INDUSTRY</t>
         </is>
       </c>
       <c r="C1154" s="2" t="inlineStr">
         <is>
-          <t>(OSK8551/502320</t>
+          <t>MSK-602-T5M / OK 92DH</t>
         </is>
       </c>
       <c r="D1154" s="2" t="inlineStr">
         <is>
-          <t>OIL SEPARATOR</t>
+          <t>MOTOR DRIVEN GREASE PUMP &amp; MANUAL FILLING PUMP</t>
         </is>
       </c>
       <c r="E1154" s="2" t="inlineStr">
         <is>
-          <t>BITZER BSE 170</t>
+          <t>BIOMULTIS EP0</t>
         </is>
       </c>
       <c r="F1154" s="3" t="inlineStr">
@@ -43156,34 +43152,34 @@
       </c>
       <c r="G1154" s="2" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
     <row r="1155">
       <c r="A1155" s="4" t="inlineStr">
         <is>
-          <t>AIR COND. PLANT</t>
+          <t>AIR CONDITIONING PLANT</t>
         </is>
       </c>
       <c r="B1155" s="4" t="inlineStr">
         <is>
-          <t>R-407C CONDENSING UNIT</t>
+          <t>HI AIR KOREA</t>
         </is>
       </c>
       <c r="C1155" s="4" t="inlineStr">
         <is>
-          <t>(OSK8551/502320</t>
+          <t>OSK7451/CRKT501917</t>
         </is>
       </c>
       <c r="D1155" s="4" t="inlineStr">
         <is>
-          <t>REPLACEMENT OIL</t>
+          <t>OIL SEPARATOR</t>
         </is>
       </c>
       <c r="E1155" s="4" t="inlineStr">
         <is>
-          <t>BITZER BSE 170</t>
+          <t>CPI SOLEST 170</t>
         </is>
       </c>
       <c r="F1155" s="5" t="inlineStr">
@@ -43193,24 +43189,24 @@
       </c>
       <c r="G1155" s="4" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
     <row r="1156">
       <c r="A1156" s="2" t="inlineStr">
         <is>
-          <t>PROV. REF. PLANT</t>
+          <t>PROVISION REFRIGERATING PLANT</t>
         </is>
       </c>
       <c r="B1156" s="2" t="inlineStr">
         <is>
-          <t>R-407C CONDENSING UNIT</t>
+          <t>HI AIR KOREA</t>
         </is>
       </c>
       <c r="C1156" s="2" t="inlineStr">
         <is>
-          <t>(4T.2/221014)</t>
+          <t>2N.2./CRKT221016</t>
         </is>
       </c>
       <c r="D1156" s="2" t="inlineStr">
@@ -43220,7 +43216,7 @@
       </c>
       <c r="E1156" s="2" t="inlineStr">
         <is>
-          <t>BITZER BSE 55</t>
+          <t>CPI SOLEST 68</t>
         </is>
       </c>
       <c r="F1156" s="3" t="inlineStr">
@@ -43230,34 +43226,34 @@
       </c>
       <c r="G1156" s="2" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
     <row r="1157">
       <c r="A1157" s="4" t="inlineStr">
         <is>
-          <t>PROV. REF. PLANT</t>
+          <t>EM'CY GEN. ENGINE</t>
         </is>
       </c>
       <c r="B1157" s="4" t="inlineStr">
         <is>
-          <t>R-407C CONDENSING UNIT</t>
+          <t>GPC-HD HYUNDAI INFRACORE</t>
         </is>
       </c>
       <c r="C1157" s="4" t="inlineStr">
         <is>
-          <t>(4T.2/221014)</t>
+          <t>4AD126TIS</t>
         </is>
       </c>
       <c r="D1157" s="4" t="inlineStr">
         <is>
-          <t>REPLACEMENT OIL</t>
+          <t>MAIN LO SYSTEM</t>
         </is>
       </c>
       <c r="E1157" s="4" t="inlineStr">
         <is>
-          <t>BITZER BSE 55</t>
+          <t>DISOLA W 15W40</t>
         </is>
       </c>
       <c r="F1157" s="5" t="inlineStr">
@@ -43267,7 +43263,7 @@
       </c>
       <c r="G1157" s="4" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
@@ -43279,22 +43275,22 @@
       </c>
       <c r="B1158" s="2" t="inlineStr">
         <is>
-          <t>GPC - BAUDOUIN</t>
+          <t>GPC-HD HYUNDAI INFRACORE</t>
         </is>
       </c>
       <c r="C1158" s="2" t="inlineStr">
         <is>
-          <t>(12M33)</t>
+          <t>4AD126TIS</t>
         </is>
       </c>
       <c r="D1158" s="2" t="inlineStr">
         <is>
-          <t>MAIN LO SYSTEM</t>
+          <t>HYDRO STARTING UNIT</t>
         </is>
       </c>
       <c r="E1158" s="2" t="inlineStr">
         <is>
-          <t>DISOLA W 15W-40</t>
+          <t>VISGA 32</t>
         </is>
       </c>
       <c r="F1158" s="3" t="inlineStr">
@@ -43304,34 +43300,34 @@
       </c>
       <c r="G1158" s="2" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>
     <row r="1159">
       <c r="A1159" s="4" t="inlineStr">
         <is>
-          <t>EM'CY GEN. ENGINE</t>
+          <t>MAIN GENERATOR</t>
         </is>
       </c>
       <c r="B1159" s="4" t="inlineStr">
         <is>
-          <t>GPC - BAUDOUIN</t>
+          <t>HDHE</t>
         </is>
       </c>
       <c r="C1159" s="4" t="inlineStr">
         <is>
-          <t>(12M33)</t>
+          <t>HFC7 716-08P</t>
         </is>
       </c>
       <c r="D1159" s="4" t="inlineStr">
         <is>
-          <t>HYDRO STARTING UNIT</t>
+          <t>SLEEVE BEARING</t>
         </is>
       </c>
       <c r="E1159" s="4" t="inlineStr">
         <is>
-          <t>VISGA 32</t>
+          <t>VISGA 68</t>
         </is>
       </c>
       <c r="F1159" s="5" t="inlineStr">
@@ -43341,7 +43337,7 @@
       </c>
       <c r="G1159" s="4" t="inlineStr">
         <is>
-          <t>3441's 7U-2000-501 LO Chart (TOTAL)_R101.pdf</t>
+          <t>3414_7U-2000-501_Lub Oil Chart(TOTAL)_R100_0001.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>